<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 6, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1316,8 +1316,664 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1168692108</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>【正規品】松の木 鎮静 シカ クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168692108</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1164469069</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>【正規品】グリーンシカ コラーゲン クリアフォーム 2.0 300ml</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164469069</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1163729695</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>【正規品】ディープポア クレンジング ソーダフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163729695</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1205554253</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>【正規品】トラネキサム酸スキンブースタークリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>メディテラピー</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205554253</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1193459511</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>【正規品】レチノコラーゲン低分子300ネックカッサクリーム 50ml (2個)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CKD_GUARANTEED</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>6490</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193459511</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1210771223</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PLUS82</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>マデカクリーム イン バブルセラム 100ml+100ml（+マデカパウダー ビタグルシ 6g）</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>6273</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210771223</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1206008325</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ペプチドショット2X 弾力アンプル 30ml（ハリ感ケア／保湿／弾力サポート美容液）</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2122</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008325</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1206008294</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ウォーターフィット リカバー BBクリーム 30ml #SPF40 PA+++ #保湿密着</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>2927</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008294</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1205912921</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>レチンアルブースターショット 30ml+30ml #レチナール2.0% #セラミド #エクトイン #カフェイン #ペプチド</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>4046</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205912921</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1205483331</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>COCOAN</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>【1+1セット】成分エディターグリーントマト NMN フォアリフティングアンプル 40ml+40ml / 毛穴のしわ 弾力 エッセンス 美容液 グリーントマト</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>グリーントマト</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205483331</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1205132300</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>COCOAN</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>[1個]ダークスポットセラム30ml (ナイアシンアミド10%, トラネキサム酸 4%)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>2350</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205132300</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1107510664</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>KSB</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>[新作]ムード レイヤー スティック クレヨン 5color 00 milky syrup 01 caramel drizzle 02 rose milk tea 03 mauve latte</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>alternative stereo</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2405</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107510664</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1154233546</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>jullyland</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ダークスポットセラム (ナイアシンアミド10%, トラネキサム酸 4%) 30ml/韓国コスメ/アンプル</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2580</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154233546</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1188839770</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>[保湿 保水 栄養 シートマスク 10枚 5種類から選択] 高保湿 まとめ買い 夜用 デイリー スキンケア</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1709</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188839770</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1197460025</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>【1+1 クリームミスト 120ml】保湿ミスト 化粧水ミスト うるおいケア 整肌ケア スプレー 韓国スキンケア デイリーケア</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197460025</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1188077394</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>[秀麗な本超保湿クリーム 50ml] 韓国漢方 高保湿 エイジングケア シワ/改/善 /弾力アップ しっとり濃密テクスチャー</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>秀麗韓</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>4427</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188077394</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J21"/>
+  <autoFilter ref="A1:J37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 9, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1972,8 +1972,623 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1147146315</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PDRN ピンク グルタチオン セラム ミスト 100ml 水分 保湿 弾力 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>2961</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147146315</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1159784308</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ビタCプラス アスコルビン酸 クリアコンプレクション フォーミングクレンザー 120ml 高濃度ビタミンC フォームクレンジング 水分 保湿 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1971</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159784308</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1198095545</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>【GIFT】洗顔/ゼロ 毛穴 ブラックヘッド ディープ クレンジングオイル 205ml/毛穴ケア/毛穴 黒ずみ/ブラックヘッド/韓国コスメ 毛穴</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="b">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198095545</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1209903581</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>【ニキビケア】1番 パントテン酸アクティブスージングクリーム 80ml/ニキビ</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209903581</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1110469138</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>【5種沢1】CICA/PDRN/毛穴/ニキビケア/保湿／トナーパット／鎮静／トナー／化粧水/毛穴ケア/ふき取り化粧水/メが割/美容液</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>2995</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110469138</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1203205247</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>vanguardvista</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>[正規品] 人気 おすすめ 韓国 クリーム Rx 30ml+7ml セット スキンケア クリーム ギフト</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ドミナス</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>5820</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203205247</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1207091863</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>リードルショット フォーメン オールインワン100 Mプラス 150ml＋30ml 企画セット メンズスキンケア 韓国コスメ 化粧水 乳液 美容液</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>3855</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091863</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1174137858</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ローズマリー &amp;amp; シーソルト &amp;amp; AHA シャンプー 500ml × 2本セット 韓国シャンプー スカルプケア 頭皮クレンジング ボリュームケア</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>オーガニスト</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174137858</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1024539184</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>[1+1]ハニーアンドマカデミア ネイチャーシャンプー 500ml+プロテイントリートメント 500mlホワイトムスクの香り</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1024539184</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1207091851</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>3番 ノーファンデ陶器肌トーンアップUVクリーム 50ml (SPF50+ PA++++) / トーンケアクリーム 保湿ベース 水分クリーム 化粧下地 ナチュラルトーンアップ</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091851</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1174312286</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>【1+1】【韓国コスメ】【正規品扱い店】[病院専用] ラポラピルナトックス 50ml - シミ改善＆肌トーンアップの機能性クリーム！</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Dermagen</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>7128</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174312286</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1146499682</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】タイムエナジーリセッティングエマルジョン 120ml - 時間を超える美肌の秘訣！</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>4781</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="b">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499682</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1146499598</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】[5番企画セット] 白玉リンガーグルタチオンCトナー200ML ＋ 白玉グルタチオンC美容液30ML - 輝く美肌へ導く！</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>7013</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="b">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499598</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1145594895</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>【正規品扱い店】【1+1】【本品+レフィル】ダイブイン低分子ヒアルロン酸セラム, 50mL*2</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>4879</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="b">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594895</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1145594718</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】シルクペプチドインテンシブリフティングアンプル35ML</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>2407</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="b">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594718</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J37"/>
+  <autoFilter ref="A1:J52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 12, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2587,8 +2587,705 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1165444330</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>アヌカチン シャンプー 525ml</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>moev</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>5150</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="b">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165444330</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1179699936</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>[輪郭アンプル] コアタイムアンプル 15ml (+7ml)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>NEURADERM</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>4340</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179699936</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1165596313</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>[1+1] 黒雲 毛根強化アンドボリュームケアシャンプー 500ml</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>呂</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>3470</v>
+      </c>
+      <c r="G55" t="n">
+        <v>3</v>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165596313</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1165513951</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラ クイック カーミングパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165513951</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1165361801</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>saleb</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>[1+1] コルツフート アンチダンドラフ シャンプー 200ml</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ラウシュ</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>6570</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165361801</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1207091316</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>レチノールスーパーバウンスセラム 20ml＋15ml 企画セット 初めてのレチノールケア 昼夜使いやすい 美容液 メイク前 なめらか肌印象 韓国コスメ スポイトタイプ 水分感 クリーム前 スキンケア</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>5324</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091316</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1210932470</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ブルー EGF カーミングミスト 100ml 韓国フェイスミスト 化粧水ミスト うるおいケア 肌コンディションケア</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>3599</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210932470</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1198423707</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ポリジェン シークニング スカルプ コンディショニングマスク 200ml / 頭皮ケア ボリュームアップケア ハリコシ ダメージケア 保湿 しっとり サロンケア ヘアパック スカルプパック</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>3296</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198423707</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1211212429</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>セルアップ マイクロ フォームクレンザー 120ml 2個＋クレンジングミルク20ml 韓国洗顔フォーム 洗顔料 毛穴汚れケア うるおい洗顔</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ラゴム</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211212429</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1196826611</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml / 保湿乳液 敏感肌対応 うるおいケア スキンケアローション 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G62" t="n">
+        <v>3</v>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196826611</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1164705875</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ウォータープルーフプロ日焼け止め 50g+サンスティック 20g / アウトドア スポーツ対応UVクリーム 汗・水に強いスティックタイプ 手を汚さない</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>5499</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164705875</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1187759601</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>joungho</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>【韓国旅行の定番】垢すり石鹸＆グローブ6個セットまるで韓国エステ！自宅で叶う極上のツルツル美肌体験</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ダイソー</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G64" t="n">
+        <v>2</v>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187759601</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1194068552</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>joungho</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>韓国国民アイテム キュアアルファカーミングアロエクリーム 50g 2個</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>CURE</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194068552</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1183178551</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Starlit</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>TN トラネキサミン5%＋ナイアシンアミド5% ブライトニング セラム60ml</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>コスデバハ</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>3880</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="b">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183178551</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1188405527</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Starlit</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ゆずグレープフルーツ ビーガン パッククレンザー 80g+毛穴ブラシ [毛穴ケア+洗顔+すっきり]</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ホイップド</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188405527</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1080770379</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>NARShA</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ライトオンインシャワーボディトーンアップボディローション ベビーパウダーの香り290ml</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>4720</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080770379</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1206876054</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>NARShA</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>[ブラシ元祖] グロウターンエクソソームブラシアンプル130ml企画(+30ml)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206876054</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J52"/>
+  <autoFilter ref="A1:J69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 15, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3284,8 +3284,664 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1206207561</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>[1+1] トーンアップ パールクリーム 本体30g+30g スキンケア / 保湿 / ベースメイク韓国コスメ 並行輸入</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>MAY ISLAND</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206207561</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1205776987</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>AGE-R グルタチオン グロウ カプセル クリーム 50ml 保湿 スキンケア 並行輸入</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205776987</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1199084782</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ヴィーガンコンブチャ ティー エッセンス 150ml 保湿 しっとり エッセンス 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Dr.Ceuracle</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>3380</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199084782</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1198940759</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Relief Sun Aqua-Fresh : Rice + B5 アクアフレッシュ UVクリーム 50ml 米 うるおい 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>2240</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198940759</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1195384789</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>durudurupanda</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>24K ゴールド トナー 保湿 化粧水 120ml 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>アンジョ</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1570</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195384789</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1172312020</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>hokkorikorea</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>【SALE】【毛穴ケア】PDRN毛穴弾力パッド 100枚 ハリ感 キメ整う エイジングケア ツヤ肌 角質ケア うるおい 人気 韓国コスメ 大容量 毎日ケア 時短 敏感肌OK 透明感 キメケア 保湿</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>3006</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172312020</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1193625970</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>glowbox</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>【公式】 グロウオイルミスト 50ml うるおい×ツヤ肌キープ</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193625970</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1206859281</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ポアブライトニングシミケアクリームマスク, 4枚 /ブライトニング/韓国マスクパック/ナイアシンアミド/保湿/水分/肌トーン改善/顔の頬リフ</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G77" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206859281</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1203000979</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>大豆エッセンス, 50ml</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ミクスン</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203000979</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1198208356</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>アヌカチンシャンプー, 300ml</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>moev</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1775</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198208356</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1117793591</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>OLIVIASHOP</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>【正規品/ PDRNスペシャル 3種 鎮静 セット】PDRNリジュビネイティングトナー 300ml+ビタトーニングアンプル 30ml+ジュビネイティングクリーム 70ml/鎮静/保湿/回復/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ジェナベール</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>11749</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117793591</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1138030129</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>OLIVIASHOP</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>【正規品】345リリーフクリーム, 50mlニキビ肌鎮静デイリークリーム relief cream</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G81" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138030129</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1210577063</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>wingkone</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>【正規品】【NEW】【脱色/染め】 眉毛脱色 イージーブロウトーンチェンジャー 5回分 / イージーブロウムードチェンジャー 5回分 / アイブロウ / 韓国コスメ / 眉毛</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G82" t="n">
+        <v>3</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210577063</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1202057165</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>[1+1] インフューズド コラーゲン コンセントレート フルイド 50ml 2件</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>4428</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202057165</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1202051148</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>インフュージングコラーゲンパウダー, 1.5g</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>3258</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202051148</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1202043668</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>[1+1] インフュージングコラーゲンミスト 50ml 2件</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>4473</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202043668</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J69"/>
+  <autoFilter ref="A1:J85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 18, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3940,8 +3940,664 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1206008183</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>247GOODLUCK</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ナイアシン トラネキサム酸13% セラム 30ml／トーンアップケア／肌荒れケア</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>1565</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008183</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1203846979</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>247GOODLUCK</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>PDRN エアクラウド メラケア サンスクリーン 50ml #SPF50+ PA++++ #アルブチン #トラネクサン酸 #ナイアシンアミド #エラスチン #コラーゲン</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203846979</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1157418989</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>busanjin</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ゼロ毛穴 黒ずみ マッドパック 100g #AHA+BHA+PHA</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157418989</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1205905548</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>FROM051</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>メラレイジングアンプルクリーム 56g #シミケア #ナイアシンアミド #トラネキサム酸 #8種ヒアルロン酸</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>シャルド</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>5883</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205905548</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1205520797</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ポアコントロール131 クレンジングオイル200ml／毛穴ケア／皮脂バランス</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>3153</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205520797</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1204558349</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>リポソームバブルブースター 95ml 2種（コラーゲン／キャビア PDRN）から1つ選択</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>3498</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204558349</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1208085435</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>[26SS/New]クリアライスサンスクリーン 50ml（+20ml＋チュンシキキーホルダー）</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208085435</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1208085817</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>(ポケモンエディション)体臭ソリューション デオドラント ボディウォッシュ 720ml 2種から1つ選択</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>46CM</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2889</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208085817</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1199735232</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>PDRNピンクエクソソームショット2000, 30ml</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199735232</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1191662969</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>bloomingseoul</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml(+ブルービーンクリーム7ml)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>2374</v>
+      </c>
+      <c r="G95" t="n">
+        <v>3</v>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191662969</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1209320737</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>[2PACK] クリーンイットゼロ 抹茶クレンジングバーム 100ml</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>4555</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209320737</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1201575924</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>[26SS/New]ピーチフェア ビーガン トーンアップ カプセルサンスクリーン 50ml #SPF50+ PA++++ #グルタチオン #ナイアシンアミド</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>ホイップド</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>3353</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201575924</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1201571343</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>[25SS/新作]4GF ザマ リペア ハイドロ セラム 30ml #エクソソーム #ナイアシンアミド #ペプチド #ノンコメドジェニック</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>CELORABY</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>5397</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201571343</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1190875712</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>[26SS/New]セビウム セラム 30ml（+センシビオ H2O 5ml×2）</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>6600</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190875712</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1190240492</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>アップルタチオン トニング トナー パッド 60枚 #独自特許原料アップルタチオン #リンゴエキス+アロエ+高純度グルタチオン #鎮静</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>farmic</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>5168</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190240492</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1152717704</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>[26SS/New]ボディタミン アルファ ブライトニング スポット ボディセラム 80ml #ナイアシンアミド10%</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>ビヨンド</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>2948</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152717704</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J85"/>
+  <autoFilter ref="A1:J101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 21, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4596,8 +4596,664 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1125754461</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>[1+1]レッドブレミッシュクリアスージングクリーム 50ml 2個+10ml 2個/正規品</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>3469</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125754461</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1212553298</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>【正規品+GIFT付き】リードルショット コラーゲンクリーム 50ml＋スティックパウチ 3個</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>3021</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212553298</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1212350487</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>[1+1]MEDI AHAイボ取りクリーム25ml 2個&amp;nbsp; / メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>3666</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350487</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1212350471</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>[1+1]メディオルガブライトニングクリーム30ml 2個/しみ取りクリーム お肌のトーンアップ</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>3055</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350471</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1212350473</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>MEDI AHAイボ取りクリーム25ml/ メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G106" t="n">
+        <v>1</v>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350473</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1172083985</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>KBEAT</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>【公式】ティーツリー グリーン ボディウォッシュ 500ml</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>原料工房</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>3739</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172083985</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1194074735</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>octaglobal</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸カプセル100 セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194074735</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1213314755</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>[1+1] エアリーフィットサンスティック　/　2個入り</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>3801</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213314755</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1213007507</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>エアリーフィットサンスティック</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>2077</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213007507</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1208546349</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>[1+1] ピュアクレンジングオイル 200ml　/　2個入り</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208546349</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1204555836</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>cosone</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>PDRNビタペプチド毛穴リペアセラム, 35ml</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G112" t="n">
+        <v>2</v>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204555836</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1201560856</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>[NEW] PDRN カフェイン 1000 オーバーナイト ラッピング マスク 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>P.CALM</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201560856</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1208992240</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>[NEW] マイルド ヴィーガン トーンアップ 日焼け止め 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208992240</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1191141866</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>[NEW] スーパー コラーゲン バブル セラム マスク 90g 1個</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>AROCELL</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>5550</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191141866</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1168717728</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>[新商品] キャロット カロチン モイスト エフェクター 55ml 1個</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168717728</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1146804177</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>[正品] ゼロ 毛穴 ブラックヘッド ディープ クレンジングオイル 205ml 1個</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="b">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146804177</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J101"/>
+  <autoFilter ref="A1:J117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 24, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5252,8 +5252,377 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1160418590</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>[2種セット]ブリングリーン ティーツリー シカスージングトナー 250ml + クリーム100ml</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="b">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160418590</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1152030824</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>[人気2種セット]ホワイトトリュフファーストスプレーセラム 100ml +ウォータフルトーンアップサンクリーム50ml</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>5640</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="b">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152030824</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1211694332</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>ジュリーク JURLIQUE RO バランシングミスト 100ml 化粧水 [169628]</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ジュリーク</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>4460</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="b">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211694332</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1205909859</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>【本体フィルム剥がれあり】クラランス CLARINS グランアイセラムV 15ml [448368]</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>5580</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205909859</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1191657535</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>シカケア クリア アンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191657535</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1191655869</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>[新作]オールデイ ノーセバム トーンアップ サンクッション 2種 SPF45 PA++++ lilac fog vanilla lemon</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>3982</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="b">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191655869</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>1188483946</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>キャロット カロテン デイリーマスク 30枚 #毎日使える栄養たっぷりのフェイスマスク</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>3777</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="b">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188483946</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>1203329038</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>beauty69</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>【新作】スムース＆ピュア アイス クーリング デオ スプレー 150ml 2種</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>アリウル</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>1581</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="b">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203329038</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1210434904</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>beauty69</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>[新作] NAD フリーズセル グロウブーストクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>5390</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="b">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210434904</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J117"/>
+  <autoFilter ref="A1:J126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 3, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5621,8 +5621,377 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1210877861</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>【NEW・化粧ノリUPミスト】シェイキングシナジーミスト 50ml 3種</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>2438</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="b">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210877861</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1197720706</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>【今だけ限定！企画】キャロットカロテンカーミングウォーターパッド, 60枚</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>1964</v>
+      </c>
+      <c r="G128" t="n">
+        <v>3</v>
+      </c>
+      <c r="H128" t="b">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197720706</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1142629949</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>zozoro0213</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>セラ 水分バリア 日焼け止め SPF50+ PA++++ 50ml x 2個 (鎮静/弾力/保湿/栄養供給/活力/しわ防止)</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>リアルバリア</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="b">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142629949</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1212154617</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>belif ビリーフ ザ・トゥルー クリーム モイスチャライジングバーム 50ml（保湿クリーム） (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>ビリーフ</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" t="b">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212154617</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1207926681</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>トリデン バランスフル シカ 鎮静クリーム 80ml(贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="b">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207926681</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1210186472</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>ポリジェン シックニング ボリューム強化 スカルプトニック 120ml (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>3775</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="b">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210186472</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1207682253</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>resear</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>【4種から選べる】リッサー バイオミラパッド 10枚入り (ポアピーリング / シカカーミング / ビタシャイニング / トリプルショット) 鎮静・透明感・毛穴・ハリケア 韓国スキンケア トナーパッド</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>resear</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="b">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207682253</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1209235398</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿クリーム 50ml 韓国コスメ 韓国ブランド 公式ショップ 韓国スキンケア スキンケア 化粧品 敏感肌 乾燥肌 水分ケア うるおい 韓国アンプル ギフト PDRN CICA</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>2664</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" t="b">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209235398</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1209222941</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿トナー 150ml 韓国スキンケア 韓国コスメ スキンケア PDRN CICA ヒアルロン酸 水分ケア　乾燥肌 ローション 化粧水 整肌成分 毎日のケア 弱酸性 韓国商品 高保湿</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>2472</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0</v>
+      </c>
+      <c r="H135" t="b">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209222941</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J126"/>
+  <autoFilter ref="A1:J135"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 1)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J155"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6810,8 +6810,49 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>1137329434</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>k-beauty2279</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>ダークスポットセラム, 30ml (ナイアシンアミド10%, トラネキサム酸 4%)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>4810</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="b">
+        <v>0</v>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137329434</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J155"/>
+  <autoFilter ref="A1:J156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 2)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$162</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6851,8 +6851,254 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>1204156842</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>[1+1] トン＆スポット コレクターアンプル 30ml +30ml</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Redence</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G157" t="n">
+        <v>2</v>
+      </c>
+      <c r="H157" t="b">
+        <v>0</v>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204156842</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>1186174034</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>[1+1]アルガンオイルダメージトリートメント300ml+300ml</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>エラスティン</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="b">
+        <v>0</v>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186174034</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>1156719535</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>ソウルシークレットブロッサム香水30ml</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="b">
+        <v>0</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156719535</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>1175560636</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>seoulselectstore</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>ヘアケア マルチ ペプチド セラム フォー ヘア デンシティ 60ml</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>5720</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="b">
+        <v>0</v>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175560636</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>1146350870</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>seoulselectstore</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>【NEW】 オードパルファム 08 ラブポーション 25ml</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>6580</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="b">
+        <v>0</v>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146350870</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>1185652076</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>bestkr</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>エリクシールウルティム オリジナルヘアオイル 30ml 1個 艶髪ケア うるおい 洗い流さないトリートメント サロン品質 ヘアケア デイリーケア 人気 コスパ 話題 限定 定番 口コミ多数 おすすめ</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>ケラスターゼ</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>7140</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="b">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185652076</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J156"/>
+  <autoFilter ref="A1:J162"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 3)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$168</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7097,8 +7097,254 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>1200996478</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>スリーピング コパック カミング 10枚 大容量 / ブラックヘッド 毛穴 鎮静</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>ケアプラス</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G163" t="n">
+        <v>1</v>
+      </c>
+      <c r="H163" t="b">
+        <v>0</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200996478</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>1146775594</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>【計100枚】緑豆 弱酸性 クレンジングティッシュ 20枚 x 5個</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>3330</v>
+      </c>
+      <c r="G164" t="n">
+        <v>3</v>
+      </c>
+      <c r="H164" t="b">
+        <v>0</v>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146775594</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>1193530958</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>【1+1】ポアシュリンカー バクチオールクリーム 60ml x 2個</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>マモンド</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>7560</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="b">
+        <v>0</v>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193530958</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>1152063267</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>低刺激 フェイスアンド ボディ 大容量 日焼け止め 150mL (SPF50+ PA++++)</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>シンムルナラ</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G166" t="n">
+        <v>2</v>
+      </c>
+      <c r="H166" t="b">
+        <v>0</v>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152063267</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>1196819316</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>グルタチオンビタシートマスク デイリーピック 30枚</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>2734</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="b">
+        <v>0</v>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196819316</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>1182043662</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>エクソソームシカ ツボクサ鎮静クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="b">
+        <v>0</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182043662</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J162"/>
+  <autoFilter ref="A1:J168"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 27, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$393</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$399</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J393"/>
+  <dimension ref="A1:J399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16568,8 +16568,254 @@
         </is>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>1109964483</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Beauty-Life</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>ハイドラローションマックス 400ml</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>エステダム</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>8125</v>
+      </c>
+      <c r="G394" t="n">
+        <v>0</v>
+      </c>
+      <c r="H394" t="b">
+        <v>0</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109964483</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>1109951025</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Beauty-Life</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>シアーシュガー スクラブ 510g 11種 ビタミンC</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Tree Hut</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>4225</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0</v>
+      </c>
+      <c r="H395" t="b">
+        <v>0</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109951025</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>1175324790</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>センシティブ スージング ジェルクリーム 100g ひんやりうるおい 低刺激 水分クリーム ベタつきにくい 敏感肌 朝夜兼用 オイルフリー ノンコメド印象 軽い使用感</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>2760</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0</v>
+      </c>
+      <c r="H396" t="b">
+        <v>0</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175324790</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>1201200397</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>アクネブレミッシュ鎮静ボディウォッシュ 460ml 背中ニキビ・肌トラブルを改善する 背中ニキビ・ボディのざらつきケア さっぱり洗浄 つっぱりにくい デイリー用</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Nodor</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>3970</v>
+      </c>
+      <c r="G397" t="n">
+        <v>3</v>
+      </c>
+      <c r="H397" t="b">
+        <v>0</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201200397</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>1148702438</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>KBEAUTYCREW</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>RXザビタミンC23セラム, 20ml</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G398" t="n">
+        <v>1</v>
+      </c>
+      <c r="H398" t="b">
+        <v>0</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148702438</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>1189376677</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>velaskin</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>[NEW]シェイキング シナジー ミスト 50ml / 保湿ミスト / ツヤミスト / メイクキープ / うるおいケア / ミスト化粧水</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>3637</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0</v>
+      </c>
+      <c r="H399" t="b">
+        <v>0</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189376677</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J393"/>
+  <autoFilter ref="A1:J399"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 30, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$399</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$411</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J399"/>
+  <dimension ref="A1:J411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16814,8 +16814,500 @@
         </is>
       </c>
     </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>1203766483</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ サーフィン サンスティック 20g</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>3201</v>
+      </c>
+      <c r="G400" t="n">
+        <v>0</v>
+      </c>
+      <c r="H400" t="b">
+        <v>0</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203766483</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>1096782550</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>アクア ヒアルロニック エッセンス 大容量, 250ml</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>3888</v>
+      </c>
+      <c r="G401" t="n">
+        <v>0</v>
+      </c>
+      <c r="H401" t="b">
+        <v>0</v>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096782550</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>1205563457</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>ガラクトミー エンザイム ピーリングジェル, 75ml, 1個</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>1829</v>
+      </c>
+      <c r="G402" t="n">
+        <v>0</v>
+      </c>
+      <c r="H402" t="b">
+        <v>0</v>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205563457</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>1171042034</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>アクティブクリーンアップクレンジングパウダー酵素洗顔剤, 80g</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>4005</v>
+      </c>
+      <c r="G403" t="n">
+        <v>1</v>
+      </c>
+      <c r="H403" t="b">
+        <v>0</v>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171042034</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>1212713877</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Lulupi</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>【フィー】 シェイキングシナジーミスト 50ml 全3種</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>2654</v>
+      </c>
+      <c r="G404" t="n">
+        <v>0</v>
+      </c>
+      <c r="H404" t="b">
+        <v>0</v>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212713877</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>1211134600</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>seimyongkorea</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>【NEW】 シェイキングミスト</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>2222</v>
+      </c>
+      <c r="G405" t="n">
+        <v>2</v>
+      </c>
+      <c r="H405" t="b">
+        <v>0</v>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211134600</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>1206908379</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>onme</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>(+マスクパック贈呈)MGFリターンクリーム 70ml 再生クリーム</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>8600</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0</v>
+      </c>
+      <c r="H406" t="b">
+        <v>0</v>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206908379</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>1136826440</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>onme</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>特許技術BBTMとともに安全に使用できる プレミアムビーガン女性用 プレミアム ビーガン 育毛シャンプー 韓国シャンプー 400ml</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>AGAIN ME</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>5050</v>
+      </c>
+      <c r="G407" t="n">
+        <v>1</v>
+      </c>
+      <c r="H407" t="b">
+        <v>0</v>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136826440</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>1213399617</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>SKINFOODHQ</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>【トナーパッド】キャロットカロテンカーミングウォーターパッド( 60枚入り, 2個)</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0</v>
+      </c>
+      <c r="H408" t="b">
+        <v>0</v>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213399617</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>1207120904</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>ALife07</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>ダーマトロジー クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>8823</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0</v>
+      </c>
+      <c r="H409" t="b">
+        <v>0</v>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207120904</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>1196025757</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>ALife07</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>ポア ダークスポット ブライトニングクリーム 35ml</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>1938</v>
+      </c>
+      <c r="G410" t="n">
+        <v>0</v>
+      </c>
+      <c r="H410" t="b">
+        <v>0</v>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196025757</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>1057808818</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>djshopping</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>LAB+トリプルウォーターピールスージングパッド 60枚</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>SNP</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G411" t="n">
+        <v>0</v>
+      </c>
+      <c r="H411" t="b">
+        <v>0</v>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1057808818</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J399"/>
+  <autoFilter ref="A1:J411"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 33, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$411</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$425</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J411"/>
+  <dimension ref="A1:J425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17306,8 +17306,582 @@
         </is>
       </c>
     </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>1196382835</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>HAPPYLADY</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>[100時間保湿/かゆみ緩和/会社員A] [正規品]シカサルブクリーム 230ml</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>MECHAI</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>5352</v>
+      </c>
+      <c r="G412" t="n">
+        <v>0</v>
+      </c>
+      <c r="H412" t="b">
+        <v>0</v>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196382835</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>1183055576</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Asteroid</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>シャンプー ダマスクローズの香り 1L</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>ミルクバオバブ</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>2745</v>
+      </c>
+      <c r="G413" t="n">
+        <v>0</v>
+      </c>
+      <c r="H413" t="b">
+        <v>0</v>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183055576</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>1133994465</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Asteroid</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>24K ラグジュアリー ゴールド アンプル 110ml</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>BERGAMO</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>3813</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0</v>
+      </c>
+      <c r="H414" t="b">
+        <v>0</v>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133994465</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>1206870778</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>mood_k</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>345 リリーフ クリームミスト 100ml+60ml 保湿ミスト 韓国コスメ 敏感肌 乾燥対策 フェイスミスト スキンケア</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>4240</v>
+      </c>
+      <c r="G415" t="n">
+        <v>0</v>
+      </c>
+      <c r="H415" t="b">
+        <v>0</v>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206870778</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>1209089569</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml1個 韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G416" t="n">
+        <v>0</v>
+      </c>
+      <c r="H416" t="b">
+        <v>0</v>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089569</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>1209089497</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml 2個 set/韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0</v>
+      </c>
+      <c r="H417" t="b">
+        <v>0</v>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089497</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>1177385233</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>フィックスディテールヘアマスカラ 15ml</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>チャホン</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>3230</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0</v>
+      </c>
+      <c r="H418" t="b">
+        <v>0</v>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177385233</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>1170230232</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>ドクダミシルキーモイスチャー日焼け止め 50ml</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G419" t="n">
+        <v>0</v>
+      </c>
+      <c r="H419" t="b">
+        <v>0</v>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170230232</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>1177545076</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>[!!超人気!!]ダーマヒーラーポアタイトニングトナーパッド 60枚</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G420" t="n">
+        <v>1</v>
+      </c>
+      <c r="H420" t="b">
+        <v>0</v>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177545076</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>1205368128</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>ドクダミポアディープクレンジングフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G421" t="n">
+        <v>0</v>
+      </c>
+      <c r="H421" t="b">
+        <v>0</v>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205368128</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>1195011504</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>doitsistersseoul</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>ドクダミ トラベル クレンジングセット (オイル20ml + フォーム25ml)</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G422" t="n">
+        <v>0</v>
+      </c>
+      <c r="H422" t="b">
+        <v>0</v>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195011504</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>1209905260</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>オドール オールインワン クリアボディウォッシュ 2個, 460ml</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Nodor</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>6898</v>
+      </c>
+      <c r="G423" t="n">
+        <v>0</v>
+      </c>
+      <c r="H423" t="b">
+        <v>0</v>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905260</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>1209905066</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>ポケモンエディションクリアボディミスト 200ml 企画 (ミニチュア 30ml + イーブイ防水パック)</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>NOT4U</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>3448</v>
+      </c>
+      <c r="G424" t="n">
+        <v>0</v>
+      </c>
+      <c r="H424" t="b">
+        <v>0</v>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905066</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>1209905054</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>ホワイトアプリコット ソリッドパフューム 塗る固体香水 フレグランス 携帯用 30ml</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>LUAFEE</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>2249</v>
+      </c>
+      <c r="G425" t="n">
+        <v>0</v>
+      </c>
+      <c r="H425" t="b">
+        <v>0</v>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905054</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J411"/>
+  <autoFilter ref="A1:J425"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 36, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$425</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$444</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J425"/>
+  <dimension ref="A1:J444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17880,8 +17880,787 @@
         </is>
       </c>
     </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>1196415617</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>【WiD2】 AHA・BHA配合 28デイズヒアルクリーム (30ml) ザラつきOFF！なめらか透明肌へ 1個</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G426" t="n">
+        <v>1</v>
+      </c>
+      <c r="H426" t="b">
+        <v>0</v>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196415617</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>1196366572</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>【WiD2】 ガラクトナイアシンエッセンスマスク 10枚入り 肌をクリアに・高保湿・エイジングケア</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>2851</v>
+      </c>
+      <c r="G427" t="n">
+        <v>0</v>
+      </c>
+      <c r="H427" t="b">
+        <v>0</v>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196366572</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>1189270361</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>【Wid】 フォリゲン トニック 120ml 2個セット・頭皮ケア・ヘアトニック・抜け毛予防・頭皮栄養・スカルプケア</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>5287</v>
+      </c>
+      <c r="G428" t="n">
+        <v>0</v>
+      </c>
+      <c r="H428" t="b">
+        <v>0</v>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189270361</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>1188452071</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>【Wid】 アスコルビルテトラィソパルミテート ソリューション 20% イン ビタミンF / 30ml / 1個 / ビタミンC美容液 / オイル美容液 / 透明感 / ハリケア</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>5841</v>
+      </c>
+      <c r="G429" t="n">
+        <v>0</v>
+      </c>
+      <c r="H429" t="b">
+        <v>0</v>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452071</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>1188452072</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>【Wid】 グリコール酸 7% エクスフォリエイティング トナー / 240ml / 2個セット / ふき取り化粧水 / 角質ケア / 肌キメ整え / ツヤ肌</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>6385</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0</v>
+      </c>
+      <c r="H430" t="b">
+        <v>0</v>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452072</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>1179809144</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>[角質ケア] マンデル酸 10％ + HA 30ml 毛穴ケア つるつる美肌 セラム</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0</v>
+      </c>
+      <c r="H431" t="b">
+        <v>0</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179809144</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>1211721947</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>ポアタイトニング クレンジングバーム 50ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G432" t="n">
+        <v>0</v>
+      </c>
+      <c r="H432" t="b">
+        <v>0</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211721947</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>1137919225</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>パンテノール クリームウォッシュ 300ml × 2本</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>6253</v>
+      </c>
+      <c r="G433" t="n">
+        <v>0</v>
+      </c>
+      <c r="H433" t="b">
+        <v>0</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137919225</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>1211388494</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>ウォーターカプセル サンセラム SPF50+ / PA+++ 40ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G434" t="n">
+        <v>0</v>
+      </c>
+      <c r="H434" t="b">
+        <v>0</v>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211388494</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>1190175660</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>マダガスカルセントラアンプル 55ml, 1個</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>2795</v>
+      </c>
+      <c r="G435" t="n">
+        <v>1</v>
+      </c>
+      <c r="H435" t="b">
+        <v>0</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175660</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>1190175438</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>ノーセバム サンクッション EX SPF50+ PA++++, 1個</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G436" t="n">
+        <v>0</v>
+      </c>
+      <c r="H436" t="b">
+        <v>0</v>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175438</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>1139859503</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>doricoco</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>【ポケモンコラボ限定】リリイーブ グロウターン エクソソーム ブラシアンプル 130ml + 30ml + ミニブラシ / 韓国頭皮ケア・育毛ケア</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>4390</v>
+      </c>
+      <c r="G437" t="n">
+        <v>0</v>
+      </c>
+      <c r="H437" t="b">
+        <v>0</v>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139859503</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>1117483504</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>doricoco</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>ヘアパフューム ヘアオイル4種30ml/ヘアエッセンス/毛髪の厚さ別に選択可能/香水 ヘアオイル/頭に塗る香水</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>La'dor</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>2560</v>
+      </c>
+      <c r="G438" t="n">
+        <v>0</v>
+      </c>
+      <c r="H438" t="b">
+        <v>0</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117483504</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>1183855839</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>ardistore</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>ジェイエムソリューション B5 ヒアモイスチャライジングクリーム 60ml 3本 JM 솔루션 B5 히어 모이스처라이징 크림 60ml 3병</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G439" t="n">
+        <v>0</v>
+      </c>
+      <c r="H439" t="b">
+        <v>0</v>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183855839</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>1208177592</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>ardistore</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>イェジフ ヨンビン 紅参化粧品 5種 1セット 예지후 영빈 홍삼 화장품 5종 1세트</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>禮知后</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G440" t="n">
+        <v>0</v>
+      </c>
+      <c r="H440" t="b">
+        <v>0</v>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208177592</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>1169201226</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>[1+1]ジェントルブラック フレッシュ クレンジングオイル 150ml+150ml</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>4584</v>
+      </c>
+      <c r="G441" t="n">
+        <v>0</v>
+      </c>
+      <c r="H441" t="b">
+        <v>0</v>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169201226</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>1110101930</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>フォリゲンシャンプー 500ml</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>2847</v>
+      </c>
+      <c r="G442" t="n">
+        <v>0</v>
+      </c>
+      <c r="H442" t="b">
+        <v>0</v>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110101930</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>1092755563</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>ベイキング パウダー サクサク 毛穴 スクラブ 200gx2個</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>エチュード</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>3148</v>
+      </c>
+      <c r="G443" t="n">
+        <v>5</v>
+      </c>
+      <c r="H443" t="b">
+        <v>0</v>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1092755563</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>1172777299</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>fmalwm</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>パフューム ヘアミスト サンセットフォグ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>ハクスリー</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>5833</v>
+      </c>
+      <c r="G444" t="n">
+        <v>0</v>
+      </c>
+      <c r="H444" t="b">
+        <v>0</v>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172777299</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J425"/>
+  <autoFilter ref="A1:J444"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 39, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$444</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$450</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J444"/>
+  <dimension ref="A1:J450"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18659,8 +18659,254 @@
         </is>
       </c>
     </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>1202396707</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュ フォーメン オイルカットローションオールインワン, 150ml, 1本</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>2373</v>
+      </c>
+      <c r="G445" t="n">
+        <v>0</v>
+      </c>
+      <c r="H445" t="b">
+        <v>0</v>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202396707</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>1204813717</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>大容量トナー ツボクサ グリーンダーマ マイルド シカ ビッグトナー 500ml</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>3230</v>
+      </c>
+      <c r="G446" t="n">
+        <v>2</v>
+      </c>
+      <c r="H446" t="b">
+        <v>0</v>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204813717</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>1204188494</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>ドクダミ シカ クーリング 水分 クリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>2760</v>
+      </c>
+      <c r="G447" t="n">
+        <v>0</v>
+      </c>
+      <c r="H447" t="b">
+        <v>0</v>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204188494</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>1201899429</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>ドクダミ 70 スージング コラーゲン マスク 4枚</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F448" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G448" t="n">
+        <v>0</v>
+      </c>
+      <c r="H448" t="b">
+        <v>0</v>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201899429</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>1188680199</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>relationmarketing</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>プラスリストア UVローション日焼け止めローション SPF50+ PA++++30ml</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>プラスリストア</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>3912</v>
+      </c>
+      <c r="G449" t="n">
+        <v>0</v>
+      </c>
+      <c r="H449" t="b">
+        <v>0</v>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188680199</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>1188680603</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>relationmarketing</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>ルベル IAU イオ クレンジング リラックスメント シャンプー 1000ml＆イオ クリーム シルキーリペア トリートメント1000ml 詰め替え セット</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>イオ</t>
+        </is>
+      </c>
+      <c r="F450" t="n">
+        <v>7709</v>
+      </c>
+      <c r="G450" t="n">
+        <v>1</v>
+      </c>
+      <c r="H450" t="b">
+        <v>0</v>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188680603</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J444"/>
+  <autoFilter ref="A1:J450"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 42, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$450</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$462</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J450"/>
+  <dimension ref="A1:J462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18905,8 +18905,500 @@
         </is>
       </c>
     </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1209051021</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>zeesea</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>全日オイルコントロールメイクキープミスト 化粧崩れ防止 [ミルキーウェイ],[スプレー],[セッティング]</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>ZEESEA</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G451" t="n">
+        <v>2</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209051021</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>1210528997</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>【1+1セット】クリーンティーツリーリポソーム カーミングマスク 5枚入×2個 ヒアルロン酸 パンテノール 水分 鎮静 保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F452" t="n">
+        <v>3069</v>
+      </c>
+      <c r="G452" t="n">
+        <v>0</v>
+      </c>
+      <c r="H452" t="b">
+        <v>0</v>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210528997</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>1210272622</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>【1+1セット】ウォータフルエッセンスサンクリーム SPF50+ PA++++ 50ml×2個 保湿 UVケア エッセンス 日焼け止め 化粧下地 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>6442</v>
+      </c>
+      <c r="G453" t="n">
+        <v>0</v>
+      </c>
+      <c r="H453" t="b">
+        <v>0</v>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210272622</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>1206508858</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>【1+1セット】ソフトリセット グリーンクレンジングバーム 100ml 2個 メイク落とし 保湿洗顔 角質ケア 毛穴汚れケア 韓国コスメ しっとりディープクレンジング</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>ヒュッゲ</t>
+        </is>
+      </c>
+      <c r="F454" t="n">
+        <v>6279</v>
+      </c>
+      <c r="G454" t="n">
+        <v>0</v>
+      </c>
+      <c r="H454" t="b">
+        <v>0</v>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206508858</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>1206240655</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>ウォーターtoアンプルトリートメント 200ml 1個 毛髪保湿 ツヤ髪ケア しっとりヘアケア ホームケア 韓国コスメ 上品な香り デイリーケア</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>6459</v>
+      </c>
+      <c r="G455" t="n">
+        <v>0</v>
+      </c>
+      <c r="H455" t="b">
+        <v>0</v>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206240655</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>781856183</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>モイスチャライジング トナー UFT （ウルトラフェイシャルトナー） 250ml</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>キールズ</t>
+        </is>
+      </c>
+      <c r="F456" t="n">
+        <v>3631</v>
+      </c>
+      <c r="G456" t="n">
+        <v>3</v>
+      </c>
+      <c r="H456" t="b">
+        <v>0</v>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=781856183</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>1204378750</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>フェイシャル トリートメント エッセンス 330ml 1個</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>SK-Ⅱ</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>33266</v>
+      </c>
+      <c r="G457" t="n">
+        <v>0</v>
+      </c>
+      <c r="H457" t="b">
+        <v>0</v>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204378750</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>1173903686</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>レプリカ ハンドクリーム レイジーサンデー モーニング 50ml/1.6fl.oz.</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F458" t="n">
+        <v>4191</v>
+      </c>
+      <c r="G458" t="n">
+        <v>1</v>
+      </c>
+      <c r="H458" t="b">
+        <v>0</v>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173903686</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>638382548</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>ヴァーベナ ボディローション 250ml</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>ロクシタン</t>
+        </is>
+      </c>
+      <c r="F459" t="n">
+        <v>3135</v>
+      </c>
+      <c r="G459" t="n">
+        <v>2</v>
+      </c>
+      <c r="H459" t="b">
+        <v>0</v>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=638382548</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>1059030924</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>strawberrynet-beauty</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Davines モアインサイド ディス イズ ア カールビルディング セラム (カールヘア用)</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>ダビネス</t>
+        </is>
+      </c>
+      <c r="F460" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G460" t="n">
+        <v>1</v>
+      </c>
+      <c r="H460" t="b">
+        <v>0</v>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1059030924</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>1135055592</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>strawberrynet-beauty</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Valentino バレンチノ ウォモ ボーン イン ローマ オー ド トワレ スプレー*</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>ヴァレンティノ</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>20200</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0</v>
+      </c>
+      <c r="H461" t="b">
+        <v>0</v>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135055592</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>1181475483</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>strawberrynet-beauty</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Giorgio Armani ルミナス シルク ファンデーション - # 4 (Light Sand) 202611</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>ジョルジオアルマーニ</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>10300</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0</v>
+      </c>
+      <c r="H462" t="b">
+        <v>0</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181475483</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J450"/>
+  <autoFilter ref="A1:J462"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 45, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$462</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$478</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J462"/>
+  <dimension ref="A1:J478"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19397,8 +19397,664 @@
         </is>
       </c>
     </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>1123317400</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>withgaia</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>[1+1]レッド センテラカ マスク 10枚</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>7390</v>
+      </c>
+      <c r="G463" t="n">
+        <v>1</v>
+      </c>
+      <c r="H463" t="b">
+        <v>0</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123317400</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>1133684811</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>withgaia</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>プレミアムブリリアントミスト, 90ml</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Kopher</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>5350</v>
+      </c>
+      <c r="G464" t="n">
+        <v>0</v>
+      </c>
+      <c r="H464" t="b">
+        <v>0</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133684811</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>1143959163</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>ggoolnim</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>ロレアルパリトタルリフェア5モイスチャークリームプロエックスヘアローション 110g x 1個 あるいは 2個 選択</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>アモーレパシフィック</t>
+        </is>
+      </c>
+      <c r="F465" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G465" t="n">
+        <v>1</v>
+      </c>
+      <c r="H465" t="b">
+        <v>0</v>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143959163</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>1206682479</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>cafebespoke</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>グリーンプロポリス 頭皮クレンジング シャンプー+トリートメント [1000ml+1000ml] セット</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F466" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G466" t="n">
+        <v>3</v>
+      </c>
+      <c r="H466" t="b">
+        <v>0</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206682479</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>1112935346</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>【選べる2個セット】デビルズ パフュームファンタジーシャンプー &amp;amp; コンディショナー, 1L+1L</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G467" t="n">
+        <v>1</v>
+      </c>
+      <c r="H467" t="b">
+        <v>0</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1112935346</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>1084157476</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>【NEW COLOR】イージーブロウトーンチェンジャー (5回分) /ブリーチ / 眉毛脱色 /眉カラーケア</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>サムバイミー</t>
+        </is>
+      </c>
+      <c r="F468" t="n">
+        <v>4110</v>
+      </c>
+      <c r="G468" t="n">
+        <v>0</v>
+      </c>
+      <c r="H468" t="b">
+        <v>0</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1084157476</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>1192529297</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>cald</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>ポア リフティング アンプル プラス 75ml</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>グリーントマト</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>3825</v>
+      </c>
+      <c r="G469" t="n">
+        <v>2</v>
+      </c>
+      <c r="H469" t="b">
+        <v>0</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192529297</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>1188176132</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>cald</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>デイリーケアマスクパック5枚企画4種（+1枚追加贈呈）</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F470" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G470" t="n">
+        <v>0</v>
+      </c>
+      <c r="H470" t="b">
+        <v>0</v>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188176132</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>1208012735</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>cald</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>【トーンアップ・UVケア】ディオプラス ブルーフェザー トーンアップ サンスクリーン 40ml</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>ディオプラス</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>3610</v>
+      </c>
+      <c r="G471" t="n">
+        <v>0</v>
+      </c>
+      <c r="H471" t="b">
+        <v>0</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208012735</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>1203960088</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>345リリーフクリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F472" t="n">
+        <v>2453</v>
+      </c>
+      <c r="G472" t="n">
+        <v>1</v>
+      </c>
+      <c r="H472" t="b">
+        <v>0</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203960088</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>1192047927</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%トーニングソリューション 240ml トーニング ソリューション</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F473" t="n">
+        <v>2216</v>
+      </c>
+      <c r="G473" t="n">
+        <v>2</v>
+      </c>
+      <c r="H473" t="b">
+        <v>0</v>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192047927</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>1205625745</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>パンテノールクリーム 80ml</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F474" t="n">
+        <v>2882</v>
+      </c>
+      <c r="G474" t="n">
+        <v>0</v>
+      </c>
+      <c r="H474" t="b">
+        <v>0</v>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205625745</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>1201757060</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>マルチペプチドセラムフォーヘアデンシティ 60ml 2個 ヘアケア</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F475" t="n">
+        <v>8612</v>
+      </c>
+      <c r="G475" t="n">
+        <v>0</v>
+      </c>
+      <c r="H475" t="b">
+        <v>0</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201757060</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>1194137533</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>ルティナー マルチバーム 15ml</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F476" t="n">
+        <v>4232</v>
+      </c>
+      <c r="G476" t="n">
+        <v>1</v>
+      </c>
+      <c r="H476" t="b">
+        <v>0</v>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194137533</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>1194137521</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>ユース シナジー リフティング ファーストエッセンス 100ml</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F477" t="n">
+        <v>6573</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0</v>
+      </c>
+      <c r="H477" t="b">
+        <v>0</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194137521</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>1194573796</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュクリアスージングクリーム, 70ml, 2個</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F478" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0</v>
+      </c>
+      <c r="H478" t="b">
+        <v>0</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194573796</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J462"/>
+  <autoFilter ref="A1:J478"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 48, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$478</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$485</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J478"/>
+  <dimension ref="A1:J485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20053,8 +20053,295 @@
         </is>
       </c>
     </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>1203144925</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>【企画】オールアバウト グロウ カバークリーム (35g) + 大王パフ 1枚付き SPF50+ PA++++ 韓国コスメ ベースメイク 24時間持続 崩れない</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>CHASIN’ RABBITS</t>
+        </is>
+      </c>
+      <c r="F479" t="n">
+        <v>1946</v>
+      </c>
+      <c r="G479" t="n">
+        <v>1</v>
+      </c>
+      <c r="H479" t="b">
+        <v>0</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203144925</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>1186319083</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>韓国正規品 AMPLE:N ペプチドショットアンプル2X 100ml 大容量美容液 ペプチド 高保湿 ハリケア 弾力ケア 韓国コスメ 韓国直送</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F480" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G480" t="n">
+        <v>0</v>
+      </c>
+      <c r="H480" t="b">
+        <v>0</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186319083</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>1174996099</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>韓国正規品 3Dハリクリームセット 50ml 美容液15ml+ミスト20ml付 豪華2点特典 保湿 ハリケア 韓国コスメ 韓国直送</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F481" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G481" t="n">
+        <v>1</v>
+      </c>
+      <c r="H481" t="b">
+        <v>0</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174996099</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>1213260537</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>韓国正規品 リニューアル MLE保湿ローション 120ml／200ml 敏感肌 乾燥肌 ベビー 全身 肌バリア 韓国直送</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F482" t="n">
+        <v>2465</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0</v>
+      </c>
+      <c r="H482" t="b">
+        <v>0</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213260537</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>1171696930</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>C2Y</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>ワセリン マスクパック シリーズ 3種 23ml*30枚(1箱10枚入)/保湿ケア/水分/シカ/弾力 3種 選択</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>C2Y</t>
+        </is>
+      </c>
+      <c r="F483" t="n">
+        <v>3726</v>
+      </c>
+      <c r="G483" t="n">
+        <v>0</v>
+      </c>
+      <c r="H483" t="b">
+        <v>0</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171696930</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>1193418611</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>KVIVE</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>ヒーラー ポア タイトニング トナーパッド 本品60枚+詰め替え用 60枚入り/PDRN トナーパッド 美容液 /韓国 人気 トナーパッド/弾力/保湿/水分アンプル/c-PDRN/エイジングケアトナー</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F484" t="n">
+        <v>6870</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0</v>
+      </c>
+      <c r="H484" t="b">
+        <v>0</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193418611</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>1191891158</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>KVIVE</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>赤小豆 毛穴クレイマスク 140ml + 水分ウォータージェル 100ml セット/毛穴ケア/皮脂ケア/角質ケア/毛穴汚れ/韓国コスメ/韓国スキンケア/boj 赤小豆/米蜜グロウマスク</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F485" t="n">
+        <v>7130</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0</v>
+      </c>
+      <c r="H485" t="b">
+        <v>0</v>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191891158</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J478"/>
+  <autoFilter ref="A1:J485"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 51, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$485</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$498</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J485"/>
+  <dimension ref="A1:J498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20340,8 +20340,541 @@
         </is>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>1212343699</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>pickary</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>【5枚入り】 垢すりグローブ ソフトボディ レッドグローブ クリーン角質ケア・ボディクレンジング 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F486" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0</v>
+      </c>
+      <c r="H486" t="b">
+        <v>0</v>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212343699</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>1192678454</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】 肌荒れ・乾燥くすみ対策に！エイシカ365 トラブルリリーフセラムpH4.5 40ml 肌荒れ くすみ 乾燥 美容液</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F487" t="n">
+        <v>2910</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0</v>
+      </c>
+      <c r="H487" t="b">
+        <v>0</v>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192678454</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>1192676012</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】アトバリア365 クリーム 80mL 保湿クリーム 水分クリーム 保湿カプセル セラミド クリーム 肌荒れ 水分</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F488" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G488" t="n">
+        <v>1</v>
+      </c>
+      <c r="H488" t="b">
+        <v>0</v>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192676012</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>1192160801</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>レチノール シカ リペア セラム 30mL</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F489" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0</v>
+      </c>
+      <c r="H489" t="b">
+        <v>0</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192160801</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>1192597637</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>strawberryshop</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Axenda ルティナー クリーム 毛穴バーム スリープバーム マルチバーム 15ml 2個</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F490" t="n">
+        <v>9850</v>
+      </c>
+      <c r="G490" t="n">
+        <v>0</v>
+      </c>
+      <c r="H490" t="b">
+        <v>0</v>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192597637</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>1189809546</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>strawberryshop</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>レッドフィルティンググルセラム 35ml + レッドピルホワイトセラム 35ML</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F491" t="n">
+        <v>6999</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0</v>
+      </c>
+      <c r="H491" t="b">
+        <v>0</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189809546</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>1123787663</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>BOMAMALL</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>UVイデア XL プロテクショントーンアップ ローズ 30ml</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>ラロッシュポゼ</t>
+        </is>
+      </c>
+      <c r="F492" t="n">
+        <v>6961</v>
+      </c>
+      <c r="G492" t="n">
+        <v>0</v>
+      </c>
+      <c r="H492" t="b">
+        <v>0</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123787663</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>1146152293</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>BOMAMALL</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>パフュームヘアトリートメント/ヒノキ/ふんわりヒノキの香り/Hinoki/香水のトリートメント/髪の栄養と香りを一度に解決/毛髪栄養改善/毛髪切れ改善/柔らかさ改善</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>La'dor</t>
+        </is>
+      </c>
+      <c r="F493" t="n">
+        <v>5811</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0</v>
+      </c>
+      <c r="H493" t="b">
+        <v>0</v>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146152293</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>1205514714</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Nandak</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>[ダーママスク10枚プレゼント] マデカクリームハイドラカーミング50ml3個韓国人気化粧品</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F494" t="n">
+        <v>5850</v>
+      </c>
+      <c r="G494" t="n">
+        <v>1</v>
+      </c>
+      <c r="H494" t="b">
+        <v>0</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205514714</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>1093898160</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>発酵豆 バウンス タンパク質 エッセンス 80ml/低刺激/保湿/水分/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>フラスキン</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>4372</v>
+      </c>
+      <c r="G495" t="n">
+        <v>0</v>
+      </c>
+      <c r="H495" t="b">
+        <v>0</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093898160</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>1096256291</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>【正規品】コラーゲンプロフェッショナルプログラムセット (マイクロコラーゲン200mg*4ea+アクティベーションブースター30ml+ドロッパー4ea)/コラーゲン/光沢/高栄養/活力/弾力</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>LAVIEN</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>15010</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0</v>
+      </c>
+      <c r="H496" t="b">
+        <v>0</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096256291</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>1094315646</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>【1+1】ブイ コラーゲン ハートフィット マルチバーム 10g/肌バリアケア/ スローエイジング/ 高濃縮/ 弾力/ 水分バリア/ 鎮静/ 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>6786</v>
+      </c>
+      <c r="G497" t="n">
+        <v>1</v>
+      </c>
+      <c r="H497" t="b">
+        <v>0</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094315646</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>1093734916</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>【1+1】スピキュールセラム(ニードルアクション100) 30ml/ 塗る毛穴セラム針 / ニードルショット / ブースティングセラム / 肌のキメ改善 / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>BIOME ACTIVATE</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0</v>
+      </c>
+      <c r="H498" t="b">
+        <v>0</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093734916</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J485"/>
+  <autoFilter ref="A1:J498"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 54, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$498</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$515</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J498"/>
+  <dimension ref="A1:J515"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20873,8 +20873,705 @@
         </is>
       </c>
     </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>1097540476</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>EPONA</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>【公式】 プレミアム紅参ゴールドクリーム / 50ml / 1個</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>エポナ</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>5090</v>
+      </c>
+      <c r="G499" t="n">
+        <v>1</v>
+      </c>
+      <c r="H499" t="b">
+        <v>0</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097540476</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>1175249089</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>ザ セラミド スキンバリア モイスチャライザークリーム 80ml 2個</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F500" t="n">
+        <v>6230</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0</v>
+      </c>
+      <c r="H500" t="b">
+        <v>0</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175249089</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>1152704413</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>オーガニック ホホバオイル ゴールド 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>FRANCOISE&amp;amp;Fragrance</t>
+        </is>
+      </c>
+      <c r="F501" t="n">
+        <v>2506</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0</v>
+      </c>
+      <c r="H501" t="b">
+        <v>0</v>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152704413</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>1154992110</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>レッド ブレミッシュ スージング アップ サンクリーム SPF50+ PA++++ 50ml 2個</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F502" t="n">
+        <v>4149</v>
+      </c>
+      <c r="G502" t="n">
+        <v>0</v>
+      </c>
+      <c r="H502" t="b">
+        <v>0</v>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154992110</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>1154991907</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラ エアフィット サンクリーム プラス 50ml 2個</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F503" t="n">
+        <v>3984</v>
+      </c>
+      <c r="G503" t="n">
+        <v>0</v>
+      </c>
+      <c r="H503" t="b">
+        <v>0</v>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154991907</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>1202152284</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Probioderm Collagen Remodeling Booster Shot Program 35ml</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F504" t="n">
+        <v>3360</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0</v>
+      </c>
+      <c r="H504" t="b">
+        <v>0</v>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202152284</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>1202519032</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>[Glory exclusive]AZ Care Cleansing Oil, 200mL</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F505" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G505" t="n">
+        <v>0</v>
+      </c>
+      <c r="H505" t="b">
+        <v>0</v>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202519032</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>1202165457</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>[RYO] Root Gen Hair Loss Care Scalp Essence, 80mL</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>No Brand</t>
+        </is>
+      </c>
+      <c r="F506" t="n">
+        <v>2040</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0</v>
+      </c>
+      <c r="H506" t="b">
+        <v>0</v>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202165457</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>1162421706</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>クラシック ウォームコットン EDP 30ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>クリーン</t>
+        </is>
+      </c>
+      <c r="F507" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G507" t="n">
+        <v>0</v>
+      </c>
+      <c r="H507" t="b">
+        <v>0</v>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162421706</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>1159643310</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>ハッピー フォーメン EDC 50ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>クリニーク</t>
+        </is>
+      </c>
+      <c r="F508" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G508" t="n">
+        <v>0</v>
+      </c>
+      <c r="H508" t="b">
+        <v>0</v>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159643310</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>1158430479</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>アベンヌウォーター 300ml 3本セット （化粧水）</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>アベンヌ</t>
+        </is>
+      </c>
+      <c r="F509" t="n">
+        <v>3620</v>
+      </c>
+      <c r="G509" t="n">
+        <v>3</v>
+      </c>
+      <c r="H509" t="b">
+        <v>0</v>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158430479</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>1110913352</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>hottempr</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Olive Young ideal FOR MEN パーフェクト オールインワン企画 (オールインワン150ml+150ml)</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>アイデアルforメンズ</t>
+        </is>
+      </c>
+      <c r="F510" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G510" t="n">
+        <v>0</v>
+      </c>
+      <c r="H510" t="b">
+        <v>0</v>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110913352</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>1193980815</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>hottempr</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>【産毛スタイリング】ハイプフィットヘアケアマスカラ／ハードフィックスヘアマスカラ／エギョモリ／バーコード前髪／韓国アイドルヘア／アホ毛スティック／前髪アレンジ</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>narka</t>
+        </is>
+      </c>
+      <c r="F511" t="n">
+        <v>2960</v>
+      </c>
+      <c r="G511" t="n">
+        <v>0</v>
+      </c>
+      <c r="H511" t="b">
+        <v>0</v>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193980815</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>1203744619</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>ベルベット クレンジング ミルク 200ml x 2 お得な2個セット</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F512" t="n">
+        <v>6230</v>
+      </c>
+      <c r="G512" t="n">
+        <v>0</v>
+      </c>
+      <c r="H512" t="b">
+        <v>0</v>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203744619</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>1173946856</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>デイリーPD 50ml/1.7fl.oz.</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>ZO SKIN</t>
+        </is>
+      </c>
+      <c r="F513" t="n">
+        <v>21465</v>
+      </c>
+      <c r="G513" t="n">
+        <v>0</v>
+      </c>
+      <c r="H513" t="b">
+        <v>0</v>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173946856</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>1154827017</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>メン ハード バーム 60g</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F514" t="n">
+        <v>1979</v>
+      </c>
+      <c r="G514" t="n">
+        <v>0</v>
+      </c>
+      <c r="H514" t="b">
+        <v>0</v>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154827017</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>1204744207</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>TOMOSONGSTORE</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>リードルショット 300 50ml 2個セット（1+1）</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F515" t="n">
+        <v>8720</v>
+      </c>
+      <c r="G515" t="n">
+        <v>0</v>
+      </c>
+      <c r="H515" t="b">
+        <v>0</v>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204744207</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J498"/>
+  <autoFilter ref="A1:J515"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 57, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$515</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$526</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J515"/>
+  <dimension ref="A1:J526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21570,8 +21570,459 @@
         </is>
       </c>
     </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>1206857284</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>k_town</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>【正規品】コンブチャミスト 100ml + 選べるプレゼント / スペシャルケアマスクパック</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>エリシャコイ</t>
+        </is>
+      </c>
+      <c r="F516" t="n">
+        <v>2123</v>
+      </c>
+      <c r="G516" t="n">
+        <v>0</v>
+      </c>
+      <c r="H516" t="b">
+        <v>0</v>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206857284</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>1193149194</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>realkbeauty</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>[NEW] A.G.E. インタラプター ウルトラ弾力リフティングセラムセット(+4ml+ 4ml+ 4ml)＋スーパーカラゲンマスク</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>スキンシューティカルズ</t>
+        </is>
+      </c>
+      <c r="F517" t="n">
+        <v>21695</v>
+      </c>
+      <c r="G517" t="n">
+        <v>0</v>
+      </c>
+      <c r="H517" t="b">
+        <v>0</v>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193149194</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>1190578211</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>realkbeauty</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>デイリーマスク7種+1マスク/毛穴の弾力 ドングリ/ニキビ跡 ジャガイモ/水分保湿 キャロット/ビタユズ/美白 栄養ライス/肌の鎮静/バジルティーツリー</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F518" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G518" t="n">
+        <v>0</v>
+      </c>
+      <c r="H518" t="b">
+        <v>0</v>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190578211</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>1139807140</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>gpgp</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>パルファムボディウォッシュ/ 500ml/ 2個</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>ミルクバオバブ</t>
+        </is>
+      </c>
+      <c r="F519" t="n">
+        <v>3492</v>
+      </c>
+      <c r="G519" t="n">
+        <v>0</v>
+      </c>
+      <c r="H519" t="b">
+        <v>0</v>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139807140</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>1139805675</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>gpgp</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>オードパルファム(07シュガーフローラル)/ 25ml/ 1個</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F520" t="n">
+        <v>5505</v>
+      </c>
+      <c r="G520" t="n">
+        <v>1</v>
+      </c>
+      <c r="H520" t="b">
+        <v>0</v>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139805675</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>1203684966</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>elom トラブルスケーリングパッチマスク 3枚 /トラブルケア</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>EIoM</t>
+        </is>
+      </c>
+      <c r="F521" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G521" t="n">
+        <v>0</v>
+      </c>
+      <c r="H521" t="b">
+        <v>0</v>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203684966</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>1179656795</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>こすアールエックス ワンステップパッド/おじさんパッド/ピンプルパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F522" t="n">
+        <v>3490</v>
+      </c>
+      <c r="G522" t="n">
+        <v>0</v>
+      </c>
+      <c r="H522" t="b">
+        <v>0</v>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179656795</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>1190674241</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>カロテンクラリファイングビタパッド, 60枚</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F523" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G523" t="n">
+        <v>0</v>
+      </c>
+      <c r="H523" t="b">
+        <v>0</v>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190674241</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>1202082347</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>lindalinda</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>【垢すり/角質ケア】ソフトボディ レッドグローブ クリーン 1BOX(5枚入) / 個包装 / ボディクレンジング / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F524" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G524" t="n">
+        <v>5</v>
+      </c>
+      <c r="H524" t="b">
+        <v>0</v>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202082347</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>1138225289</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>dreamus</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>シグネチャーパルファム, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F525" t="n">
+        <v>5517</v>
+      </c>
+      <c r="G525" t="n">
+        <v>0</v>
+      </c>
+      <c r="H525" t="b">
+        <v>0</v>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138225289</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>1109209881</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>korkorshop</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>[NEW]ヒストラップイージーエフコンプレックスアンプル63％80ml / EGF</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>HISTOLAB</t>
+        </is>
+      </c>
+      <c r="F526" t="n">
+        <v>9737</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0</v>
+      </c>
+      <c r="H526" t="b">
+        <v>0</v>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109209881</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J515"/>
+  <autoFilter ref="A1:J526"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 60, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$526</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$537</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J526"/>
+  <dimension ref="A1:J537"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22021,8 +22021,459 @@
         </is>
       </c>
     </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>1211103356</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>ツバキディープコラーゲン弾力アンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F527" t="n">
+        <v>2160</v>
+      </c>
+      <c r="G527" t="n">
+        <v>0</v>
+      </c>
+      <c r="H527" t="b">
+        <v>0</v>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211103356</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>1192583562</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>ツバキディープコラーゲン弾力クリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F528" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G528" t="n">
+        <v>0</v>
+      </c>
+      <c r="H528" t="b">
+        <v>0</v>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192583562</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>1192583554</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>[正規品] Biodance ハイドロセラノールアンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F529" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G529" t="n">
+        <v>0</v>
+      </c>
+      <c r="H529" t="b">
+        <v>0</v>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192583554</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>1213549964</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>【SEVENTEEN ミンギュ ミニスタンディ2種付き】アノブ 選べるヘアケアセット / ヘアオイル / 洗い流さないトリートメント / シャンプー / ヘアマスク / 韓国ヘアケア</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F530" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G530" t="n">
+        <v>0</v>
+      </c>
+      <c r="H530" t="b">
+        <v>0</v>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213549964</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>1206876078</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>[1+1] 復活草ビフィダセラム ファーミングドロップ 50ml</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F531" t="n">
+        <v>3660</v>
+      </c>
+      <c r="G531" t="n">
+        <v>0</v>
+      </c>
+      <c r="H531" t="b">
+        <v>0</v>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206876078</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>1194719971</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>アイラッシュ ティンティング セラム ショット 1個</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>ミュード</t>
+        </is>
+      </c>
+      <c r="F532" t="n">
+        <v>1790</v>
+      </c>
+      <c r="G532" t="n">
+        <v>1</v>
+      </c>
+      <c r="H532" t="b">
+        <v>0</v>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194719971</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>1211535086</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>【選べる2点SET】PDRNゼリーセラムミスト/キャビアPDRNリアルディープマスク(4枚)/PDRNリポソームバブルブースター</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F533" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G533" t="n">
+        <v>0</v>
+      </c>
+      <c r="H533" t="b">
+        <v>0</v>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211535086</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>1073637416</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>バイタル ハイドラ ソリューション ハイドロプランプ ウォータークリーム 50ml 1EA</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F534" t="n">
+        <v>3170</v>
+      </c>
+      <c r="G534" t="n">
+        <v>0</v>
+      </c>
+      <c r="H534" t="b">
+        <v>0</v>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1073637416</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>1073637368</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>シカペア スリーペア インテンシブ S リペア マスク 75ml 1EA</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>3340</v>
+      </c>
+      <c r="G535" t="n">
+        <v>0</v>
+      </c>
+      <c r="H535" t="b">
+        <v>0</v>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1073637368</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>1141815797</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>skincept</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>[正規品] ヒョヨン 自養(ジャヤン) アイクリーム30ml+クリーム15ml贈呈_蓮華ステムセル/ハリ_目元の弾力/保湿/集中栄養ケア</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>クダモノナラ</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G536" t="n">
+        <v>1</v>
+      </c>
+      <c r="H536" t="b">
+        <v>0</v>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141815797</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>1194263979</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>skincept</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>[1+1] フレグランスボディウォッシュ 600mlx2個セット_選べる2種 [White Musk/Citrus]_ブライトニング/パフューム ボディクレンザー</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>VEILMENT</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>3700</v>
+      </c>
+      <c r="G537" t="n">
+        <v>0</v>
+      </c>
+      <c r="H537" t="b">
+        <v>0</v>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194263979</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J526"/>
+  <autoFilter ref="A1:J537"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 63, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$537</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J537"/>
+  <dimension ref="A1:J550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22472,8 +22472,541 @@
         </is>
       </c>
     </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>1080048114</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>ルミワイズブライトニングアンプルセラム30mL</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>雪花秀</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>12299</v>
+      </c>
+      <c r="G538" t="n">
+        <v>0</v>
+      </c>
+      <c r="H538" t="b">
+        <v>0</v>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080048114</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>1067976758</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>クレンジングミルク500ml/カレンデュラクリーム75ml</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Bioturm</t>
+        </is>
+      </c>
+      <c r="F539" t="n">
+        <v>6299</v>
+      </c>
+      <c r="G539" t="n">
+        <v>0</v>
+      </c>
+      <c r="H539" t="b">
+        <v>0</v>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1067976758</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>1210139793</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>UV プロテクター トーンアップ ピーチ / ラベンダー 50ml SPF50+ PA++++ トーンアップ 日焼け止め UVカット＆保湿ケア</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>ヘラ</t>
+        </is>
+      </c>
+      <c r="F540" t="n">
+        <v>3699</v>
+      </c>
+      <c r="G540" t="n">
+        <v>0</v>
+      </c>
+      <c r="H540" t="b">
+        <v>0</v>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210139793</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>1202568510</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>HonestHouse</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>プロテインクリニック 10000 タンパク質 1L (シャンプー／トリートメント)</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>エラスティン</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G541" t="n">
+        <v>0</v>
+      </c>
+      <c r="H541" t="b">
+        <v>0</v>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202568510</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>1191542494</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>HonestHouse</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>モデリングパック スーパーレモン グルタチオン 10個</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F542" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G542" t="n">
+        <v>0</v>
+      </c>
+      <c r="H542" t="b">
+        <v>0</v>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191542494</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>1209154400</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>AnchorBlue</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>[密着ハリツヤ/5枚入] コラーゲン 100 メルティング シート マスク 2.5g x 5枚 / 濃密 潤い 水分 パッチ 弾力 肌キメ ス킨케어 高保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F543" t="n">
+        <v>7376</v>
+      </c>
+      <c r="G543" t="n">
+        <v>0</v>
+      </c>
+      <c r="H543" t="b">
+        <v>0</v>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209154400</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>1208338165</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>AnchorBlue</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>[サロン級ホームケア] エクストリーム ダメージ クリニック ヘア アンプル 10ml 9個入り / 傷んだ髪 高濃縮 補修 保湿 ツヤ髪 トリートメント 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F544" t="n">
+        <v>3818</v>
+      </c>
+      <c r="G544" t="n">
+        <v>0</v>
+      </c>
+      <c r="H544" t="b">
+        <v>0</v>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208338165</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>1199411031</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>[2+2] 白樺 水分 日焼け止めスプレー, 100ml 4ea(SPF 50 + PA ++++)</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F545" t="n">
+        <v>6007</v>
+      </c>
+      <c r="G545" t="n">
+        <v>0</v>
+      </c>
+      <c r="H545" t="b">
+        <v>0</v>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199411031</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>1136125175</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>テラクネ 365 ハイドロ アクティブ トナー 化粧水, 200ml</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F546" t="n">
+        <v>2967</v>
+      </c>
+      <c r="G546" t="n">
+        <v>5</v>
+      </c>
+      <c r="H546" t="b">
+        <v>0</v>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136125175</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>1143335244</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>jjunabeauty</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>[CLAIR-GYN]クレアジン 女性ウォッシュ 200ml+50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Hanmi PRO-CALM</t>
+        </is>
+      </c>
+      <c r="F547" t="n">
+        <v>2467</v>
+      </c>
+      <c r="G547" t="n">
+        <v>0</v>
+      </c>
+      <c r="H547" t="b">
+        <v>0</v>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143335244</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>1129888999</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>jjunabeauty</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>スージング リペアクリーム R4, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>DERMAFIRM</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>3828</v>
+      </c>
+      <c r="G548" t="n">
+        <v>0</v>
+      </c>
+      <c r="H548" t="b">
+        <v>0</v>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1129888999</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>1202055978</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>UVクリーム SPF50+ PA ++++ 敏感肌向けトーンアップ韓国コスメの人気日焼け止め</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G549" t="n">
+        <v>0</v>
+      </c>
+      <c r="H549" t="b">
+        <v>0</v>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202055978</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>1174315936</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>1. マデカラボ マスク 10枚×2箱（リンクル リバイタライズ）</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G550" t="n">
+        <v>0</v>
+      </c>
+      <c r="H550" t="b">
+        <v>0</v>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174315936</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J537"/>
+  <autoFilter ref="A1:J550"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 66, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$561</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J550"/>
+  <dimension ref="A1:J561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23005,8 +23005,459 @@
         </is>
       </c>
     </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>1087617512</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>QueenMall</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>パフューム スプレー ボディローション 250ml 5種</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>hedn</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>4320</v>
+      </c>
+      <c r="G551" t="n">
+        <v>1</v>
+      </c>
+      <c r="H551" t="b">
+        <v>0</v>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1087617512</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>1170080586</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>QueenMall</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>PDRN ピンク ジェル ツーフォーム クレンザー 200ml 企画(+クレンジングブラシ 贈呈)</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F552" t="n">
+        <v>2972</v>
+      </c>
+      <c r="G552" t="n">
+        <v>0</v>
+      </c>
+      <c r="H552" t="b">
+        <v>0</v>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170080586</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>1199098148</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>kiri</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>[モンチッチコラボ] ベージュトーンアップ365ヴィーガンサンクリーム 40ml SPF50 トーンアップUV ノーファンデ 化粧下地 韓国日焼け止め</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>アミューズ</t>
+        </is>
+      </c>
+      <c r="F553" t="n">
+        <v>3470</v>
+      </c>
+      <c r="G553" t="n">
+        <v>1</v>
+      </c>
+      <c r="H553" t="b">
+        <v>0</v>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199098148</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>1109779971</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>[V T] リードルショット 2ステップ マスク 5枚セット (50/100/300) 針美容 毛穴 導入 フェイスパック 集中ケア スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F554" t="n">
+        <v>2739</v>
+      </c>
+      <c r="G554" t="n">
+        <v>0</v>
+      </c>
+      <c r="H554" t="b">
+        <v>0</v>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109779971</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>1192596376</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>[メガ割] manyo factory 魔女工場 ガラクナイアシン エッセンス クリーム 50ml ガラクトミセス 保湿 弾力 ハリ ツヤ 潤い 浸透 スキンケア 基礎化粧品 韓国コスメ 人気 公式</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F555" t="n">
+        <v>4726</v>
+      </c>
+      <c r="G555" t="n">
+        <v>0</v>
+      </c>
+      <c r="H555" t="b">
+        <v>0</v>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192596376</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>1193869990</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>[1+1特典] S*NATURE エ*スネイチャー アクア スクワラン 水分クリーム 2個セット 120ml 保湿 ツヤ肌 卵肌 韓国 スキンケア オリーブヤング プレゼント 敏感肌 乾燥肌</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>エスネイチャー</t>
+        </is>
+      </c>
+      <c r="F556" t="n">
+        <v>3930</v>
+      </c>
+      <c r="G556" t="n">
+        <v>0</v>
+      </c>
+      <c r="H556" t="b">
+        <v>0</v>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193869990</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>1190058759</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>slowhummingjp</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>【Slow Humming公式】フルーティナリーリリーフパフュームバーム 6.5g タッチピーチ/練り香水/香水/パヒューム/ヘアパヒューム</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Slow Humming</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G557" t="n">
+        <v>0</v>
+      </c>
+      <c r="H557" t="b">
+        <v>0</v>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190058759</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>1135414332</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>calluna</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>[ギフト包装] ミスト セラム 100ml + ハンドクリーム 30ml + 鏡</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F558" t="n">
+        <v>3934</v>
+      </c>
+      <c r="G558" t="n">
+        <v>2</v>
+      </c>
+      <c r="H558" t="b">
+        <v>0</v>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135414332</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>1170532806</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>calluna</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>【ポムポムプリン限定企画】ビーガンパックレンザー3種択1 (グリーントマト120ml/ レッドトマト120ml/ ライスドウ130ml)</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>FULLY</t>
+        </is>
+      </c>
+      <c r="F559" t="n">
+        <v>2525</v>
+      </c>
+      <c r="G559" t="n">
+        <v>3</v>
+      </c>
+      <c r="H559" t="b">
+        <v>0</v>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170532806</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>1102457193</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>JJDD</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>ブランマジックティーツリーオイル 20ml 5倍高濃縮ティーツリー成分 /ニキビ超急速ケア/赤ニキビ,白ニキビ,大人ニキビ,思春期ニキビ,ニキビ跡</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>ブランネイチャー</t>
+        </is>
+      </c>
+      <c r="F560" t="n">
+        <v>2350</v>
+      </c>
+      <c r="G560" t="n">
+        <v>1</v>
+      </c>
+      <c r="H560" t="b">
+        <v>0</v>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102457193</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>1081864235</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>kor-store</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>テリーファーマー 160g スタンダード ホテルタオル 10枚 タオル タオルセット タオル 洗面タオル 輪</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Terry Special</t>
+        </is>
+      </c>
+      <c r="F561" t="n">
+        <v>4930</v>
+      </c>
+      <c r="G561" t="n">
+        <v>0</v>
+      </c>
+      <c r="H561" t="b">
+        <v>0</v>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1081864235</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J550"/>
+  <autoFilter ref="A1:J561"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 69, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$561</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$571</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J561"/>
+  <dimension ref="A1:J571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23456,8 +23456,418 @@
         </is>
       </c>
     </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>1209641531</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>[1+]NEWサイトカインブースタープロ 70ml＋70ml</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Refilled</t>
+        </is>
+      </c>
+      <c r="F562" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G562" t="n">
+        <v>0</v>
+      </c>
+      <c r="H562" t="b">
+        <v>0</v>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209641531</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>1209148971</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>【韓国正規品/NEW】Gureum o de perfume EDP 50ml</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F563" t="n">
+        <v>11419</v>
+      </c>
+      <c r="G563" t="n">
+        <v>0</v>
+      </c>
+      <c r="H563" t="b">
+        <v>0</v>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209148971</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>1206526891</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>[NEW]エアロクーリングシャンプー 400ml＋70ml / -5.2度急速冷却</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F564" t="n">
+        <v>3859</v>
+      </c>
+      <c r="G564" t="n">
+        <v>0</v>
+      </c>
+      <c r="H564" t="b">
+        <v>0</v>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206526891</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>1129908462</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>leelix</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>PHセンシティブ クリーム 60ml x 2個セット (チューブタイプ 高保湿 敏感肌)</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>9322</v>
+      </c>
+      <c r="G565" t="n">
+        <v>0</v>
+      </c>
+      <c r="H565" t="b">
+        <v>0</v>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1129908462</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>1132004375</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>leelix</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>フルフィット プロポリス ライト アンプル 40ml +40ml</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F566" t="n">
+        <v>3996</v>
+      </c>
+      <c r="G566" t="n">
+        <v>1</v>
+      </c>
+      <c r="H566" t="b">
+        <v>0</v>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132004375</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>1101761023</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>sharonne</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>[NEW]オールデイ ノーセバム トーンアップ サンクッション / SPF50+ PA++++ / UVカット / トーンアップ / ノーセバム / 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F567" t="n">
+        <v>3321</v>
+      </c>
+      <c r="G567" t="n">
+        <v>1</v>
+      </c>
+      <c r="H567" t="b">
+        <v>0</v>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1101761023</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>1074817764</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>sharonne</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>紅茶栄養頭皮シャンプー450ml</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>ANILLO</t>
+        </is>
+      </c>
+      <c r="F568" t="n">
+        <v>6124</v>
+      </c>
+      <c r="G568" t="n">
+        <v>0</v>
+      </c>
+      <c r="H568" t="b">
+        <v>0</v>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1074817764</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>1188002169</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>steadyseller</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>リフティングクリーム 1618 グローラディアンス 保湿 50ml</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>AlpenMOOR1618</t>
+        </is>
+      </c>
+      <c r="F569" t="n">
+        <v>1690</v>
+      </c>
+      <c r="G569" t="n">
+        <v>0</v>
+      </c>
+      <c r="H569" t="b">
+        <v>0</v>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188002169</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>1179082021</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>steadyseller</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>エクソソーム PDRN ブースター アンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>IZEZE</t>
+        </is>
+      </c>
+      <c r="F570" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G570" t="n">
+        <v>0</v>
+      </c>
+      <c r="H570" t="b">
+        <v>0</v>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179082021</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>1204443091</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>steadyseller</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>プレミアム水染め 3+3リフィル企画 3種 択1</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>SEEDBEE</t>
+        </is>
+      </c>
+      <c r="F571" t="n">
+        <v>4470</v>
+      </c>
+      <c r="G571" t="n">
+        <v>0</v>
+      </c>
+      <c r="H571" t="b">
+        <v>0</v>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204443091</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J561"/>
+  <autoFilter ref="A1:J571"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 72, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$571</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$584</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J571"/>
+  <dimension ref="A1:J584"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23866,8 +23866,541 @@
         </is>
       </c>
     </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>1067475495</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>A-HASHOP</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>ビタミンヒアルロニックアンプルトナー 150mL&amp;amp;エマルジョン150mL企画(クリーム30mL贈呈)</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F572" t="n">
+        <v>4988</v>
+      </c>
+      <c r="G572" t="n">
+        <v>0</v>
+      </c>
+      <c r="H572" t="b">
+        <v>0</v>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1067475495</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>1072009140</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>バイオ スキン クレンジング パッド 6g 30枚入 x 2</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>EKE</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G573" t="n">
+        <v>0</v>
+      </c>
+      <c r="H573" t="b">
+        <v>0</v>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1072009140</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>1079690675</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>CELL LINE PRO リペアクリーム [100口] 半永久化粧材料 アフターケア 1g100個入り</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Clear_pro</t>
+        </is>
+      </c>
+      <c r="F574" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G574" t="n">
+        <v>0</v>
+      </c>
+      <c r="H574" t="b">
+        <v>0</v>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079690675</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>1142729311</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>CreatorBUBU</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>[SNP] Glutathione Dark Zero Toning Patch 60ea, Gold Collagen Perfection Eye Patch 60ea</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>SNP</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>3236</v>
+      </c>
+      <c r="G575" t="n">
+        <v>0</v>
+      </c>
+      <c r="H575" t="b">
+        <v>0</v>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142729311</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>1090206932</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>linada</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>キューティクル3-Stepケアキット(キューティクルオイル+キューティクルリムーバー+クリスタルペンプッシャー)</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>BANDI</t>
+        </is>
+      </c>
+      <c r="F576" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G576" t="n">
+        <v>0</v>
+      </c>
+      <c r="H576" t="b">
+        <v>0</v>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1090206932</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>1180616865</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>linada</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>ソウルマイティバンブーパンテノールクリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Purito</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G577" t="n">
+        <v>0</v>
+      </c>
+      <c r="H577" t="b">
+        <v>0</v>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180616865</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>1193439407</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>linada</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>1.05 アスタキサンチン0.05％ NAD1％ 30ml</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F578" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G578" t="n">
+        <v>0</v>
+      </c>
+      <c r="H578" t="b">
+        <v>0</v>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193439407</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>1091577701</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>linada</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>チェスナットAHA 8%クリアエッセンス 100ml</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>イズエンツリー</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G579" t="n">
+        <v>0</v>
+      </c>
+      <c r="H579" t="b">
+        <v>0</v>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1091577701</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>1209384322</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>linada</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>アルファクレンジングフォーム 200ml</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>HISTOLAB</t>
+        </is>
+      </c>
+      <c r="F580" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G580" t="n">
+        <v>0</v>
+      </c>
+      <c r="H580" t="b">
+        <v>0</v>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209384322</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>1188963997</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Qoo10JapanDaae</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>タイムレボリューション ザ ファースト エッセンス パッド 250ml 75枚入 1個</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>3011</v>
+      </c>
+      <c r="G581" t="n">
+        <v>0</v>
+      </c>
+      <c r="H581" t="b">
+        <v>0</v>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188963997</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>1175139603</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Qoo10JapanDaae</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>モイスチャー バランシング 無シリコン シャンプー 530ml 1個</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>アドル</t>
+        </is>
+      </c>
+      <c r="F582" t="n">
+        <v>3743</v>
+      </c>
+      <c r="G582" t="n">
+        <v>0</v>
+      </c>
+      <c r="H582" t="b">
+        <v>0</v>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175139603</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>1139814745</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>ティルティールオフザサンエアムース/ 40ml/ 1個</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F583" t="n">
+        <v>2247</v>
+      </c>
+      <c r="G583" t="n">
+        <v>0</v>
+      </c>
+      <c r="H583" t="b">
+        <v>0</v>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139814745</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>1151569871</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>デイリー アンチヘアロス タンパク質 トリートメント 500ml</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F584" t="n">
+        <v>3048</v>
+      </c>
+      <c r="G584" t="n">
+        <v>0</v>
+      </c>
+      <c r="H584" t="b">
+        <v>0</v>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151569871</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J571"/>
+  <autoFilter ref="A1:J584"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 75, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$584</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$600</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J584"/>
+  <dimension ref="A1:J600"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24399,8 +24399,664 @@
         </is>
       </c>
     </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>1097995675</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>kor_shop</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>ルビーセル最新本物の保護マイルドラインミルク50ml強力で純粋なデイリーラインミルク50+</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Ruby-Cell</t>
+        </is>
+      </c>
+      <c r="F585" t="n">
+        <v>5826</v>
+      </c>
+      <c r="G585" t="n">
+        <v>0</v>
+      </c>
+      <c r="H585" t="b">
+        <v>0</v>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097995675</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>1141190063</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>korchannel</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>[1+1]トゥクールフォースクールアートクラスアーティストモチパフ</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>トゥークールフォースクール</t>
+        </is>
+      </c>
+      <c r="F586" t="n">
+        <v>2430</v>
+      </c>
+      <c r="G586" t="n">
+        <v>1</v>
+      </c>
+      <c r="H586" t="b">
+        <v>0</v>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141190063</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>1141209058</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>korchannel</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>ユーソプルニチ香水ベリーノワール50ml 30代男性香水</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>YOUSSOFUL</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>11610</v>
+      </c>
+      <c r="G587" t="n">
+        <v>1</v>
+      </c>
+      <c r="H587" t="b">
+        <v>0</v>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141209058</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>1210683594</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>82lounge</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>メディAHAクリーム 25ml :: AHAクリーム / クリーム 角質除去 / クリーム スポットケア / クリーム ニキビ</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F588" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G588" t="n">
+        <v>0</v>
+      </c>
+      <c r="H588" t="b">
+        <v>0</v>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210683594</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>1158685803</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>hahahaya</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>グリコリック アシッド 7% エクスポリエイティングトナー 100ml</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>1860</v>
+      </c>
+      <c r="G589" t="n">
+        <v>1</v>
+      </c>
+      <c r="H589" t="b">
+        <v>0</v>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158685803</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>1211859799</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>ゼロキャスト デイリー 透明 保湿サンスクリーン 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F590" t="n">
+        <v>3211</v>
+      </c>
+      <c r="G590" t="n">
+        <v>0</v>
+      </c>
+      <c r="H590" t="b">
+        <v>0</v>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211859799</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>1211855765</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>ビタC フォーストリックス トーニング セラムマスク 22ml 10枚</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F591" t="n">
+        <v>3173</v>
+      </c>
+      <c r="G591" t="n">
+        <v>0</v>
+      </c>
+      <c r="H591" t="b">
+        <v>0</v>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211855765</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>1209466651</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>ラクトリメディ レディース カミングクリーム 15ml</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>メディオン</t>
+        </is>
+      </c>
+      <c r="F592" t="n">
+        <v>5161</v>
+      </c>
+      <c r="G592" t="n">
+        <v>1</v>
+      </c>
+      <c r="H592" t="b">
+        <v>0</v>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209466651</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>1209446667</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>【クーリング/Yーンケア】ポエリエ フェミニン インナーパフューム デイリー マルチ香水</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>フォエリー</t>
+        </is>
+      </c>
+      <c r="F593" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G593" t="n">
+        <v>1</v>
+      </c>
+      <c r="H593" t="b">
+        <v>0</v>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209446667</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>1172106877</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>ジークップ ケアセラ エコアスノウ 硫黄石鹸 (4個入)</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>ケアセラ</t>
+        </is>
+      </c>
+      <c r="F594" t="n">
+        <v>3710</v>
+      </c>
+      <c r="G594" t="n">
+        <v>0</v>
+      </c>
+      <c r="H594" t="b">
+        <v>0</v>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172106877</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>1169173710</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>ニューヨーク インティリー オードパルファムEDP 10ml</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>7780</v>
+      </c>
+      <c r="G595" t="n">
+        <v>0</v>
+      </c>
+      <c r="H595" t="b">
+        <v>0</v>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169173710</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>1169173462</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>ローストウッド オードパルファムEDP 10ml</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F596" t="n">
+        <v>7780</v>
+      </c>
+      <c r="G596" t="n">
+        <v>0</v>
+      </c>
+      <c r="H596" t="b">
+        <v>0</v>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169173462</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>1181384570</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>[ギャラリア] MADET LEN レッドムスク オードパルファム RED MUSC</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>MAD et LEN</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>63970</v>
+      </c>
+      <c r="G597" t="n">
+        <v>0</v>
+      </c>
+      <c r="H597" t="b">
+        <v>0</v>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181384570</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>1082804410</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>SuperStarK</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>【国内発送】 ターンオーバーアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F598" t="n">
+        <v>5478</v>
+      </c>
+      <c r="G598" t="n">
+        <v>1</v>
+      </c>
+      <c r="H598" t="b">
+        <v>0</v>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1082804410</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>1200649177</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>cosmenana</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>ululis ウルリス プレミアム ウォーターコンク ブラックセラム ヘアオイル 100ml 黒[3559] 宅配無料</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F599" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G599" t="n">
+        <v>0</v>
+      </c>
+      <c r="H599" t="b">
+        <v>0</v>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200649177</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>1198894604</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>bestone1</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>ティファニー TIFFANY ＆ラブ フォーヒム EDT + ＆ラブ フォーハー EDP ミニ香水 セット 1.2ml×2 サンプル[6495] メール便無料[B][BP3]</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Tiffany</t>
+        </is>
+      </c>
+      <c r="F600" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G600" t="n">
+        <v>1</v>
+      </c>
+      <c r="H600" t="b">
+        <v>0</v>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198894604</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J584"/>
+  <autoFilter ref="A1:J600"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 78, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$600</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J600"/>
+  <dimension ref="A1:J616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25055,8 +25055,664 @@
         </is>
       </c>
     </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>1091387881</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>バイビード インアンドアウト マスクパック,1個入り,5個,/In &amp;amp; Out Facial Mask/毛穴の老廃物を除去</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>バイビッド</t>
+        </is>
+      </c>
+      <c r="F601" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G601" t="n">
+        <v>5</v>
+      </c>
+      <c r="H601" t="b">
+        <v>0</v>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1091387881</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>1095687901</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>[KERASYS] ADVANCED KERAMIDE トリートメント！ ヘアパック！ シャンプー！ 人気商品集電線 1+1 [正規品] 韓国ブランド(鎮静/弾力/保湿/栄養供給/活力)</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F602" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G602" t="n">
+        <v>0</v>
+      </c>
+      <c r="H602" t="b">
+        <v>0</v>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1095687901</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>1101562835</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>ビフィダ バイオーム アンプル パッド 70枚</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F603" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G603" t="n">
+        <v>1</v>
+      </c>
+      <c r="H603" t="b">
+        <v>0</v>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1101562835</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>1094393233</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>THEビタAレチナールショットタイトニングブースター 15ml</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F604" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G604" t="n">
+        <v>4</v>
+      </c>
+      <c r="H604" t="b">
+        <v>0</v>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094393233</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>1103977398</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>ノスカナゲル /アクノンクリーム /アクリンゲル /メラトーニンクリーム /メラノサ ヒドロキノン /Dパンテノール軟膏</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>6256</v>
+      </c>
+      <c r="G605" t="n">
+        <v>0</v>
+      </c>
+      <c r="H605" t="b">
+        <v>0</v>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1103977398</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>1093319609</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>THE ビタA レチノールセラム 30ml + レチナールブースター 15ml セット</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F606" t="n">
+        <v>4250</v>
+      </c>
+      <c r="G606" t="n">
+        <v>3</v>
+      </c>
+      <c r="H606" t="b">
+        <v>0</v>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093319609</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>1119598747</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>ノニアクネバブルクレンザー 155ml</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G607" t="n">
+        <v>1</v>
+      </c>
+      <c r="H607" t="b">
+        <v>0</v>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119598747</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>1167121017</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>リンゼイ 鎮静薬草モデリングパック (カップパック) 28g [66冠/1位]</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>LINDSAY</t>
+        </is>
+      </c>
+      <c r="F608" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G608" t="n">
+        <v>1</v>
+      </c>
+      <c r="H608" t="b">
+        <v>0</v>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167121017</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>1204303349</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>ラエル オーガニックコットンカバー 履くオーバーナイト M 2個入 x3個</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>ラエル</t>
+        </is>
+      </c>
+      <c r="F609" t="n">
+        <v>3059</v>
+      </c>
+      <c r="G609" t="n">
+        <v>0</v>
+      </c>
+      <c r="H609" t="b">
+        <v>0</v>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204303349</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>1202040262</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>ジョソンアビューティ ワンダーバス レモンシロップ パッククレンザー 200ml (+50ml)</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>WONDER BATH</t>
+        </is>
+      </c>
+      <c r="F610" t="n">
+        <v>4332</v>
+      </c>
+      <c r="G610" t="n">
+        <v>0</v>
+      </c>
+      <c r="H610" t="b">
+        <v>0</v>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202040262</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>1199549438</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>sunnyline</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>クライオ ソルベ アイシー フェイシャル マスク (4個入) / クーリング 冷却 パック むくみケア</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F611" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G611" t="n">
+        <v>1</v>
+      </c>
+      <c r="H611" t="b">
+        <v>0</v>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199549438</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>1205600340</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>sunnyline</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>デカッソシド サンスティック エアリフィット 10g + 10g (1+1 セット) 日焼け止め スティック UVケア CICA 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F612" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G612" t="n">
+        <v>0</v>
+      </c>
+      <c r="H612" t="b">
+        <v>0</v>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205600340</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>1204317855</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>sunnyline</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>プロテインボンド ウォーターエッセンス＋ピカチュウ ミラーコーム セット</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>ヘアプラス</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G613" t="n">
+        <v>1</v>
+      </c>
+      <c r="H613" t="b">
+        <v>0</v>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204317855</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>1119858758</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>エピエルアボカドオイル+ヒマワリオイル抽出モイスチャーハンドパック/バルパック12パック</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>epille</t>
+        </is>
+      </c>
+      <c r="F614" t="n">
+        <v>2137</v>
+      </c>
+      <c r="G614" t="n">
+        <v>1</v>
+      </c>
+      <c r="H614" t="b">
+        <v>0</v>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119858758</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>1151670543</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>[国内百貨店]ディープディックフレッドポッドボディバーム200ml</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>ディプティック</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>16500</v>
+      </c>
+      <c r="G615" t="n">
+        <v>0</v>
+      </c>
+      <c r="H615" t="b">
+        <v>0</v>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151670543</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>1148898608</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>エバーセルセルバイタルセルチャージャーエッセンス14p252ml1個</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>エバーセル</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>8150</v>
+      </c>
+      <c r="G616" t="n">
+        <v>0</v>
+      </c>
+      <c r="H616" t="b">
+        <v>0</v>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148898608</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J600"/>
+  <autoFilter ref="A1:J616"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 81, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$625</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J616"/>
+  <dimension ref="A1:J625"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25711,8 +25711,377 @@
         </is>
       </c>
     </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>1162204761</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>[NEW] クライオアイスマスク 30枚</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F617" t="n">
+        <v>2070</v>
+      </c>
+      <c r="G617" t="n">
+        <v>4</v>
+      </c>
+      <c r="H617" t="b">
+        <v>0</v>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162204761</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>1190357115</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>アゼライン酸CICAスキンクリアトナー 250ml</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F618" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G618" t="n">
+        <v>0</v>
+      </c>
+      <c r="H618" t="b">
+        <v>0</v>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190357115</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>1157789377</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>ドクダミLHAモイスチャーピーリングジェル 120ml</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F619" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G619" t="n">
+        <v>0</v>
+      </c>
+      <c r="H619" t="b">
+        <v>0</v>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157789377</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>1148824104</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>HappyBGLD</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>【20%OFF 全ブランド跨ぎ割引】 イロン 当帰スディンゲル 500ml 大容量 水分エッセンス 肌バリア 赤み 속건조+マスクパックをプレゼント</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F620" t="n">
+        <v>7970</v>
+      </c>
+      <c r="G620" t="n">
+        <v>4</v>
+      </c>
+      <c r="H620" t="b">
+        <v>0</v>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148824104</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>1176812478</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>meisonmatcha</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>[2個]トータルリペア5 ミラクル ヘアパック 170ml</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F621" t="n">
+        <v>1626</v>
+      </c>
+      <c r="G621" t="n">
+        <v>0</v>
+      </c>
+      <c r="H621" t="b">
+        <v>0</v>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176812478</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>1197665370</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>オンリーフォーマンオールインワンエッセンス 200ml 2個 皮脂ケア テカリ防止</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F622" t="n">
+        <v>5683</v>
+      </c>
+      <c r="G622" t="n">
+        <v>0</v>
+      </c>
+      <c r="H622" t="b">
+        <v>0</v>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665370</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>1197665508</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュフォーマン鎮静オールインワン 200ml 3個 お得 ストック</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>12618</v>
+      </c>
+      <c r="G623" t="n">
+        <v>0</v>
+      </c>
+      <c r="H623" t="b">
+        <v>0</v>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665508</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>1197665474</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>メンズグッドルックスアイブローペンシル ナチュラルブラック 1個 目力 男子メイク</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>1921</v>
+      </c>
+      <c r="G624" t="n">
+        <v>0</v>
+      </c>
+      <c r="H624" t="b">
+        <v>0</v>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665474</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>1197665466</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>広報ジンクリーム 50ml 1個 栄養補給 ツヤ</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>多娜嫺</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>2396</v>
+      </c>
+      <c r="G625" t="n">
+        <v>1</v>
+      </c>
+      <c r="H625" t="b">
+        <v>0</v>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665466</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J616"/>
+  <autoFilter ref="A1:J625"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 84, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$625</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$627</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J625"/>
+  <dimension ref="A1:J627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26080,8 +26080,90 @@
         </is>
       </c>
     </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>1209471077</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>HMseller</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>【正規品】ダブルショットパフュームボディミスト 120ml</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>ヘトラス</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G626" t="n">
+        <v>2</v>
+      </c>
+      <c r="H626" t="b">
+        <v>0</v>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209471077</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>1047570493</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>SJOCEAN</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>[1+1] リアル ヒアルロニック 100 クリーム 80ml+80ml / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>WELLAGE</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>5040</v>
+      </c>
+      <c r="G627" t="n">
+        <v>0</v>
+      </c>
+      <c r="H627" t="b">
+        <v>0</v>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1047570493</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J625"/>
+  <autoFilter ref="A1:J627"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 87, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$627</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$647</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J627"/>
+  <dimension ref="A1:J647"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26162,8 +26162,828 @@
         </is>
       </c>
     </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>1115552034</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>[1+1] [SNS, AMAZON 大人気] 米サンクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>3558</v>
+      </c>
+      <c r="G628" t="n">
+        <v>0</v>
+      </c>
+      <c r="H628" t="b">
+        <v>0</v>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115552034</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>1193643194</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>【正規品】【Qoo10人気】レチノールリペアセラム30ml ヴィーガンリポソームレチノール3%セラム</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>スキンアンドラブ</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>4736</v>
+      </c>
+      <c r="G629" t="n">
+        <v>0</v>
+      </c>
+      <c r="H629" t="b">
+        <v>0</v>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193643194</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>1193643034</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>【正規品】コラーゲンナイトラッピングマスク 75ml + ブラシ</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>メディキューブバイオ</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G630" t="n">
+        <v>0</v>
+      </c>
+      <c r="H630" t="b">
+        <v>0</v>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193643034</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>1193642954</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>【正規品】[ライスシリーズ] 7 ライス セラミド グローセラム /ライス 70 インテンス モイスチャー ミルク /ライス ブライトニング酵素洗顔パウダー /ライス70 グロウミルキートナー</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>4516</v>
+      </c>
+      <c r="G631" t="n">
+        <v>0</v>
+      </c>
+      <c r="H631" t="b">
+        <v>0</v>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193642954</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>1193642948</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>GIVENCY 【正規品】 プリズム リーブル ミニパウダー No0/No1/No2/No3/No4 ジバンシイ プリズム リーブル PRISME LIBRE ルース パウダー</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>7570</v>
+      </c>
+      <c r="G632" t="n">
+        <v>0</v>
+      </c>
+      <c r="H632" t="b">
+        <v>0</v>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193642948</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>1197470722</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>mangobeautylab</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>ネイチャー シャンプー 詰め替え 4個セット ベビーパウダー 香り 400ml リフィル 大容量 まとめ買い 自然由来 家族用</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F633" t="n">
+        <v>5594</v>
+      </c>
+      <c r="G633" t="n">
+        <v>1</v>
+      </c>
+      <c r="H633" t="b">
+        <v>0</v>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197470722</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>1121575025</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>unicornmall</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>バイオコラーゲンリアルディープマスク, 8枚/バイオコラーゲンリアルディープマスク(8枚入り)/高保湿/弾力毛穴ツヤ肌ケア/アンプル１個分をそのまま固めたハイドロゲル/べたつきかない/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F634" t="n">
+        <v>6655</v>
+      </c>
+      <c r="G634" t="n">
+        <v>3</v>
+      </c>
+      <c r="H634" t="b">
+        <v>0</v>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1121575025</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>1200851127</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸カプセル100セラム30ml +モイスチャライジングクリーム30ml+ PDRN 100 ヒアルロン酸 ブースター トナー 250ml + 40ml</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>6880</v>
+      </c>
+      <c r="G635" t="n">
+        <v>4</v>
+      </c>
+      <c r="H635" t="b">
+        <v>0</v>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200851127</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>1200850420</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸 水分カプセルミスト 100ml + 100ml / 保湿ミスト 韓国ブランド ミスト</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G636" t="n">
+        <v>5</v>
+      </c>
+      <c r="H636" t="b">
+        <v>0</v>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200850420</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>1205030887</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>シラカバ保湿サンスティック + シラカバ水分サンクリーム [韓国サンスティック]</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>7380</v>
+      </c>
+      <c r="G637" t="n">
+        <v>2</v>
+      </c>
+      <c r="H637" t="b">
+        <v>0</v>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205030887</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>1201003595</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸カプセル100 セラム 30ml + PDRN ヒアルロン酸 水分カプセルミスト 100ml</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>6980</v>
+      </c>
+      <c r="G638" t="n">
+        <v>2</v>
+      </c>
+      <c r="H638" t="b">
+        <v>0</v>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201003595</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>1170454907</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>onha</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>No.9 NMN BIO リフティング シートマスク（4枚）</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>3088</v>
+      </c>
+      <c r="G639" t="n">
+        <v>0</v>
+      </c>
+      <c r="H639" t="b">
+        <v>0</v>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170454907</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>1171970507</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>onha</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>【大容量】PDRN 100＋ヒアルロン酸 ブースタートナー 250ml＋40ml保湿化粧水 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F640" t="n">
+        <v>3483</v>
+      </c>
+      <c r="G640" t="n">
+        <v>0</v>
+      </c>
+      <c r="H640" t="b">
+        <v>0</v>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171970507</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>1152724729</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>ドクダミ77%スージングトナー, 250ml</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F641" t="n">
+        <v>1760</v>
+      </c>
+      <c r="G641" t="n">
+        <v>0</v>
+      </c>
+      <c r="H641" t="b">
+        <v>0</v>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152724729</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>1191147953</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>ピュア ボディミスト ベビーパウダーの香り 128ml 2個</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F642" t="n">
+        <v>1867</v>
+      </c>
+      <c r="G642" t="n">
+        <v>1</v>
+      </c>
+      <c r="H642" t="b">
+        <v>0</v>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191147953</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>1185851789</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>[1+1] レッド ラクト コラーゲン ラッピング マスクパック 70ml *2 + ブラシ</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F643" t="n">
+        <v>3587</v>
+      </c>
+      <c r="G643" t="n">
+        <v>1</v>
+      </c>
+      <c r="H643" t="b">
+        <v>0</v>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185851789</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>1157601678</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>[SET] プロテインダメージケアシャンプー500ml+トリートメント250ml</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F644" t="n">
+        <v>3630</v>
+      </c>
+      <c r="G644" t="n">
+        <v>4</v>
+      </c>
+      <c r="H644" t="b">
+        <v>0</v>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157601678</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>1152724831</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>6番 爆睡マスクパックセラム50ml</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F645" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G645" t="n">
+        <v>0</v>
+      </c>
+      <c r="H645" t="b">
+        <v>0</v>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152724831</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>1208195309</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>klumin</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>パフュームシルキーハンドクリーム50ml フレグランス12種, ご購入でMEDIHEAL ローズPDRNマスク1枚プレゼント</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>ヘトラス</t>
+        </is>
+      </c>
+      <c r="F646" t="n">
+        <v>1940</v>
+      </c>
+      <c r="G646" t="n">
+        <v>0</v>
+      </c>
+      <c r="H646" t="b">
+        <v>0</v>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208195309</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>1209668463</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>klumin</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>[MEDIHEAL マスク1枚付き]ドクダミ77スージングトナー，350ml</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F647" t="n">
+        <v>2926</v>
+      </c>
+      <c r="G647" t="n">
+        <v>0</v>
+      </c>
+      <c r="H647" t="b">
+        <v>0</v>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209668463</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J627"/>
+  <autoFilter ref="A1:J647"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 90, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$647</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$654</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J647"/>
+  <dimension ref="A1:J654"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26982,8 +26982,295 @@
         </is>
       </c>
     </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>1205779441</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>albami</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>エストラ アトバリア365 ハイドロ スージングクリーム 80ml セット(トナー25ml+クレンジングフォーム30g)</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>ハイドロ</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>4450</v>
+      </c>
+      <c r="G648" t="n">
+        <v>0</v>
+      </c>
+      <c r="H648" t="b">
+        <v>0</v>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205779441</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>1195242230</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>イリユン セラミドアトローション 無香料 508ml 1個</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>2655</v>
+      </c>
+      <c r="G649" t="n">
+        <v>0</v>
+      </c>
+      <c r="H649" t="b">
+        <v>0</v>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195242230</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>1208323570</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>SKIN1004 マダガスカルセンテラ ヒアルーシカ ウォーターフィットサンセラム 日焼け止め SPF50+ PA++++ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>ティーゼン</t>
+        </is>
+      </c>
+      <c r="F650" t="n">
+        <v>3076</v>
+      </c>
+      <c r="G650" t="n">
+        <v>0</v>
+      </c>
+      <c r="H650" t="b">
+        <v>0</v>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208323570</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>1123888012</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>リードルショット1000 エッセンス 15ml</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F651" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G651" t="n">
+        <v>1</v>
+      </c>
+      <c r="H651" t="b">
+        <v>0</v>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123888012</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>1123548274</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド 10 TXA 4 ダークスポット コレクティング セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F652" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G652" t="n">
+        <v>0</v>
+      </c>
+      <c r="H652" t="b">
+        <v>0</v>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123548274</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>1206710414</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>超高含有ヒアルロニックインテンストナー 100時間保湿持続力300g</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F653" t="n">
+        <v>3148</v>
+      </c>
+      <c r="G653" t="n">
+        <v>0</v>
+      </c>
+      <c r="H653" t="b">
+        <v>0</v>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206710414</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>1209385392</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>アドール パフューム ヘアオイル 80ml 5種類から選べる</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>アドル</t>
+        </is>
+      </c>
+      <c r="F654" t="n">
+        <v>3456</v>
+      </c>
+      <c r="G654" t="n">
+        <v>1</v>
+      </c>
+      <c r="H654" t="b">
+        <v>0</v>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209385392</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J647"/>
+  <autoFilter ref="A1:J654"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 93, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$654</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$663</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J654"/>
+  <dimension ref="A1:J663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27269,8 +27269,377 @@
         </is>
       </c>
     </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>1168069878</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>morningmood</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>白樺 水分トナー 300ml</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F655" t="n">
+        <v>2345</v>
+      </c>
+      <c r="G655" t="n">
+        <v>1</v>
+      </c>
+      <c r="H655" t="b">
+        <v>0</v>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168069878</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>1210851756</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>kglowshop</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>「当日発送」 リアルカロテンIPMPブレミッシュセラムパックパッド, 80枚</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F656" t="n">
+        <v>2460</v>
+      </c>
+      <c r="G656" t="n">
+        <v>1</v>
+      </c>
+      <c r="H656" t="b">
+        <v>0</v>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210851756</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>1210850141</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>smuse</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>リアルカロテンIPMPブレミッシュセラムパックパッド, 80枚</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F657" t="n">
+        <v>2260</v>
+      </c>
+      <c r="G657" t="n">
+        <v>0</v>
+      </c>
+      <c r="H657" t="b">
+        <v>0</v>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210850141</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>1195129454</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>K_AUTHENTIC</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>[韓國正品店]NEW Love portion オードパルファム 香水 9種/韓国人氣</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F658" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G658" t="n">
+        <v>0</v>
+      </c>
+      <c r="H658" t="b">
+        <v>0</v>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195129454</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>1194218772</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>glowkorea</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>ハイドロセラミック水分エッセンス日焼け止めクリーム50ml2個</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F659" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G659" t="n">
+        <v>0</v>
+      </c>
+      <c r="H659" t="b">
+        <v>0</v>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194218772</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>1193987745</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>kstar_pick</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>ミジャンセンサロン10 プロテイントリートメント ダメージヘア用250ml3個</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F660" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G660" t="n">
+        <v>0</v>
+      </c>
+      <c r="H660" t="b">
+        <v>0</v>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193987745</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>1203335944</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>ボディローション ホワイトマスク520ml /韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>ブーケガルニ</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G661" t="n">
+        <v>0</v>
+      </c>
+      <c r="H661" t="b">
+        <v>0</v>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203335944</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>1196699361</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>蓮花PDRNヒアルロン光彩セラム 30ml 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>ハンスキン</t>
+        </is>
+      </c>
+      <c r="F662" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G662" t="n">
+        <v>0</v>
+      </c>
+      <c r="H662" t="b">
+        <v>0</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196699361</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>1193167209</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>パンテノール クリーム 100ml 韓国スキンケア 韓国 コスメ #水分#保湿 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F663" t="n">
+        <v>4504</v>
+      </c>
+      <c r="G663" t="n">
+        <v>1</v>
+      </c>
+      <c r="H663" t="b">
+        <v>0</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193167209</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J654"/>
+  <autoFilter ref="A1:J663"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 96, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$663</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$674</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J663"/>
+  <dimension ref="A1:J674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27638,8 +27638,459 @@
         </is>
       </c>
     </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>1209812267</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>thebest_mall</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>SOSセラム, 50ml</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>3524</v>
+      </c>
+      <c r="G664" t="n">
+        <v>0</v>
+      </c>
+      <c r="H664" t="b">
+        <v>0</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209812267</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>1210345860</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>luxstargaram</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>ハートブラシ コンパクト ヘアブラシ</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>リファ</t>
+        </is>
+      </c>
+      <c r="F665" t="n">
+        <v>3579</v>
+      </c>
+      <c r="G665" t="n">
+        <v>0</v>
+      </c>
+      <c r="H665" t="b">
+        <v>0</v>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210345860</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>1196942000</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>luxstargaram</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>デーマトロジー ファーストパッケージ【ブースター130ml＋セラム45ml】</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F666" t="n">
+        <v>13449</v>
+      </c>
+      <c r="G666" t="n">
+        <v>3</v>
+      </c>
+      <c r="H666" t="b">
+        <v>0</v>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196942000</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>1183523136</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>luxstargaram</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>韓国スキンケア 洗顔パウダー 酵素洗顔 毛穴ケア フェイスウォッシュ クレンジングパウダー 80g</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F667" t="n">
+        <v>5177</v>
+      </c>
+      <c r="G667" t="n">
+        <v>1</v>
+      </c>
+      <c r="H667" t="b">
+        <v>0</v>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183523136</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>1191781202</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>MEDIHEAL トナーパッド2.0 リフィル 70枚×2個セット 4タイプ選択可</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F668" t="n">
+        <v>1918</v>
+      </c>
+      <c r="G668" t="n">
+        <v>0</v>
+      </c>
+      <c r="H668" t="b">
+        <v>0</v>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191781202</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>1204359324</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>【1+1 / SNS話題】ツヤ肌バブルエッセンストナー 95ml</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>curest</t>
+        </is>
+      </c>
+      <c r="F669" t="n">
+        <v>2131</v>
+      </c>
+      <c r="G669" t="n">
+        <v>0</v>
+      </c>
+      <c r="H669" t="b">
+        <v>0</v>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204359324</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>1180354766</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>[1+1/限定企画] スキンフード キャロット カロチン カミング ウォーターパッド 60枚 ダブル企画</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F670" t="n">
+        <v>6791</v>
+      </c>
+      <c r="G670" t="n">
+        <v>0</v>
+      </c>
+      <c r="H670" t="b">
+        <v>0</v>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180354766</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>1207273381</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>PDRN ピンク コラーゲン バーム セラム 95ml 炭酸 泡 美容液 水光肌 弾力 ほうれい線 乾燥肌 エイジングケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F671" t="n">
+        <v>5049</v>
+      </c>
+      <c r="G671" t="n">
+        <v>0</v>
+      </c>
+      <c r="H671" t="b">
+        <v>0</v>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207273381</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>1171947071</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>【正規品】 デイリートナーパッド 80枚</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>NEEDLY</t>
+        </is>
+      </c>
+      <c r="F672" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G672" t="n">
+        <v>0</v>
+      </c>
+      <c r="H672" t="b">
+        <v>0</v>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171947071</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>1171946936</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>【正規品】 センテラクイックカーミングパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F673" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G673" t="n">
+        <v>3</v>
+      </c>
+      <c r="H673" t="b">
+        <v>0</v>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171946936</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>1197892266</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>【正規品】 グロウクリーミーボディスクラブ ヌバニラ 300ml</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G674" t="n">
+        <v>0</v>
+      </c>
+      <c r="H674" t="b">
+        <v>0</v>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197892266</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J663"/>
+  <autoFilter ref="A1:J674"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 99, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$674</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$688</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J674"/>
+  <dimension ref="A1:J688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28089,8 +28089,582 @@
         </is>
       </c>
     </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>1093761271</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>インテンシブロングラスティングサンスクリーンEX 60ml /SPF50+PA++++</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>1575</v>
+      </c>
+      <c r="G675" t="n">
+        <v>0</v>
+      </c>
+      <c r="H675" t="b">
+        <v>0</v>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093761271</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>1177950809</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>ブドウ糖ハイドロエッセンストナー, 500ml</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>パティオン</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>3105</v>
+      </c>
+      <c r="G676" t="n">
+        <v>0</v>
+      </c>
+      <c r="H676" t="b">
+        <v>0</v>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177950809</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>1172804214</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>海ぶどう レチノール 毛穴弾力クリーム 50g</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Mommy Care</t>
+        </is>
+      </c>
+      <c r="F677" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G677" t="n">
+        <v>1</v>
+      </c>
+      <c r="H677" t="b">
+        <v>0</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172804214</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>1162838579</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>tmashop</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>[単独企画]清楚ビタCジョブティケアパッド70枚（10枚贈呈）</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F678" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G678" t="n">
+        <v>0</v>
+      </c>
+      <c r="H678" t="b">
+        <v>0</v>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162838579</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>1213378280</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>ザ・ビタA レチナールショット タイトニングブースター 15ml/더 비타 A 레티날 샷 타이트닝 부스터 15ml</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F679" t="n">
+        <v>2386</v>
+      </c>
+      <c r="G679" t="n">
+        <v>0</v>
+      </c>
+      <c r="H679" t="b">
+        <v>0</v>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213378280</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>1167189215</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>ドクダミヒアルロンスージング アンプル 50ml/ 어성초 히알루론 수딩 앰플 50ml</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F680" t="n">
+        <v>2212</v>
+      </c>
+      <c r="G680" t="n">
+        <v>0</v>
+      </c>
+      <c r="H680" t="b">
+        <v>0</v>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167189215</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>1083286884</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>[ エンジェルスリキッド ] グルタチオンプラス ナイアシンアミド 700vクリーム 50ml/나이아신아마이드 700v 크림</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Angel's Liquid</t>
+        </is>
+      </c>
+      <c r="F681" t="n">
+        <v>3085</v>
+      </c>
+      <c r="G681" t="n">
+        <v>3</v>
+      </c>
+      <c r="H681" t="b">
+        <v>0</v>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083286884</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>1180574367</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>fromAnswer</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>[10Sマイクロバブルパック 4種] エア** バブルCDS マスク パック 80ml, 4種の中から選択 (ハリ/ブライトニング/鎮静/水分) 150 回分</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Gear By Gash</t>
+        </is>
+      </c>
+      <c r="F682" t="n">
+        <v>4014</v>
+      </c>
+      <c r="G682" t="n">
+        <v>0</v>
+      </c>
+      <c r="H682" t="b">
+        <v>0</v>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180574367</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>1212561469</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>kselects</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>ディープクリーン クーリングシャンプー 500ml 2本</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F683" t="n">
+        <v>5240</v>
+      </c>
+      <c r="G683" t="n">
+        <v>0</v>
+      </c>
+      <c r="H683" t="b">
+        <v>0</v>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212561469</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>1209152772</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>kselects</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>ミステリーチョコマシュマロ 40g 6個セット 韓国お菓子 チョコマシュマロ 個包装</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Pongsindang</t>
+        </is>
+      </c>
+      <c r="F684" t="n">
+        <v>6500</v>
+      </c>
+      <c r="G684" t="n">
+        <v>0</v>
+      </c>
+      <c r="H684" t="b">
+        <v>0</v>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209152772</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>1142237251</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>BTSジョングクPerfume 50ml / フォルメント コットンハグ BTS ジョングク</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F685" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G685" t="n">
+        <v>1</v>
+      </c>
+      <c r="H685" t="b">
+        <v>0</v>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142237251</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>1159827458</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>クリーンイットゼロ ピンク 水分 トナー パッド</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F686" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G686" t="n">
+        <v>0</v>
+      </c>
+      <c r="H686" t="b">
+        <v>0</v>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159827458</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>1089140326</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>セラミド アト集中クリーム 無香, 500ml 1個</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F687" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G687" t="n">
+        <v>4</v>
+      </c>
+      <c r="H687" t="b">
+        <v>0</v>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089140326</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>1080079065</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>デイリー マスクパック 30枚</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F688" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G688" t="n">
+        <v>1</v>
+      </c>
+      <c r="H688" t="b">
+        <v>0</v>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080079065</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J674"/>
+  <autoFilter ref="A1:J688"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 102, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$688</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$692</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J688"/>
+  <dimension ref="A1:J692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28663,8 +28663,172 @@
         </is>
       </c>
     </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>1200859567</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>ALLROUNDERBEAUTY</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>ティーツリーシカ ディープクレンジングオイル 200ml</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F689" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G689" t="n">
+        <v>0</v>
+      </c>
+      <c r="H689" t="b">
+        <v>0</v>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200859567</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>1213547055</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>トリプルシールド ハイドロロック サンセラム SPF50+ PA++++ 50ml</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Forencos</t>
+        </is>
+      </c>
+      <c r="F690" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G690" t="n">
+        <v>0</v>
+      </c>
+      <c r="H690" t="b">
+        <v>0</v>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213547055</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>1212836013</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>スキン パーフェクティング BHA リキッド エクスフォリエント 118ml + 30ml / 角質ケア 毛穴ケア ピーリング 低刺激 スキンケア</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>ポーラチョイス</t>
+        </is>
+      </c>
+      <c r="F691" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G691" t="n">
+        <v>0</v>
+      </c>
+      <c r="H691" t="b">
+        <v>0</v>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212836013</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>1211205774</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>マルチペプチドトナー 50ml x 5個 / 肌保湿 / 保湿充填</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>ルネセル</t>
+        </is>
+      </c>
+      <c r="F692" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G692" t="n">
+        <v>0</v>
+      </c>
+      <c r="H692" t="b">
+        <v>0</v>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211205774</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J688"/>
+  <autoFilter ref="A1:J692"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 105, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$692</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$701</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J692"/>
+  <dimension ref="A1:J701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28827,8 +28827,377 @@
         </is>
       </c>
     </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>1169812368</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>coneco</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>[NEW]ラウンドアラウンド センテッド ヘア&amp;amp;ボディ ミスト 100ml</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>ROUND A ROUND</t>
+        </is>
+      </c>
+      <c r="F693" t="n">
+        <v>1618</v>
+      </c>
+      <c r="G693" t="n">
+        <v>0</v>
+      </c>
+      <c r="H693" t="b">
+        <v>0</v>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169812368</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>1155304298</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>coneco</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>ZARA 香水 HIBISCUS 90ML オードパフューム [EDP]</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>ザラ</t>
+        </is>
+      </c>
+      <c r="F694" t="n">
+        <v>4669</v>
+      </c>
+      <c r="G694" t="n">
+        <v>0</v>
+      </c>
+      <c r="H694" t="b">
+        <v>0</v>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155304298</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>1178796694</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>[最新リニューアル] セルメディックス エムジーエフ リターンクリーム 70ml</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F695" t="n">
+        <v>8860</v>
+      </c>
+      <c r="G695" t="n">
+        <v>1</v>
+      </c>
+      <c r="H695" t="b">
+        <v>0</v>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178796694</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>1180095461</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>イーロン アンプル 50ml センシエンド</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F696" t="n">
+        <v>15970</v>
+      </c>
+      <c r="G696" t="n">
+        <v>0</v>
+      </c>
+      <c r="H696" t="b">
+        <v>0</v>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095461</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>1180095290</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>イーロン ダンギ クレンジングジェル 200ml + 贈呈:マスクパック1枚</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F697" t="n">
+        <v>6550</v>
+      </c>
+      <c r="G697" t="n">
+        <v>0</v>
+      </c>
+      <c r="H697" t="b">
+        <v>0</v>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095290</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>1180095287</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>ザ·イーロン イーロン メゾプロ プラスキット 1箱 2gx2個入 + スージング マスクパック 2枚</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F698" t="n">
+        <v>11880</v>
+      </c>
+      <c r="G698" t="n">
+        <v>0</v>
+      </c>
+      <c r="H698" t="b">
+        <v>0</v>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095287</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>1180092834</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>サンテ 日焼け止め アズレン スーダー サンエッセンス 75ml 2個 デュオセット</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>SANTE</t>
+        </is>
+      </c>
+      <c r="F699" t="n">
+        <v>15970</v>
+      </c>
+      <c r="G699" t="n">
+        <v>1</v>
+      </c>
+      <c r="H699" t="b">
+        <v>0</v>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180092834</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>1178760167</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>toseo</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>オードパルファムスノーサイ 30ML Snow Sai</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>LIBER</t>
+        </is>
+      </c>
+      <c r="F700" t="n">
+        <v>7430</v>
+      </c>
+      <c r="G700" t="n">
+        <v>0</v>
+      </c>
+      <c r="H700" t="b">
+        <v>0</v>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J700" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178760167</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>1168152797</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>beautyofkorea</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>米麹酵素サウナ コマジュフォーム 170ml 1個</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F701" t="n">
+        <v>1862</v>
+      </c>
+      <c r="G701" t="n">
+        <v>0</v>
+      </c>
+      <c r="H701" t="b">
+        <v>0</v>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J701" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168152797</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J692"/>
+  <autoFilter ref="A1:J701"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 108, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$701</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$711</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J701"/>
+  <dimension ref="A1:J711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29196,8 +29196,418 @@
         </is>
       </c>
     </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>1125939784</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>【正規品】グローアップインシャワートーンアップミルク300g</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>MEDIPICKME</t>
+        </is>
+      </c>
+      <c r="F702" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G702" t="n">
+        <v>2</v>
+      </c>
+      <c r="H702" t="b">
+        <v>0</v>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J702" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125939784</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>1111189488</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>[単品] JunJun共同開発_クレンジングバーム2種 100ml (毛穴/トーンアップ)</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F703" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G703" t="n">
+        <v>0</v>
+      </c>
+      <c r="H703" t="b">
+        <v>0</v>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J703" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1111189488</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>1205453339</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>ネックパッチプレステージ（5枚入り）首　シワ　弾力 ネックケア　アイロン　ハリケア 首のシワ 保湿 たるみ デコルテケア</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>VELLA</t>
+        </is>
+      </c>
+      <c r="F704" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G704" t="n">
+        <v>0</v>
+      </c>
+      <c r="H704" t="b">
+        <v>0</v>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J704" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205453339</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>1168778005</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>BnD_official</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>コンプリートセット 5点セット ビーエヌディ アンダーアームクリーム100ｇ+ＡＨＡスクラブ200ｇ＋ネッククリーム50ｇ+ヒップクリーム100ｇ+ブルーミングヘアオイル</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>BnD</t>
+        </is>
+      </c>
+      <c r="F705" t="n">
+        <v>15437</v>
+      </c>
+      <c r="G705" t="n">
+        <v>3</v>
+      </c>
+      <c r="H705" t="b">
+        <v>0</v>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J705" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168778005</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>1211601601</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>【アヌ ア美容液】アゼライン酸10％マイルドスージングセラム 30ml(混合肌 敏感肌向け 韓国スキンケア)</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F706" t="n">
+        <v>3180</v>
+      </c>
+      <c r="G706" t="n">
+        <v>0</v>
+      </c>
+      <c r="H706" t="b">
+        <v>0</v>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J706" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211601601</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>1209266440</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>【PDRN配合/リピートアイテム】ペプタシカ セラムパッド ダブルセット（60枚＋60枚）</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>トーン28</t>
+        </is>
+      </c>
+      <c r="F707" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G707" t="n">
+        <v>0</v>
+      </c>
+      <c r="H707" t="b">
+        <v>0</v>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J707" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209266440</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>1212027043</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>【重ね塗りしやすい首ケアスティック】プレミアムネックスティック, 20g　首のシワ改善クリーム／べたつかないネックケアライン／首元のハリケア／首のしわ ／首クリーム／首トーンアップ／首用クリーム／</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F708" t="n">
+        <v>3674</v>
+      </c>
+      <c r="G708" t="n">
+        <v>0</v>
+      </c>
+      <c r="H708" t="b">
+        <v>0</v>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J708" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212027043</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>1203787114</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>【保湿クリーム】 クリームスカムトゥルー スクワランバリアリペアクリーム 50ml ツヤ肌 乾燥肌 水光肌 水分 乾燥 高保湿 うるおい もちもち ベタつかない 水分チャージ 肌荒れ</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>De:maf</t>
+        </is>
+      </c>
+      <c r="F709" t="n">
+        <v>4857</v>
+      </c>
+      <c r="G709" t="n">
+        <v>0</v>
+      </c>
+      <c r="H709" t="b">
+        <v>0</v>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J709" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203787114</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>1204259978</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>【インナードライクリーム】ブラックライス5モイスチャライジングクリーム 50ml 保湿 乾燥肌 水光肌 水分 乾燥 高保湿 うるおい もちもち ベタつかない 水分チャージ</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>haruharu wonder</t>
+        </is>
+      </c>
+      <c r="F710" t="n">
+        <v>4396</v>
+      </c>
+      <c r="G710" t="n">
+        <v>0</v>
+      </c>
+      <c r="H710" t="b">
+        <v>0</v>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J710" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204259978</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>1208516387</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>SEOUL_ON</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>【夏向けサラサラ日焼け止め】3番 ノーファンデ陶器肌トーンアップUVクリームEX, 50ml／ベタつかない／さっぱり／日差し対策／紫外線対策／ベースメイク／化粧下地／</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F711" t="n">
+        <v>2609</v>
+      </c>
+      <c r="G711" t="n">
+        <v>0</v>
+      </c>
+      <c r="H711" t="b">
+        <v>0</v>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J711" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208516387</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J701"/>
+  <autoFilter ref="A1:J711"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 111, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$711</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$715</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J711"/>
+  <dimension ref="A1:J715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29606,8 +29606,172 @@
         </is>
       </c>
     </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>1199604337</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>ヨモギクーリングカミングジェル100ml/アロエベラ/熱感鎮静/ナイトパック/鎮静パック/敏感肌/トラブル/熱感鎮静</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>グレイメリン</t>
+        </is>
+      </c>
+      <c r="F712" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G712" t="n">
+        <v>2</v>
+      </c>
+      <c r="H712" t="b">
+        <v>0</v>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J712" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199604337</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>1202850935</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>[単品]センテラクイックカーミングパッド70枚入り/パック/パッド/トナーパッド/化粧水/トナー/拭き取りシート/鎮静/水分/保湿</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F713" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G713" t="n">
+        <v>0</v>
+      </c>
+      <c r="H713" t="b">
+        <v>0</v>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J713" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202850935</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>1202849422</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>[1+1]センテラアンプルマダガスカル産CICA 美容液55ml/弱酸性pH/敏感肌/天然由来成分/ツボクサエキス/敏感肌鎮静効果</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F714" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G714" t="n">
+        <v>0</v>
+      </c>
+      <c r="H714" t="b">
+        <v>0</v>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J714" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202849422</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>1202836073</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>[単品][集中ケア用]リードルショットヘアエッセンス300dL/スカルプエッセンス/スカルプリードルショット/ヘアアンプル</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F715" t="n">
+        <v>3580</v>
+      </c>
+      <c r="G715" t="n">
+        <v>0</v>
+      </c>
+      <c r="H715" t="b">
+        <v>0</v>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J715" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202836073</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J711"/>
+  <autoFilter ref="A1:J715"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 114, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$715</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$725</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J715"/>
+  <dimension ref="A1:J725"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29770,8 +29770,418 @@
         </is>
       </c>
     </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>1149453077</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>dal24</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>プロフェッショナル頭皮シャンプーブラシ1本 韓国 頭皮 ブラシ シャンプー 櫛 マッサージ 角質 フケ におい ヘアー</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>rolencos</t>
+        </is>
+      </c>
+      <c r="F716" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G716" t="n">
+        <v>0</v>
+      </c>
+      <c r="H716" t="b">
+        <v>0</v>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J716" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149453077</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>1116944837</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>9種の中から 選択1 / ゴールドコアマックスキッズ肝臓ケア植物性糖ケアスリム50代 韓国製品 韓国乳酸菌 乳酸菌 キッズ プロバイオティクス ミルクシスル ガルシニア ビタミンD 生乳酸菌</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>ラクトフィット</t>
+        </is>
+      </c>
+      <c r="F717" t="n">
+        <v>2580</v>
+      </c>
+      <c r="G717" t="n">
+        <v>5</v>
+      </c>
+      <c r="H717" t="b">
+        <v>0</v>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J717" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116944837</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>1115638534</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>旅行用ヘアボディ5種+コットンポーチ1セット 韓国シャンプー 純正品 旅行キット トラベルキット トリートメント ボディウォッシュ ボディローション クレンジングフォーム 旅行 携帯用シャンプー</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>NARD</t>
+        </is>
+      </c>
+      <c r="F718" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G718" t="n">
+        <v>0</v>
+      </c>
+      <c r="H718" t="b">
+        <v>0</v>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J718" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115638534</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>1135071615</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>fineskin</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>【うるおいケア】アトラク スキンフェンス クリーム ミスト140ml 140ml ナイトクリーム 保湿クリーム 韓国コスメ エイジングケアクリーム シカクリーム シカバーム バリアクリーム</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Ruby-Cell</t>
+        </is>
+      </c>
+      <c r="F719" t="n">
+        <v>5900</v>
+      </c>
+      <c r="G719" t="n">
+        <v>0</v>
+      </c>
+      <c r="H719" t="b">
+        <v>0</v>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J719" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135071615</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>1191487583</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>marumarushop</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>大豆エッセンス 50ml</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>ミクスン</t>
+        </is>
+      </c>
+      <c r="F720" t="n">
+        <v>5076</v>
+      </c>
+      <c r="G720" t="n">
+        <v>1</v>
+      </c>
+      <c r="H720" t="b">
+        <v>0</v>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J720" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191487583</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>1176819992</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>marumarushop</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>フルイド フェルメント トーンアップパッド 250ml（50枚入り）</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>ネオゼン</t>
+        </is>
+      </c>
+      <c r="F721" t="n">
+        <v>5057</v>
+      </c>
+      <c r="G721" t="n">
+        <v>0</v>
+      </c>
+      <c r="H721" t="b">
+        <v>0</v>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176819992</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>1124910554</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>marumarushop</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>フレッシュマスク 10枚</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F722" t="n">
+        <v>2070</v>
+      </c>
+      <c r="G722" t="n">
+        <v>0</v>
+      </c>
+      <c r="H722" t="b">
+        <v>0</v>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1124910554</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>1168203274</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>happyclover</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>スピーディー マスカラリムーバー</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>ヒロインメイク</t>
+        </is>
+      </c>
+      <c r="F723" t="n">
+        <v>2417</v>
+      </c>
+      <c r="G723" t="n">
+        <v>4</v>
+      </c>
+      <c r="H723" t="b">
+        <v>0</v>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J723" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168203274</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>1202779298</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>ooznary</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>【New 毛穴レスケア】アイスレチノール37セラム 30ml　レチノール 美容液 ハリ キメケア 角質ケア 水光肌 毛穴引き締め たるみ毛穴 ナイアシンアミド AHA BHA</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>オーズナリー</t>
+        </is>
+      </c>
+      <c r="F724" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G724" t="n">
+        <v>0</v>
+      </c>
+      <c r="H724" t="b">
+        <v>0</v>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J724" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202779298</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>1191236161</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>tiam_official</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>【毛穴ケア】 ポアミニマイジング21セラム 40ml</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>ティアム</t>
+        </is>
+      </c>
+      <c r="F725" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G725" t="n">
+        <v>2</v>
+      </c>
+      <c r="H725" t="b">
+        <v>0</v>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J725" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191236161</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J715"/>
+  <autoFilter ref="A1:J725"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 117, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$725</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$729</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J725"/>
+  <dimension ref="A1:J729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30180,8 +30180,172 @@
         </is>
       </c>
     </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>1205730098</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>dsire88</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>[NEW]アトバリア 365 カプセルトナー 300ml/アトバリア/韓国スキンケア/PHA/カプセルトナー/セラミド/保湿/アトバリア 化粧水/乾燥肌/水分</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F726" t="n">
+        <v>3996</v>
+      </c>
+      <c r="G726" t="n">
+        <v>0</v>
+      </c>
+      <c r="H726" t="b">
+        <v>0</v>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205730098</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>1093447562</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>dsire88</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>ーモイスチャートリトメントマスク 5枚/保湿ケア</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F727" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G727" t="n">
+        <v>1</v>
+      </c>
+      <c r="H727" t="b">
+        <v>0</v>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J727" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093447562</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>1064912468</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>mayoomi</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>エイシカ365ハイドレーティングリリーフトナー pH4.5 200ml</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F728" t="n">
+        <v>2550</v>
+      </c>
+      <c r="G728" t="n">
+        <v>2</v>
+      </c>
+      <c r="H728" t="b">
+        <v>0</v>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1064912468</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>1064609458</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>mayoomi</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>テラクネ365アクティブセラム, 30ml</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F729" t="n">
+        <v>3520</v>
+      </c>
+      <c r="G729" t="n">
+        <v>5</v>
+      </c>
+      <c r="H729" t="b">
+        <v>0</v>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1064609458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J725"/>
+  <autoFilter ref="A1:J729"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 120, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$729</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$738</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J729"/>
+  <dimension ref="A1:J738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30344,8 +30344,377 @@
         </is>
       </c>
     </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>1174587339</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>angelrainbow</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>ブライトニング ピーリング ジェル ピーチ 100g + 100g フェイシャル スクラブ 顔 角質除去 敏感肌 低刺激 韓国 コスメ スキンケア</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>プル</t>
+        </is>
+      </c>
+      <c r="F730" t="n">
+        <v>2659</v>
+      </c>
+      <c r="G730" t="n">
+        <v>0</v>
+      </c>
+      <c r="H730" t="b">
+        <v>0</v>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174587339</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>1172128294</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>angelrainbow</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>コットンフット 足を洗おう フットシャンプー 385mlX2本 石鹸の香り さらさら 足 匂い ケア 韓国 スキンケア</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>オン・ザ・ボディー</t>
+        </is>
+      </c>
+      <c r="F731" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G731" t="n">
+        <v>0</v>
+      </c>
+      <c r="H731" t="b">
+        <v>0</v>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172128294</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>1168738382</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>angelrainbow</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>シークレット ライス 麹 ピーリング ツーフォーム クレンザー 120g デイリー 毛穴 角質 フェイシャル 洗顔 ケア キメ 低刺激 敏感肌 韓国 コスメ スキンケア</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F732" t="n">
+        <v>4089</v>
+      </c>
+      <c r="G732" t="n">
+        <v>0</v>
+      </c>
+      <c r="H732" t="b">
+        <v>0</v>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J732" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168738382</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>1191171558</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>sonny</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>[正規品] SKIN1004 プロバイオシカグロウサンアンプル, 50ml / SPF50+ PA++++ / 保湿 / スキンケア / 紫外線 / 乳液 / 白浮しない日焼け止め / オマケも /</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F733" t="n">
+        <v>2640</v>
+      </c>
+      <c r="G733" t="n">
+        <v>4</v>
+      </c>
+      <c r="H733" t="b">
+        <v>0</v>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191171558</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>1206023291</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>oreumpick</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>マジックプレス ペディキュア トマトクラッシュ 磁石ネイル 韓国 ペディチップ</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>ダッシングディバ</t>
+        </is>
+      </c>
+      <c r="F734" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G734" t="n">
+        <v>0</v>
+      </c>
+      <c r="H734" t="b">
+        <v>0</v>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J734" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206023291</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>1205988538</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>oreumpick</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>プライム プライマー セッティング フィクサー 50ml x 2個 韓国コスメ メイクキープ 韓国コスメ メイク</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F735" t="n">
+        <v>2557</v>
+      </c>
+      <c r="G735" t="n">
+        <v>2</v>
+      </c>
+      <c r="H735" t="b">
+        <v>0</v>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J735" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205988538</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>1164534478</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>lee0608</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>ハイドロセラミックトーンアップエッセンスサンクリーム50ml 2個</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F736" t="n">
+        <v>3410</v>
+      </c>
+      <c r="G736" t="n">
+        <v>0</v>
+      </c>
+      <c r="H736" t="b">
+        <v>0</v>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J736" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164534478</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>1136786757</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>lee0608</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>グリーンティーヒアルロン酸ミスト150ml 1個</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F737" t="n">
+        <v>1635</v>
+      </c>
+      <c r="G737" t="n">
+        <v>4</v>
+      </c>
+      <c r="H737" t="b">
+        <v>0</v>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J737" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136786757</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>1194316158</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>mijin-cosme</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>メール便 無料 - アクロパス ニードルパッチ 目元 ほうれい線 レチアールエヌ スリム パッチ 3box - PDRN × レチノール配合 - 部分集中ケア - 正規品</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>ACROPASS</t>
+        </is>
+      </c>
+      <c r="F738" t="n">
+        <v>8700</v>
+      </c>
+      <c r="G738" t="n">
+        <v>1</v>
+      </c>
+      <c r="H738" t="b">
+        <v>0</v>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J738" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194316158</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J729"/>
+  <autoFilter ref="A1:J738"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 123, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$738</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$755</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J738"/>
+  <dimension ref="A1:J755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30713,8 +30713,705 @@
         </is>
       </c>
     </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>1208658337</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>[Tamburins] SUMMER TAILS ディスカバリーセット</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F739" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G739" t="n">
+        <v>0</v>
+      </c>
+      <c r="H739" t="b">
+        <v>0</v>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J739" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208658337</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>1203988364</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>[大容量] オービタミネボディミルク 400ml</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>ビオテルム</t>
+        </is>
+      </c>
+      <c r="F740" t="n">
+        <v>6250</v>
+      </c>
+      <c r="G740" t="n">
+        <v>0</v>
+      </c>
+      <c r="H740" t="b">
+        <v>0</v>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J740" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203988364</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>1193624609</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>TXT愛用 BOMBSHELLUTH バムシェル 10ml Oil Perfumeオイル香水</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>DANIELS TRUTH</t>
+        </is>
+      </c>
+      <c r="F741" t="n">
+        <v>6550</v>
+      </c>
+      <c r="G741" t="n">
+        <v>3</v>
+      </c>
+      <c r="H741" t="b">
+        <v>0</v>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J741" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193624609</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>1189436342</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>VT リードルショット ユニバース キット 2ml × 5本 x 9種（全45本）正規品 韓国化粧品 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F742" t="n">
+        <v>3250</v>
+      </c>
+      <c r="G742" t="n">
+        <v>3</v>
+      </c>
+      <c r="H742" t="b">
+        <v>0</v>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J742" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189436342</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>1199921848</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>10by</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>【10+10】 リアルネイチャー エッセンス マスクパック アロエ 20枚 韓国コスメ デイリーマスク</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F743" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G743" t="n">
+        <v>0</v>
+      </c>
+      <c r="H743" t="b">
+        <v>0</v>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J743" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199921848</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>1199921787</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>10by</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>【10+10】 リアルネイチャー エッセンス マスクパックグリーンティー 韓国コスメ デイリーマスク</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F744" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G744" t="n">
+        <v>0</v>
+      </c>
+      <c r="H744" t="b">
+        <v>0</v>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J744" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199921787</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>1199921791</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>10by</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>【10+10】 リアルネイチャー エッセンス マスクパック バラ20枚 韓国コスメ デイリーマスク</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F745" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G745" t="n">
+        <v>0</v>
+      </c>
+      <c r="H745" t="b">
+        <v>0</v>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J745" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199921791</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>1160698785</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>DRsChoice</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>ジェントルマンオードパルファム50ml（3種類の香り）</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>I GENTLEMAN</t>
+        </is>
+      </c>
+      <c r="F746" t="n">
+        <v>5890</v>
+      </c>
+      <c r="G746" t="n">
+        <v>0</v>
+      </c>
+      <c r="H746" t="b">
+        <v>0</v>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J746" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160698785</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>1160698982</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>DRsChoice</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>ジェニーハウスプレミアムヘアカラー1+1企画セット5種類から選1</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>ジェニーハウス</t>
+        </is>
+      </c>
+      <c r="F747" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G747" t="n">
+        <v>1</v>
+      </c>
+      <c r="H747" t="b">
+        <v>0</v>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J747" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160698982</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>1193601980</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 100ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F748" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G748" t="n">
+        <v>2</v>
+      </c>
+      <c r="H748" t="b">
+        <v>0</v>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J748" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193601980</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>1206909143</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 240ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F749" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G749" t="n">
+        <v>0</v>
+      </c>
+      <c r="H749" t="b">
+        <v>0</v>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206909143</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>1202095634</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 240ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F750" t="n">
+        <v>4020</v>
+      </c>
+      <c r="G750" t="n">
+        <v>0</v>
+      </c>
+      <c r="H750" t="b">
+        <v>0</v>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202095634</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>1164831338</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>unipic</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>[選べる4タイプ] メイクアップセッティングフィクサー4種 / メイクキープ / フィクサーミスト / メイクキープスプレー／ウォータープルーフ/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F751" t="n">
+        <v>3390</v>
+      </c>
+      <c r="G751" t="n">
+        <v>0</v>
+      </c>
+      <c r="H751" t="b">
+        <v>0</v>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J751" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164831338</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>1193917787</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>unipic</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>[New] 1+1 バナナ PDRN 2X セラム 30ml+30ml T4コラーゲン ビタミンC ヒアルロン酸 30代 40代 スキンケア 韓国 マルチブースター</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F752" t="n">
+        <v>10870</v>
+      </c>
+      <c r="G752" t="n">
+        <v>0</v>
+      </c>
+      <c r="H752" t="b">
+        <v>0</v>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J752" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193917787</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>1183386465</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>unipic</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>[1+1]コラーゲンバブルアンプル 115ml + 115mlマイクロバブルセラム 美容導入液 化粧ノリが良くなる 20代 30代 40代 スキンケア しわ たるみ ほうれい線 美容液 泡 美容液</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>PO:DL</t>
+        </is>
+      </c>
+      <c r="F753" t="n">
+        <v>7999</v>
+      </c>
+      <c r="G753" t="n">
+        <v>0</v>
+      </c>
+      <c r="H753" t="b">
+        <v>0</v>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J753" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183386465</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>1162812871</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>unipic</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>[1+1]【BTS J-HOPE使用】シカ配合 鎮静トナーパッド 60枚+60枚 /シカ パック/韓国スキンケア/ 敏感肌 夏用/ K-ビューティー/スージングカームトナーパッド</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>neaf neaf</t>
+        </is>
+      </c>
+      <c r="F754" t="n">
+        <v>7770</v>
+      </c>
+      <c r="G754" t="n">
+        <v>0</v>
+      </c>
+      <c r="H754" t="b">
+        <v>0</v>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J754" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162812871</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>1163862886</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>unipic</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>[ウォーターバム出演者も使用！]メイクアップ セッティング マルチ マジック シラー 10ml /アイメイク用フィクサー/プールメイク/ウォータープルーフ/アイライン/マスカラ/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F755" t="n">
+        <v>2710</v>
+      </c>
+      <c r="G755" t="n">
+        <v>1</v>
+      </c>
+      <c r="H755" t="b">
+        <v>0</v>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J755" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163862886</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J738"/>
+  <autoFilter ref="A1:J755"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 58)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$987</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$988</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J987"/>
+  <dimension ref="A1:J988"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40922,8 +40922,49 @@
         </is>
       </c>
     </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>1111308183</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>momo_mall</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>8番 韓方エキスセラム, 50ml</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F988" t="n">
+        <v>4950</v>
+      </c>
+      <c r="G988" t="n">
+        <v>0</v>
+      </c>
+      <c r="H988" t="b">
+        <v>0</v>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J988" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1111308183</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J987"/>
+  <autoFilter ref="A1:J988"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 1, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$255</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J242"/>
+  <dimension ref="A1:J255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10379,8 +10379,541 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>1188407209</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>lador_jp</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>【新発売】ティーツリーカーミングスカルプシャンプー/トリートメント/頭皮ケアシリーズ/爽快頭皮ケア/敏感頭皮</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>La'dor</t>
+        </is>
+      </c>
+      <c r="F243" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G243" t="n">
+        <v>0</v>
+      </c>
+      <c r="H243" t="b">
+        <v>0</v>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188407209</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>1194978052</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>aekyungjapan</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>【KERASYS日本公式ストア】【1Lx1個】韓国シャンプー ケラシス デビルズ パフューム 香水シャンプー＆コンディショナー ヘアケア</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F244" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G244" t="n">
+        <v>9</v>
+      </c>
+      <c r="H244" t="b">
+        <v>0</v>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194978052</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>1128056319</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>aekyungjapan</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>【KERASYS日本公式ストア】(750ml×2個)韓国シャンプー ケラシス シカラボ シャンプー＆コンディショナー シカ 頭皮ケア ヘアケア</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F245" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G245" t="n">
+        <v>11</v>
+      </c>
+      <c r="H245" t="b">
+        <v>0</v>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1128056319</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>1209047604</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>aekyungjapan</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>【KERASYS日本公式ストア】【1L×4個】韓国シャンプー ケラシス デビルズ パフューム 香水シャンプー＆コンディショナー ヘアケア</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F246" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G246" t="n">
+        <v>6</v>
+      </c>
+      <c r="H246" t="b">
+        <v>0</v>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209047604</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>1097778656</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>aihada</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>[大容量]パフュームシャンプー+リンスセット(Sweet&amp;amp;Flowery)(Fresh&amp;amp;Lush)香り高い毛髪ツヤケア</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F247" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G247" t="n">
+        <v>9</v>
+      </c>
+      <c r="H247" t="b">
+        <v>0</v>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097778656</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>1210156637</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>kdstore</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>1+1+1+1 デンギヘアジンギシャンプートリートメント500ml(4個選択)</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>デンギモリ</t>
+        </is>
+      </c>
+      <c r="F248" t="n">
+        <v>5580</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="b">
+        <v>0</v>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210156637</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>1178120581</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>forest_by_greenfinger_official</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>【１＋１】訳あり / フォレストギュルタミンビタトーニングセラム 50mL /美容液/ナイアシンアミド</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>FoRest</t>
+        </is>
+      </c>
+      <c r="F249" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G249" t="n">
+        <v>6</v>
+      </c>
+      <c r="H249" t="b">
+        <v>0</v>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178120581</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>1176613711</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>forest_by_greenfinger_official</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>【1+1】訳あり/フォレストギュルタミンビタトーニングゲルセラムパッド 75枚入り /ナイアシンアミド/集中ケアパッド</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>FoRest</t>
+        </is>
+      </c>
+      <c r="F250" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G250" t="n">
+        <v>11</v>
+      </c>
+      <c r="H250" t="b">
+        <v>0</v>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176613711</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>1178120837</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>forest_by_greenfinger_official</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>【１＋１】訳あり /フォレストピトン水分CICAクリーム 50ml /インナードライ/しっとり保湿</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>FoRest</t>
+        </is>
+      </c>
+      <c r="F251" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G251" t="n">
+        <v>7</v>
+      </c>
+      <c r="H251" t="b">
+        <v>0</v>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178120837</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>1176613894</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>forest_by_greenfinger_official</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>【１＋１】訳あり / フォレストギュルタミンビタトーニングサンクリーム 50mL /トーンアップ日焼け止めクリーム/メイク下地/SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>FoRest</t>
+        </is>
+      </c>
+      <c r="F252" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G252" t="n">
+        <v>8</v>
+      </c>
+      <c r="H252" t="b">
+        <v>0</v>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176613894</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>1132023348</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>TigerStore</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>1+1 オム ウォーター Whitening スキンローション オールインワンエッセンス 211ml 2個</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>PAUL MEDISON</t>
+        </is>
+      </c>
+      <c r="F253" t="n">
+        <v>4590</v>
+      </c>
+      <c r="G253" t="n">
+        <v>0</v>
+      </c>
+      <c r="H253" t="b">
+        <v>0</v>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132023348</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>1209949431</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>droracle_official</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>【鎮静バリア美容液】 センテラバイオームシカアンプル 50ml CICA ゆらぎ肌 敏感肌 水分チャージ ベタつかない バリアケア 鎮静 Centella Biome</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>ドクターオラクル</t>
+        </is>
+      </c>
+      <c r="F254" t="n">
+        <v>4140</v>
+      </c>
+      <c r="G254" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" t="b">
+        <v>0</v>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209949431</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>1206813636</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>droracle_official</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>【鎮静サンセラム】 センテラバイオームスージングサンセラム 日焼け止め 50ml SPF50+ PA++++ CICA UVケア クーリング 紫外線ダメージ 鎮静 Centella Biome</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>ドクターオラクル</t>
+        </is>
+      </c>
+      <c r="F255" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G255" t="n">
+        <v>1</v>
+      </c>
+      <c r="H255" t="b">
+        <v>0</v>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206813636</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J242"/>
+  <autoFilter ref="A1:J255"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 2, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$271</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$274</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J271"/>
+  <dimension ref="A1:J274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11568,8 +11568,131 @@
         </is>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>1212263577</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>niko66</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>NAKICO 薬用フェイスジェルクリーム 30g サラ肌 制汗 顔汗 メイク 仕上げ 崩れ防止 テカリ防止 フェイス クリーム</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>NAKICO</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="b">
+        <v>0</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212263577</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>1178438838</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>milo</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>【セット販売】LADAMER ラダメール セラム 50ml・ピーリング ピンプルパッド 30枚入 正規品</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LADAMER</t>
+        </is>
+      </c>
+      <c r="F273" t="n">
+        <v>15400</v>
+      </c>
+      <c r="G273" t="n">
+        <v>1</v>
+      </c>
+      <c r="H273" t="b">
+        <v>0</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178438838</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>1196260969</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>BeautyTokTok</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>ハミング 米とぎ水 BBローション 30ml ナチュラルツヤ肌 カバー 下地 ファンデーション 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>haming</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G274" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" t="b">
+        <v>0</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196260969</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J271"/>
+  <autoFilter ref="A1:J274"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 4, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$295</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$296</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J295"/>
+  <dimension ref="A1:J296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12552,8 +12552,49 @@
         </is>
       </c>
     </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>1176114530</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>jellyko</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>【毛穴ケア 美容液 1+1】グリーントマト フォアリフティング セラム プレーン 30ml / 韓国コスメ / 毛穴 美容液</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="b">
+        <v>0</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176114530</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J295"/>
+  <autoFilter ref="A1:J296"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 7, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$302</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$307</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J302"/>
+  <dimension ref="A1:J307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12839,8 +12839,213 @@
         </is>
       </c>
     </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>1130723477</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>alos-hmo</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>洗顔 濃密泡 敏感肌 クレイ 酢 オーガニック 無添加 120g 高保湿 美肌菌 乾燥肌 メンズ 毛穴 ケア 泥 洗顔フォーム 保湿 肌荒れ 対策 洗顔料 毛穴汚れ ビタミンc レチノール 黒ずみ</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>ALOS ORGANIC</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G303" t="n">
+        <v>2</v>
+      </c>
+      <c r="H303" t="b">
+        <v>0</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130723477</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>1120927911</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>alos-hmo</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>アイリンビューティクリーム ボディクリーム 保湿 乾燥肌 敏感肌 手荒れ クリーム 保湿クリーム 潤い ツヤ ハリ アロエ 大容量 215g ハンドクリーム メンズ レディース フェイスクリーム</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>アイリン</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G304" t="n">
+        <v>6</v>
+      </c>
+      <c r="H304" t="b">
+        <v>0</v>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120927911</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>1095957006</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>thefuture</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>BBクリーム 30g　毛穴 赤み 青髭 ニキビ跡 クマ</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>THE FUTURE</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G305" t="n">
+        <v>3</v>
+      </c>
+      <c r="H305" t="b">
+        <v>0</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1095957006</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>1208305485</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>thefuture</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>THE FUTURE 洗顔料 150g 黒ずみ 毛穴 皮脂 毛穴汚れ 泡立て不要 ジェル洗顔 洗顔</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>THE FUTURE</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="b">
+        <v>0</v>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208305485</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>1181187092</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>thefuture</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>フェイスシートパック 50枚 洗顔 化粧水 部分用シートマスク</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>THE FUTURE</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G307" t="n">
+        <v>6</v>
+      </c>
+      <c r="H307" t="b">
+        <v>0</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181187092</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J302"/>
+  <autoFilter ref="A1:J307"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 8, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$307</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$308</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J307"/>
+  <dimension ref="A1:J308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13044,8 +13044,49 @@
         </is>
       </c>
     </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>969182336</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>secondtable</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>【詰め替え用】 モイスト シャンプー 400mL 2種類のヒト幹細胞培養液配合 ヒト幹細胞シャンプー クレイシャンプー 泥シャンプー レディース メンズ ギフト</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>JOIE CELU</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>1430</v>
+      </c>
+      <c r="G308" t="n">
+        <v>6</v>
+      </c>
+      <c r="H308" t="b">
+        <v>0</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=969182336</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J307"/>
+  <autoFilter ref="A1:J308"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 5, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$312</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$315</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J312"/>
+  <dimension ref="A1:J315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13249,8 +13249,131 @@
         </is>
       </c>
     </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>1194718785</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>taroshop01</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>アンドラム ( レスレクション ) アロマティック ハンドウォッシュ 500ml ハンド ソープ ハンドソープ</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>イソップ</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>6400</v>
+      </c>
+      <c r="G313" t="n">
+        <v>1</v>
+      </c>
+      <c r="H313" t="b">
+        <v>0</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194718785</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>1198295280</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>taroshop01</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>アトピアd 美白保湿クリーム 90g アライアンスファーマー薬用アトピアd美白保湿 薬用 薬用美白 オールインワンジェル 乾燥肌 スキンケア 保湿クリーム 保湿 ヘパリン類似物質 プラセンタ</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>アトピアD</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G314" t="n">
+        <v>1</v>
+      </c>
+      <c r="H314" t="b">
+        <v>0</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198295280</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>1187953336</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>taroshop01</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>スキンピールバー 赤 黒 ハイドロキノール ピーリング ピーリング石鹼 洗顔せっけん 洗顔 洗顔石鹼 固形石鹼 AHAマイルド AHA ティートゥリー ハイドロキノール</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>サンソリット</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>2380</v>
+      </c>
+      <c r="G315" t="n">
+        <v>4</v>
+      </c>
+      <c r="H315" t="b">
+        <v>0</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187953336</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J312"/>
+  <autoFilter ref="A1:J315"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 10, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$517</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$522</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J517"/>
+  <dimension ref="A1:J522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21478,8 +21478,213 @@
         </is>
       </c>
     </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>1211777191</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>korea_gudz</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>【リルリル】4世代 エアフィット 保湿 鎮静 日焼け止め 50ml SPF50+/PA++++</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>LYLYL</t>
+        </is>
+      </c>
+      <c r="F518" t="n">
+        <v>6820</v>
+      </c>
+      <c r="G518" t="n">
+        <v>0</v>
+      </c>
+      <c r="H518" t="b">
+        <v>0</v>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211777191</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>1154522502</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>【跡ケア＆ブライトニング】ナイアシンアミド 20% セラム20ml+20ml / 低刺激 / 集中ケア / 皮脂ケア / 滑らか肌 / 角層浸透 / 高濃縮 / 輝き</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F519" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G519" t="n">
+        <v>0</v>
+      </c>
+      <c r="H519" t="b">
+        <v>0</v>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154522502</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>1169527041</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>ブロッサム ボディウォッシュ 900ml (ピーチ /ピオニー/チェリー)</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>ハッピーバス</t>
+        </is>
+      </c>
+      <c r="F520" t="n">
+        <v>1450</v>
+      </c>
+      <c r="G520" t="n">
+        <v>0</v>
+      </c>
+      <c r="H520" t="b">
+        <v>0</v>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169527041</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>1169174214</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>プロポリス レスキューアンプル 50mL</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>CNP Laboratory</t>
+        </is>
+      </c>
+      <c r="F521" t="n">
+        <v>3250</v>
+      </c>
+      <c r="G521" t="n">
+        <v>0</v>
+      </c>
+      <c r="H521" t="b">
+        <v>0</v>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169174214</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>1157772908</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>プリミュンモイスチャーローション 350ml+350ml</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>GOONGBE</t>
+        </is>
+      </c>
+      <c r="F522" t="n">
+        <v>7300</v>
+      </c>
+      <c r="G522" t="n">
+        <v>0</v>
+      </c>
+      <c r="H522" t="b">
+        <v>0</v>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157772908</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J517"/>
+  <autoFilter ref="A1:J522"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 11, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$522</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$526</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J522"/>
+  <dimension ref="A1:J526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21683,8 +21683,172 @@
         </is>
       </c>
     </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>1175555635</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>BboBboShop</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>ヒアテノールハイドラカプセルエッセンス50ml+トナー150ml+クリーム50ml</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F523" t="n">
+        <v>6360</v>
+      </c>
+      <c r="G523" t="n">
+        <v>0</v>
+      </c>
+      <c r="H523" t="b">
+        <v>0</v>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175555635</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>1189005367</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>BboBboShop</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>コラーゲンドリームクリーム50ml 2個</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F524" t="n">
+        <v>5040</v>
+      </c>
+      <c r="G524" t="n">
+        <v>0</v>
+      </c>
+      <c r="H524" t="b">
+        <v>0</v>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189005367</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>1185447621</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>BboBboShop</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>語彙草トライアルキット（スキンブースター20ml＋セラム15ml＋チューブ30ml＋フォーム30ml）</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F525" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G525" t="n">
+        <v>0</v>
+      </c>
+      <c r="H525" t="b">
+        <v>0</v>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185447621</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>1185044020</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>BboBboShop</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>"ホテルセラピー大容量ボディウォッシュスイセン1.013L2個 "</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>ヘトラス</t>
+        </is>
+      </c>
+      <c r="F526" t="n">
+        <v>4420</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0</v>
+      </c>
+      <c r="H526" t="b">
+        <v>0</v>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185044020</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J522"/>
+  <autoFilter ref="A1:J526"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 13, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$526</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$530</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J526"/>
+  <dimension ref="A1:J530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21847,8 +21847,172 @@
         </is>
       </c>
     </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>1207660785</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>marynmayjp</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>【公式】鎮静ケア３種セット・トナー1種・クリーム2種／美容液／アゼライン酸／CICA／ニキビ／肌荒れ／ゆらぎ肌／トラブル肌／ハリツヤ肌／毛穴ケア／なめらか肌／うるおい</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F527" t="n">
+        <v>3301</v>
+      </c>
+      <c r="G527" t="n">
+        <v>1</v>
+      </c>
+      <c r="H527" t="b">
+        <v>0</v>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207660785</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>1214413889</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>marynmayjp</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>【公式】デイリーマスク1+1セット30枚入り５種／パック／CICA／ビタミンC／ヒアルロン酸／コラーゲン／イデベノン／保湿・毛穴・ハリケア／韓国コスメ／ヴィーガン</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F528" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G528" t="n">
+        <v>1</v>
+      </c>
+      <c r="H528" t="b">
+        <v>0</v>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214413889</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>1214410208</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>marynmayjp</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>【公式】選べる1+1セットスピキュールPDRNクリーム／レチノール／コラーゲン／アゼライン酸／ニキビケア／毛穴／なめらか肌／肌荒れ／化粧ノリ／うるおい／ハリケア／スポットケア</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F529" t="n">
+        <v>2744</v>
+      </c>
+      <c r="G529" t="n">
+        <v>0</v>
+      </c>
+      <c r="H529" t="b">
+        <v>0</v>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214410208</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>1159021623</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>ztu_jp</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>【顔用】リーズフィット タイトニング コラーゲン 石膏パック 13g 5枚入【せっこうパック, 石膏マスクパック, 韓国パック】</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>ZTU</t>
+        </is>
+      </c>
+      <c r="F530" t="n">
+        <v>2430</v>
+      </c>
+      <c r="G530" t="n">
+        <v>0</v>
+      </c>
+      <c r="H530" t="b">
+        <v>0</v>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159021623</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J526"/>
+  <autoFilter ref="A1:J530"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 14, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$530</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$535</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J530"/>
+  <dimension ref="A1:J535"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22011,8 +22011,213 @@
         </is>
       </c>
     </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>1104805693</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>esfolio</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>コラーゲン モイスチャー エッセンス 大容量 クリーム 200g コラーゲン レチノール しわ 弾力ケア 保湿ケア 30代以上の必須アイテム</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>esfolio</t>
+        </is>
+      </c>
+      <c r="F531" t="n">
+        <v>1690</v>
+      </c>
+      <c r="G531" t="n">
+        <v>1</v>
+      </c>
+      <c r="H531" t="b">
+        <v>0</v>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1104805693</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>1104881357</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>esfolio</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>ビタミン アンプルマスクシート4種//ビタミンABCEアンプルマスクパック計40枚 弾力保湿週間改善</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>esfolio</t>
+        </is>
+      </c>
+      <c r="F532" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G532" t="n">
+        <v>7</v>
+      </c>
+      <c r="H532" t="b">
+        <v>0</v>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1104881357</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>1104879132</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>esfolio</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>ペプチド コラーゲン トナー 180ml/レチノール化粧水 /レチノール化粧品/レチノール 肌の弾力効果</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>esfolio</t>
+        </is>
+      </c>
+      <c r="F533" t="n">
+        <v>1180</v>
+      </c>
+      <c r="G533" t="n">
+        <v>2</v>
+      </c>
+      <c r="H533" t="b">
+        <v>0</v>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1104879132</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>1141646474</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>VENDERMA</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>スージング ブースター・毛穴ゼロ・ニキビケア・高保湿 レッドカーミング シカ エクソ スーディングクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>VENDERMA</t>
+        </is>
+      </c>
+      <c r="F534" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G534" t="n">
+        <v>0</v>
+      </c>
+      <c r="H534" t="b">
+        <v>0</v>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141646474</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>1097452926</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>VENDERMA</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>ゼロ毛穴・スージングブースター・ニキビ・赤み・リファイニング レッドカーミング シカ エクソソーム トナーエッセンス 150ml</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>VENDERMA</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G535" t="n">
+        <v>5</v>
+      </c>
+      <c r="H535" t="b">
+        <v>0</v>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097452926</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J530"/>
+  <autoFilter ref="A1:J535"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 16, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$535</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$540</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J535"/>
+  <dimension ref="A1:J540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22216,8 +22216,213 @@
         </is>
       </c>
     </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>1205951710</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>レチノール ハイドロゲルマスク フェイス＆ネック用 4枚入り/5種ペプチド コラーゲン配合 保湿 密着ケア ハイドロゲルシート ナイトケア 韓国スキンケア/顔から首元まで集中保湿ケア</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G536" t="n">
+        <v>0</v>
+      </c>
+      <c r="H536" t="b">
+        <v>0</v>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205951710</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>1193888835</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>PDRN TX1 パーフェクトフィット リジュアル 幹細胞クリーム 30g/ローズ PDRN 21%配合 植物性 水分クリーム/キメケア 弾力 保湿/韓国コスメ (敏感肌/乾燥肌)/次世代スキンケア</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G537" t="n">
+        <v>3</v>
+      </c>
+      <c r="H537" t="b">
+        <v>0</v>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193888835</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>1212330250</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>シカエクソソーム＆ビタミンK複合体リポソーム配合の滑らかな肌質感を目指すトリプル角質ケアセラム 50ml</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G538" t="n">
+        <v>0</v>
+      </c>
+      <c r="H538" t="b">
+        <v>0</v>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212330250</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>1212328445</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>レチノール ロールオン アイクリーム 30ml 2個 韓国製 目元ケア しわ たるみ 乾燥 小じわ ハリ感 保湿 ステンレス製3連ローラーボール クーリングマッサージ</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F539" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G539" t="n">
+        <v>0</v>
+      </c>
+      <c r="H539" t="b">
+        <v>0</v>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212328445</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>1207653547</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>植物由来PDRN配合 保湿クリーム 60ml / 8種のヒアルロン酸 セラミド シカ 配合 べたつかない 敏感肌 デイリーケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F540" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G540" t="n">
+        <v>0</v>
+      </c>
+      <c r="H540" t="b">
+        <v>0</v>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207653547</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J535"/>
+  <autoFilter ref="A1:J540"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 17, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$540</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$543</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J540"/>
+  <dimension ref="A1:J543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22421,8 +22421,131 @@
         </is>
       </c>
     </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>1208145396</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>sogokzip</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>holitual micro balancing essence 150ml</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>HOLITUAL</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>5730</v>
+      </c>
+      <c r="G541" t="n">
+        <v>0</v>
+      </c>
+      <c r="H541" t="b">
+        <v>0</v>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208145396</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>1203305204</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>sogokzip</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>neostrata ultra moisturizing face cream 40g</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>ネオストラータ</t>
+        </is>
+      </c>
+      <c r="F542" t="n">
+        <v>7540</v>
+      </c>
+      <c r="G542" t="n">
+        <v>0</v>
+      </c>
+      <c r="H542" t="b">
+        <v>0</v>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203305204</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>1198398322</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>sogokzip</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>cell fusion c physiologocal cleansing gel 1000ml</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F543" t="n">
+        <v>6950</v>
+      </c>
+      <c r="G543" t="n">
+        <v>0</v>
+      </c>
+      <c r="H543" t="b">
+        <v>0</v>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198398322</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J540"/>
+  <autoFilter ref="A1:J543"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 19, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$547</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J547"/>
+  <dimension ref="A1:J550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22708,8 +22708,131 @@
         </is>
       </c>
     </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>778865590</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>coreacosme</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>拱辰享(ゴンジンヒャン) クレンジングオイル 1ml*30枚 サンプル/メイク落とし/Gongjinhyang</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>THE WHOO</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>990</v>
+      </c>
+      <c r="G548" t="n">
+        <v>1</v>
+      </c>
+      <c r="H548" t="b">
+        <v>0</v>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=778865590</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>1203536851</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>bravity</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>【公式】スキンリブートスピキュールセラム 30ml／美容液／角質ケア／毛穴ケア／トーンアップ／ツボクサ由来幹細胞エキス配合／うるおい</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>BRAVITY</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>4569</v>
+      </c>
+      <c r="G549" t="n">
+        <v>1</v>
+      </c>
+      <c r="H549" t="b">
+        <v>0</v>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203536851</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>1203536791</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>bravity</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>【公式】ビタフレックス91アンプル35ml／美容液／複合ビタミン／ビタミンB／ビタミンC／ツボクサエキス／美白／トーンアップ／くすみ／しみ</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>BRAVITY</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>5390</v>
+      </c>
+      <c r="G550" t="n">
+        <v>1</v>
+      </c>
+      <c r="H550" t="b">
+        <v>0</v>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203536791</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J547"/>
+  <autoFilter ref="A1:J550"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 20, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$552</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J550"/>
+  <dimension ref="A1:J552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22831,8 +22831,90 @@
         </is>
       </c>
     </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>1210626710</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>oneohoh</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>アイクリーム エイジングケア 目元ケア 人参プロコラーゲンアイクリーム 20ml 目元のシワ たるみ 乾燥 小じわケア 目元保湿 コラーゲンクリーム</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>ONEOHOH</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G551" t="n">
+        <v>0</v>
+      </c>
+      <c r="H551" t="b">
+        <v>0</v>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210626710</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>1167456598</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>itssome</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>[ランダムマスクパック10枚100円イベント！] アクアウォーター グローシカクリーム 80g / 水分補給クリーム</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>イッツソーミー</t>
+        </is>
+      </c>
+      <c r="F552" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G552" t="n">
+        <v>0</v>
+      </c>
+      <c r="H552" t="b">
+        <v>0</v>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167456598</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J550"/>
+  <autoFilter ref="A1:J552"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 25, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$558</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$560</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J558"/>
+  <dimension ref="A1:J560"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23159,8 +23159,90 @@
         </is>
       </c>
     </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>1205606322</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>cosmenara</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>ゲラン オーキデ アンペリアル ザ ロンジェビティ クリーム 21ml(7ml×3個) /Orchidee Imperiale Exceptional Complete Longevity Cream</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>ゲラン</t>
+        </is>
+      </c>
+      <c r="F559" t="n">
+        <v>8980</v>
+      </c>
+      <c r="G559" t="n">
+        <v>3</v>
+      </c>
+      <c r="H559" t="b">
+        <v>0</v>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205606322</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>1214837432</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>cosmenara</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>エスティローダー リニュートリィブ ダイヤモンド AR アイ クリーム 10ml(5ml×2個) / Re-Nutriv Ultimate Diamond Age Reversal Eye Cream</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>エスティローダー</t>
+        </is>
+      </c>
+      <c r="F560" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G560" t="n">
+        <v>0</v>
+      </c>
+      <c r="H560" t="b">
+        <v>0</v>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214837432</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J558"/>
+  <autoFilter ref="A1:J560"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 26, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$560</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$565</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J560"/>
+  <dimension ref="A1:J565"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23241,8 +23241,213 @@
         </is>
       </c>
     </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>1197712140</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>[単品/1+1]ヨモギ灸漢方温熱パック100ml/漢方スキンケア/毛穴掃除/肌鎮静/エステティックサロンケア/スティームパック</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>グレイメリン</t>
+        </is>
+      </c>
+      <c r="F561" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G561" t="n">
+        <v>1</v>
+      </c>
+      <c r="H561" t="b">
+        <v>0</v>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197712140</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>1191374592</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>[天然由来成分]ヨモギ日焼け止めSPF50+/PA++++50ml/単品&amp;amp;1+1/肌に優しいサンスクリーム/美白・しわ改善機能性/鎮静成分/ナイアシンアミド日焼け</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>グレイメリン</t>
+        </is>
+      </c>
+      <c r="F562" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G562" t="n">
+        <v>1</v>
+      </c>
+      <c r="H562" t="b">
+        <v>0</v>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191374592</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>1202852381</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>[セット特価]センテラCICAアンプル55ml+センテラクイックカーミングパッド70枚入/敏感肌/赤み/角質取り/デイリーケア</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F563" t="n">
+        <v>4750</v>
+      </c>
+      <c r="G563" t="n">
+        <v>0</v>
+      </c>
+      <c r="H563" t="b">
+        <v>0</v>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202852381</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>1200748192</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>lilyhouse_jp</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>[オリーブヤング入店]キャノーラクレイジー クレンジングオイル500ml/メイク落とし/クレンジング/p.m2.5洗浄/低刺激/角栓洗浄</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>グレイメリン</t>
+        </is>
+      </c>
+      <c r="F564" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G564" t="n">
+        <v>0</v>
+      </c>
+      <c r="H564" t="b">
+        <v>0</v>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200748192</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>1213025686</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>k-kosumekonbini</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>[2+1/ オリーブヤング 1位]レッドラクトコラーゲン 洗顔フォーム 2.0 / 毛穴収縮 / 洗顔 毛穴 / 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G565" t="n">
+        <v>0</v>
+      </c>
+      <c r="H565" t="b">
+        <v>0</v>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213025686</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J560"/>
+  <autoFilter ref="A1:J565"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 29, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$565</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$566</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J565"/>
+  <dimension ref="A1:J566"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23446,8 +23446,49 @@
         </is>
       </c>
     </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>1210182766</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>tocobojapan</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>【1日2個まで！8/13～8/17・記念タイムセール】【地上波テレビ番組で紹介！】ミニサンスティック単品/ ミニサイズ / ミニコットンソフト/ ミニシカクーリング / ミニビタウォータープルーフ</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>TOCOBO</t>
+        </is>
+      </c>
+      <c r="F566" t="n">
+        <v>990</v>
+      </c>
+      <c r="G566" t="n">
+        <v>0</v>
+      </c>
+      <c r="H566" t="b">
+        <v>0</v>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210182766</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J565"/>
+  <autoFilter ref="A1:J566"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 32, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$569</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$572</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J569"/>
+  <dimension ref="A1:J572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23610,8 +23610,131 @@
         </is>
       </c>
     </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>1157799652</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>20medicos</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>【新商品】 3エイジショット スピキュールバブルエッセンス / LED搭載 / ニードルスキンケア 50ml</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Dr.twentyproject</t>
+        </is>
+      </c>
+      <c r="F570" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G570" t="n">
+        <v>4</v>
+      </c>
+      <c r="H570" t="b">
+        <v>0</v>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157799652</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>1200869770</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>RYUSHOCORPORATION</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>ピーリング ホワイトクリアジェル 100g 薬用角質ケアジェル スキンケア ボディケア 美白 ニキビ予防</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Produced by Cure</t>
+        </is>
+      </c>
+      <c r="F571" t="n">
+        <v>1540</v>
+      </c>
+      <c r="G571" t="n">
+        <v>1</v>
+      </c>
+      <c r="H571" t="b">
+        <v>0</v>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200869770</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>1199111519</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>RYUSHOCORPORATION</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Cure キュア ナチュラルアクアジェル 100g ピーリングジェル 角質ケア Natural Aqua gel スキンケア ボディケア</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Produced by Cure</t>
+        </is>
+      </c>
+      <c r="F572" t="n">
+        <v>1320</v>
+      </c>
+      <c r="G572" t="n">
+        <v>1</v>
+      </c>
+      <c r="H572" t="b">
+        <v>0</v>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199111519</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J569"/>
+  <autoFilter ref="A1:J572"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 34, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$572</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$575</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J572"/>
+  <dimension ref="A1:J575"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23733,8 +23733,131 @@
         </is>
       </c>
     </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>1164831036</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>whitemaru</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Antiperspirant Deodorant フレッシュの香り 2本セット (74g / 本) 【並行輸入品】</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>ダヴ</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>2190</v>
+      </c>
+      <c r="G573" t="n">
+        <v>6</v>
+      </c>
+      <c r="H573" t="b">
+        <v>0</v>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164831036</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>1113164308</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>whitemaru</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>アクニドクター1stブラックディープクレンジングフォーム 75ml 韓国ブランド【正規品】 洗顔フォーム</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>アイソイ</t>
+        </is>
+      </c>
+      <c r="F574" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G574" t="n">
+        <v>8</v>
+      </c>
+      <c r="H574" t="b">
+        <v>0</v>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1113164308</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>1086692558</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>whitemaru</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>CICA セラミド クリーム 70g 韓国ブランド【正規品】 クリーム</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>ワンシング</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G575" t="n">
+        <v>9</v>
+      </c>
+      <c r="H575" t="b">
+        <v>0</v>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1086692558</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J572"/>
+  <autoFilter ref="A1:J575"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 37, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$575</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$577</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J575"/>
+  <dimension ref="A1:J577"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23856,8 +23856,90 @@
         </is>
       </c>
     </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>1116576465</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>bs-cosme</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>美容液 レチノール エッセンスTWK・20ｍL セラミド レチノール ビタミンC誘導体 アルジレリン 乳液</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>BS-COSME</t>
+        </is>
+      </c>
+      <c r="F576" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G576" t="n">
+        <v>4</v>
+      </c>
+      <c r="H576" t="b">
+        <v>0</v>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116576465</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>1172014960</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>bs-cosme</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>クール便チケット（送料）</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>BS-COSME</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>500</v>
+      </c>
+      <c r="G577" t="n">
+        <v>0</v>
+      </c>
+      <c r="H577" t="b">
+        <v>0</v>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172014960</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J575"/>
+  <autoFilter ref="A1:J577"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 40, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$578</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$580</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J578"/>
+  <dimension ref="A1:J580"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23979,8 +23979,90 @@
         </is>
       </c>
     </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>954179292</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>ciracle_cotde</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>鼻パック 毛穴悩ん 角栓除去 角栓取り 毛穴ケアコットンマスクブラックヘッドオフコットンマスク [純綿100%] (5mlx20枚)</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>シラクル</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>3860</v>
+      </c>
+      <c r="G579" t="n">
+        <v>2</v>
+      </c>
+      <c r="H579" t="b">
+        <v>0</v>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=954179292</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>1168768265</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>ciracle_cotde</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>ビタミンC 25% 美容液 30ml くすみ美容液 / 無水 / 高濃度 高濃縮 高含量 シミ ハリ対策 ブライト効果 導入美容液 先行美容液</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>シラクル</t>
+        </is>
+      </c>
+      <c r="F580" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G580" t="n">
+        <v>0</v>
+      </c>
+      <c r="H580" t="b">
+        <v>0</v>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168768265</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J578"/>
+  <autoFilter ref="A1:J580"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 41, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$580</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$581</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J580"/>
+  <dimension ref="A1:J581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24061,8 +24061,49 @@
         </is>
       </c>
     </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>1210384546</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>laferme_official</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>【NEW発売記念特価】【1+1】 肌タイプ別ボディケア 香りで選べる保湿 ラフェルム LOW pH ボディローション 480ml 弱酸性/低刺激/保湿/乾燥肌/敏感肌</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>La Ferme</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G581" t="n">
+        <v>0</v>
+      </c>
+      <c r="H581" t="b">
+        <v>0</v>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210384546</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J580"/>
+  <autoFilter ref="A1:J581"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 43, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$584</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$590</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J584"/>
+  <dimension ref="A1:J590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24225,8 +24225,254 @@
         </is>
       </c>
     </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>1210848509</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>cosmeticmall</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>メラピールクリームマスク 50ml / 塗ってはがすパック / クリームマスクパック / マスクパック / シミ / トーンアップ / 角質 / ツヤ / 美肌 / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>シャルド</t>
+        </is>
+      </c>
+      <c r="F585" t="n">
+        <v>2599</v>
+      </c>
+      <c r="G585" t="n">
+        <v>0</v>
+      </c>
+      <c r="H585" t="b">
+        <v>0</v>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210848509</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>1190323666</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>cosmeticmall</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>PDRN エッセンス100 30ml / ヴィーガンPDRN / 美容液 / ツヤ肌 / 保湿 / 弾力 / 毛穴 / シワケア / 低刺激 / 高栄養 / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F586" t="n">
+        <v>2968</v>
+      </c>
+      <c r="G586" t="n">
+        <v>0</v>
+      </c>
+      <c r="H586" t="b">
+        <v>0</v>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190323666</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>1213915729</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>cosmeticmall</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>足角質消しフットミスト 100ml / フットケア / フットピーリング / 足角質ケア / かかとスクラブ / 消しゴム / 足角質除去 / 角質ケア / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>BAREN</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>1875</v>
+      </c>
+      <c r="G587" t="n">
+        <v>0</v>
+      </c>
+      <c r="H587" t="b">
+        <v>0</v>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213915729</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>1213402507</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>cosmeticmall</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>ポアパーフェクティングコラーゲンペプチドセラム 30ml / 美容液 / 毛穴ケア / ハリケア / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F588" t="n">
+        <v>2856</v>
+      </c>
+      <c r="G588" t="n">
+        <v>0</v>
+      </c>
+      <c r="H588" t="b">
+        <v>0</v>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213402507</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>1189243900</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>yomite</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>【公式】body用(3箱セット)【自宅でハーブピーリング】美容施術 韓国化粧品研究機関共同開発</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>on:myskin</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>17940</v>
+      </c>
+      <c r="G589" t="n">
+        <v>8</v>
+      </c>
+      <c r="H589" t="b">
+        <v>0</v>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189243900</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>1189190089</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>yomite</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>【公式】デュアルクリーム毛穴 乾燥 くすみ たるみ ハリ弾力 透明感 保湿 高保湿 水光肌 ツヤ肌 バリア機能 韓国スキンケア 集中ケア エイジングケア　ピーリング　ケア　角質　もっちり</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>on:myskin</t>
+        </is>
+      </c>
+      <c r="F590" t="n">
+        <v>5980</v>
+      </c>
+      <c r="G590" t="n">
+        <v>0</v>
+      </c>
+      <c r="H590" t="b">
+        <v>0</v>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189190089</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J584"/>
+  <autoFilter ref="A1:J590"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 44, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$590</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$592</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J590"/>
+  <dimension ref="A1:J592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24471,8 +24471,90 @@
         </is>
       </c>
     </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>1189911110</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>aginloop</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>【1+1】【GIFT付き】エージー マイクロ オイル ローション 150ml×2本 保湿化粧水・鎮静・弾力・バリア強化・ハリ・敏感肌・透明感・エイジングケア</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>AG INLOOP</t>
+        </is>
+      </c>
+      <c r="F591" t="n">
+        <v>3460</v>
+      </c>
+      <c r="G591" t="n">
+        <v>3</v>
+      </c>
+      <c r="H591" t="b">
+        <v>0</v>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189911110</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>1188445312</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>aginloop</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>【オイル美容液】エージー CG ユース セラム 50ml 水溶性コラーゲン美容液・エイジングケア・シミ取り・くすみケア・透明感・弾力・高保湿</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>AG INLOOP</t>
+        </is>
+      </c>
+      <c r="F592" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G592" t="n">
+        <v>3</v>
+      </c>
+      <c r="H592" t="b">
+        <v>0</v>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188445312</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J590"/>
+  <autoFilter ref="A1:J592"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 46, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$592</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$596</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J592"/>
+  <dimension ref="A1:J596"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24553,8 +24553,172 @@
         </is>
       </c>
     </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>1181669185</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>dr19</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>【AHA+ビタミンC】ビタAHA デュアルエフェクト クレンザー 150ml 毛穴・角質ケア洗顔</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Dr.nineteen</t>
+        </is>
+      </c>
+      <c r="F593" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G593" t="n">
+        <v>3</v>
+      </c>
+      <c r="H593" t="b">
+        <v>0</v>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181669185</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>1214656269</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>heveblue</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>【公式】【miyuセレクト】 サーモンケアリング 集中ケア3種セット（トナー・アンプル・クリーム）/ PDRN配合 / 敏感肌 / 肌荒れケア</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>HEVEBLUE</t>
+        </is>
+      </c>
+      <c r="F594" t="n">
+        <v>5915</v>
+      </c>
+      <c r="G594" t="n">
+        <v>1</v>
+      </c>
+      <c r="H594" t="b">
+        <v>0</v>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214656269</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>1204352131</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>heveblue</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>【公式】ブラック ユズ ビーン ミルククレンザー 150ml / クレンジング / 低刺激 / 保湿 / 敏感肌 / 毛穴ケア / 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>HEVEBLUE</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>3790</v>
+      </c>
+      <c r="G595" t="n">
+        <v>3</v>
+      </c>
+      <c r="H595" t="b">
+        <v>0</v>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204352131</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>1199885674</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>heveblue</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>【公式】サーモンケアリングセンテラ泡洗顔料 [200ml]/ PDRN / 泡タイプ / 高保湿 / キメ・弾力ケア/ 肌再生サポート / 敏感肌</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>HEVEBLUE</t>
+        </is>
+      </c>
+      <c r="F596" t="n">
+        <v>3490</v>
+      </c>
+      <c r="G596" t="n">
+        <v>2</v>
+      </c>
+      <c r="H596" t="b">
+        <v>0</v>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199885674</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J592"/>
+  <autoFilter ref="A1:J596"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 47, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$596</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$598</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J596"/>
+  <dimension ref="A1:J598"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24717,8 +24717,90 @@
         </is>
       </c>
     </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>1206186579</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>mumuki</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>ハニーバナナBDRNクリームミスト / ミスト PDRN 保湿ミスト コラーゲン 韓国コスメ スキンケア 弾力 毛穴 ツヤ肌 ハリケア リフティング シワ対策 ペプチド</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>MUMUKI</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G597" t="n">
+        <v>4</v>
+      </c>
+      <c r="H597" t="b">
+        <v>0</v>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206186579</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>1210983541</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>mumuki</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>ハニーバナナBDRNうるツヤセット / トナー 美容液 化粧水 アンプル セラム PDRN コラーゲン 韓国コスメ スキンケア 弾力 毛穴 ツヤ肌 ハリケア リフティング シワ対策 ゆらぎ肌</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>MUMUKI</t>
+        </is>
+      </c>
+      <c r="F598" t="n">
+        <v>6932</v>
+      </c>
+      <c r="G598" t="n">
+        <v>0</v>
+      </c>
+      <c r="H598" t="b">
+        <v>0</v>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210983541</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J596"/>
+  <autoFilter ref="A1:J598"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 50, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$599</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$602</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J599"/>
+  <dimension ref="A1:J602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24840,8 +24840,131 @@
         </is>
       </c>
     </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>1107382665</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>glowm</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>ダーマ HPC 水分カーミングマスクパック　10枚</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Glow.M</t>
+        </is>
+      </c>
+      <c r="F600" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G600" t="n">
+        <v>5</v>
+      </c>
+      <c r="H600" t="b">
+        <v>0</v>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107382665</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>1204509804</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>aesthefic</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>【NEW】パンテノール5% クライオクリーム 70ml ひんやり 赤み・熱感即座鎮静 さっぱり鎮静 しっとり保湿 お家クライオ</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>AestheFic</t>
+        </is>
+      </c>
+      <c r="F601" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G601" t="n">
+        <v>0</v>
+      </c>
+      <c r="H601" t="b">
+        <v>0</v>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204509804</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>1204509914</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>aesthefic</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>【NEW】アクアセラミド100 ジェルクレンザー クレンジング 朝洗顔 泡立て不要 LHA セラミドクレンザー 敏感肌クレンザー 朝用洗顔</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>AestheFic</t>
+        </is>
+      </c>
+      <c r="F602" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G602" t="n">
+        <v>3</v>
+      </c>
+      <c r="H602" t="b">
+        <v>0</v>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204509914</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J599"/>
+  <autoFilter ref="A1:J602"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 52, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$602</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$605</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J602"/>
+  <dimension ref="A1:J605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24963,8 +24963,131 @@
         </is>
       </c>
     </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>1207926102</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>puregram</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>ヴィーガン高麗人参PDRN バリアクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>PUREGRAM</t>
+        </is>
+      </c>
+      <c r="F603" t="n">
+        <v>1299</v>
+      </c>
+      <c r="G603" t="n">
+        <v>0</v>
+      </c>
+      <c r="H603" t="b">
+        <v>0</v>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207926102</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>1195085461</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>puregram</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>ヒアルロニック ハイパーグロウ ラッピングマスク 4ml*4 みずみずしい ツヤ感 弾力ケア リフティング しっとり ツヤ肌</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>PUREGRAM</t>
+        </is>
+      </c>
+      <c r="F604" t="n">
+        <v>499</v>
+      </c>
+      <c r="G604" t="n">
+        <v>1</v>
+      </c>
+      <c r="H604" t="b">
+        <v>0</v>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195085461</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>1195084340</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>puregram</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>ハイドラ ヒアルロニッククリーム 120ml 満足度 100 点 キメの乱れを改善</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>PUREGRAM</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>1299</v>
+      </c>
+      <c r="G605" t="n">
+        <v>2</v>
+      </c>
+      <c r="H605" t="b">
+        <v>0</v>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195084340</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J602"/>
+  <autoFilter ref="A1:J605"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 53, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$605</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$613</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J605"/>
+  <dimension ref="A1:J613"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25086,8 +25086,336 @@
         </is>
       </c>
     </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>1208955036</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>KirariSoban</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>[NEW]ボディミスト 100ml（6種択1）</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>BYREDO</t>
+        </is>
+      </c>
+      <c r="F606" t="n">
+        <v>14980</v>
+      </c>
+      <c r="G606" t="n">
+        <v>0</v>
+      </c>
+      <c r="H606" t="b">
+        <v>0</v>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208955036</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>1207285957</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>KirariSoban</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>[1+1]シグネチャー フレグランスミスト 236ml / 10種択2</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>バス&amp;amp;ボディーワークス</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G607" t="n">
+        <v>0</v>
+      </c>
+      <c r="H607" t="b">
+        <v>0</v>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207285957</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>1205245488</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>KirariSoban</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>ヒアルロン アクティブB3 エイジングケアセラム 30ml（ハリ・弾力アクティブセラム）＋かっさ /イドランス ブーストセラム（保湿・くすみケアセラム）30ml×2本 / 2種択1</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>アベンヌ</t>
+        </is>
+      </c>
+      <c r="F608" t="n">
+        <v>6800</v>
+      </c>
+      <c r="G608" t="n">
+        <v>0</v>
+      </c>
+      <c r="H608" t="b">
+        <v>0</v>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205245488</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>1209777971</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>amico888</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>3点セット シャンプー＆トリートメント＆ヘアオイル 各340ml/335g/100ml モイスト ダメージケア 保湿</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F609" t="n">
+        <v>3951</v>
+      </c>
+      <c r="G609" t="n">
+        <v>0</v>
+      </c>
+      <c r="H609" t="b">
+        <v>0</v>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209777971</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>1209394853</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>amico888</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>リッチフレグランス ボディソープ 400ml サンセットフローラル 香水仕立て アゼライン酸 グリコール酸 CICA 配合 背中ニキビ 角質ケア 保湿 泡 ボディウォッシュ ボディーソープ いい匂い</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Lujoso</t>
+        </is>
+      </c>
+      <c r="F610" t="n">
+        <v>1430</v>
+      </c>
+      <c r="G610" t="n">
+        <v>0</v>
+      </c>
+      <c r="H610" t="b">
+        <v>0</v>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209394853</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>1205511306</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>amico888</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>3点セット シャンプー＆トリートメント＆ヘアオイル 各340ml/335g/100ml EXリペア ダメージケア 保湿</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F611" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G611" t="n">
+        <v>0</v>
+      </c>
+      <c r="H611" t="b">
+        <v>0</v>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205511306</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>1209777985</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>amico888</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>3点セット シャンプー＆トリートメント＆ヘアオイル 各340ml/335g/100ml EXリペア ダメージケア 保湿</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F612" t="n">
+        <v>3951</v>
+      </c>
+      <c r="G612" t="n">
+        <v>0</v>
+      </c>
+      <c r="H612" t="b">
+        <v>0</v>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209777985</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>1208852070</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>amico888</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>3点セット シャンプー＆トリートメント＆ヘアオイル 各340ml/335g/100ml コントロール ダメージケア 保湿</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G613" t="n">
+        <v>0</v>
+      </c>
+      <c r="H613" t="b">
+        <v>0</v>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208852070</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J605"/>
+  <autoFilter ref="A1:J613"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 55, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$615</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J615"/>
+  <dimension ref="A1:J616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25496,8 +25496,49 @@
         </is>
       </c>
     </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>1173532410</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>canal</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>女性用 育毛剤【医薬部外品】頭皮ケア 抜け毛 予防 薬用育毛エッセンス 120ml 産後の脱毛 日本製 女性ホルモン 薄毛 グリチルリチン酸ジカリウム パントテニルエチルエーテル センブリエキス</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>hairvity</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>2699</v>
+      </c>
+      <c r="G616" t="n">
+        <v>4</v>
+      </c>
+      <c r="H616" t="b">
+        <v>0</v>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173532410</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J615"/>
+  <autoFilter ref="A1:J616"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 58, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$619</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J616"/>
+  <dimension ref="A1:J619"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25537,8 +25537,131 @@
         </is>
       </c>
     </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>1126930806</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>donggubat_japan</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>【公式】【累積販売数28万本突破】【レモングラスの香り】フェイス＆ボディバー レモングラス / 自然由来成分・皮膚低刺激テスト済み</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Donggubat</t>
+        </is>
+      </c>
+      <c r="F617" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G617" t="n">
+        <v>9</v>
+      </c>
+      <c r="H617" t="b">
+        <v>0</v>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1126930806</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>1215123552</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>teabless_official</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>【公式】mini PICK! リリームスクホワイトティーボディローション&amp;amp;ボディソープ250g ミニボトル／ティーパフューム お茶の香り／保湿・低刺激・ポンプ式ハンドクリーム</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>TEABLESS</t>
+        </is>
+      </c>
+      <c r="F618" t="n">
+        <v>4190</v>
+      </c>
+      <c r="G618" t="n">
+        <v>0</v>
+      </c>
+      <c r="H618" t="b">
+        <v>0</v>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215123552</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>1204747567</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>teabless_official</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>【公式】リリームスクホワイトティーハンドクリーム50ml ／ティーパフューム お茶の香り／保湿・香水・ベタつかない・韓国コスメ・ギフト</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>TEABLESS</t>
+        </is>
+      </c>
+      <c r="F619" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G619" t="n">
+        <v>1</v>
+      </c>
+      <c r="H619" t="b">
+        <v>0</v>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204747567</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J616"/>
+  <autoFilter ref="A1:J619"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 61, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$622</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$627</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J622"/>
+  <dimension ref="A1:J627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25783,8 +25783,213 @@
         </is>
       </c>
     </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>1193753404</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイテ 1000 ショート ネックスティック20g+Collagen Naite Thread Neck Cream1.5ml*2ea</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>4680</v>
+      </c>
+      <c r="G623" t="n">
+        <v>1</v>
+      </c>
+      <c r="H623" t="b">
+        <v>0</v>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193753404</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>1207427325</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>リジュラン製薬会社_4倍速急速鎮静] リジュダマEXリペアリングクリーム 20g (+5g*2ea) + 滅菌綿棒(30個入り)/限定企画/施術後の専門ケアクリーム/4倍速スピード鎮静/PDRN</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>5780</v>
+      </c>
+      <c r="G624" t="n">
+        <v>0</v>
+      </c>
+      <c r="H624" t="b">
+        <v>0</v>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207427325</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>1194273240</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイター 1500ショット ネックパッチ1.0_1セット(4枚） /1か月集中管理/ 体系的管理/一日一枚の習慣で荒れていたネックラインを滑らかに~</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>4580</v>
+      </c>
+      <c r="G625" t="n">
+        <v>1</v>
+      </c>
+      <c r="H625" t="b">
+        <v>0</v>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194273240</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>1188982019</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>[限定企画]PORE+DARK SPOTブライトニング セラム 30ml+PORE+DARK SPOTブライトニング毛穴ジャブティパッド 100ml,40個+10個入/ニアシンアミド/トラネキサム酸</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>6174</v>
+      </c>
+      <c r="G626" t="n">
+        <v>1</v>
+      </c>
+      <c r="H626" t="b">
+        <v>0</v>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188982019</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>1186447113</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>[AXIS Y]グローセラム50ml+パンテノールクリーム50mlセット/ダークス ポット補正グ ローセラム/6種類の植物由来原料 611 高度なフォーミュラ/ TECA 落ち着いた保湿ケア</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>AXIS-Y</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>6480</v>
+      </c>
+      <c r="G627" t="n">
+        <v>0</v>
+      </c>
+      <c r="H627" t="b">
+        <v>0</v>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186447113</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J622"/>
+  <autoFilter ref="A1:J627"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 62, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$627</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$629</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J627"/>
+  <dimension ref="A1:J629"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25988,8 +25988,90 @@
         </is>
       </c>
     </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>1154157650</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>CamOnMall</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>レッドピール ティングル セラム 35ml／1個 / レッドピール / 角質ケア / 毛穴ケア / つるつる肌</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>2942</v>
+      </c>
+      <c r="G628" t="n">
+        <v>1</v>
+      </c>
+      <c r="H628" t="b">
+        <v>0</v>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154157650</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>1170557275</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>CamOnMall</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>ハニー＆マカダミア ヘアトリートメント 500ml 8種 / ベビーパウダー／ペア&amp;amp;フリージア／イランイラン／ホワイトムスク／アカシアモリンガ／ブラックベリーベイ／ファジーネーブル／クリーンソープ</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>1784</v>
+      </c>
+      <c r="G629" t="n">
+        <v>4</v>
+      </c>
+      <c r="H629" t="b">
+        <v>0</v>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170557275</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J627"/>
+  <autoFilter ref="A1:J629"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 65, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$633</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$638</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J633"/>
+  <dimension ref="A1:J638"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26234,8 +26234,213 @@
         </is>
       </c>
     </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>1209217973</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>dstore</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>【選べるタイプ】ヘアバーム　993 / 997　LINC ORIGINAL MAKERS　HAIR BALM　No993 No997 リンクオリジナル メーカーズ スタイリング バーム</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>LINC ORIGINAL MAKERS</t>
+        </is>
+      </c>
+      <c r="F634" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G634" t="n">
+        <v>8</v>
+      </c>
+      <c r="H634" t="b">
+        <v>0</v>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209217973</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>1213041615</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>dstore</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>【 ハード 】マークユー【 バームフォーム ハード 120g 】ヘアフォーム ヘアフォーム ツヤ バーム 高いセット力 リッジ感 1日中キープ 馴染む 泡 ヘアセット ヘアケ</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G635" t="n">
+        <v>0</v>
+      </c>
+      <c r="H635" t="b">
+        <v>0</v>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213041615</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>1209240087</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>dstore</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>【ミディアム】マークユー【 バームフォーム ミディアム 120g 】ヘアフォーム ヘアフォーム ツヤ バーム ニュアンス キープ 泡 ヘアセット ヘアケア ヘアスタイリング ツヤ メンズ</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G636" t="n">
+        <v>0</v>
+      </c>
+      <c r="H636" t="b">
+        <v>0</v>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209240087</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>1203318744</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>sinnpurete</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>【 WILDSIDE YOHJI YAMAMOTO × SINN PURETÉ 】 トゥーグッド マルチベネフィットオイル POWDER ＆ SMOKE 50ml ベスコス多数受賞 ヘアオイル</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>SINN PURETE</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G637" t="n">
+        <v>0</v>
+      </c>
+      <c r="H637" t="b">
+        <v>0</v>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203318744</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>1204583169</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>sinnpurete</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>【桜田通コラボ】 トゥーグッド マルチベネフィットオイル シルキースムースオイル 50ml ベスコス多数受賞 ヘアオイル スタイリング アウトバスオイル オーガニック 保湿 美容室 専売 サロン</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>SINN PURETE</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G638" t="n">
+        <v>9</v>
+      </c>
+      <c r="H638" t="b">
+        <v>0</v>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204583169</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J633"/>
+  <autoFilter ref="A1:J638"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 74, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$641</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$643</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J641"/>
+  <dimension ref="A1:J643"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26562,8 +26562,90 @@
         </is>
       </c>
     </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>1210458822</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>fancylifecosme</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>国内正規品 セラムヴェール ローション 180mL 化粧水 本体 グリーンフローラル しっとり 保湿 毛穴 乾燥 KOSE</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>ONE BY KOSE</t>
+        </is>
+      </c>
+      <c r="F642" t="n">
+        <v>2988</v>
+      </c>
+      <c r="G642" t="n">
+        <v>0</v>
+      </c>
+      <c r="H642" t="b">
+        <v>0</v>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210458822</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>1192672114</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>fancylifecosme</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>国内正規品 La sana 海藻 ヘア エッセンス しっとり Mサイズ 75ml 本体 しっとりタイプ 無香料</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F643" t="n">
+        <v>2518</v>
+      </c>
+      <c r="G643" t="n">
+        <v>8</v>
+      </c>
+      <c r="H643" t="b">
+        <v>0</v>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192672114</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J641"/>
+  <autoFilter ref="A1:J643"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 76, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$647</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$653</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J647"/>
+  <dimension ref="A1:J653"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26808,8 +26808,254 @@
         </is>
       </c>
     </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>1192680076</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>mmoon10</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>アルガンオイル・精製・オーガニック／50ml （クリア・有機栽培・Refined・Org anic）</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>monday moon</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G648" t="n">
+        <v>0</v>
+      </c>
+      <c r="H648" t="b">
+        <v>0</v>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192680076</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>1192681243</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>mmoon10</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>ホホバオイル・未精製・オーガニック／50ml （未精製・有機栽培・Virg in・Org anic</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>monday moon</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G649" t="n">
+        <v>2</v>
+      </c>
+      <c r="H649" t="b">
+        <v>0</v>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192681243</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>1210465765</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>FancyCosme</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>国内正規品 セラムヴェール エマルジョン 135mL 高保湿乳液 本体</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>ONE BY KOSE</t>
+        </is>
+      </c>
+      <c r="F650" t="n">
+        <v>3410</v>
+      </c>
+      <c r="G650" t="n">
+        <v>0</v>
+      </c>
+      <c r="H650" t="b">
+        <v>0</v>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210465765</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>1195846026</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>FancyCosme</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>【国内正規品 】エピステーム アイパーフェクトショットb 9g 目元用美容クリーム</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>ロート製薬</t>
+        </is>
+      </c>
+      <c r="F651" t="n">
+        <v>5777</v>
+      </c>
+      <c r="G651" t="n">
+        <v>2</v>
+      </c>
+      <c r="H651" t="b">
+        <v>0</v>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195846026</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>1191440852</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>FancyCosme</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>【国内正規品・2025年NEW】X バイタライズ リフトクリーム 50g レフィル/付け替え用 高機能クリーム 保湿 スキンケア</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>オバジ</t>
+        </is>
+      </c>
+      <c r="F652" t="n">
+        <v>10350</v>
+      </c>
+      <c r="G652" t="n">
+        <v>7</v>
+      </c>
+      <c r="H652" t="b">
+        <v>0</v>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191440852</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>1210204141</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>FancyCosme</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>26年夏数量限定・3個セット メイク キープ ミスト EX + 超COOL 80mL×3 レモンミントの香り メイクアップ 仕上げ用ローション</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Kose</t>
+        </is>
+      </c>
+      <c r="F653" t="n">
+        <v>3972</v>
+      </c>
+      <c r="G653" t="n">
+        <v>0</v>
+      </c>
+      <c r="H653" t="b">
+        <v>0</v>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210204141</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J647"/>
+  <autoFilter ref="A1:J653"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 77, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$653</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$654</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J653"/>
+  <dimension ref="A1:J654"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27054,8 +27054,49 @@
         </is>
       </c>
     </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>1172668781</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>kamicollection</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>PPT美容液スプレーN 120g 洗い流さないトリートメント</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>B/S Select</t>
+        </is>
+      </c>
+      <c r="F654" t="n">
+        <v>1870</v>
+      </c>
+      <c r="G654" t="n">
+        <v>0</v>
+      </c>
+      <c r="H654" t="b">
+        <v>0</v>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172668781</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J653"/>
+  <autoFilter ref="A1:J654"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 80, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$657</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$659</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J657"/>
+  <dimension ref="A1:J659"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27218,8 +27218,90 @@
         </is>
       </c>
     </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>1139337511</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>tamago-kichi</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>【公式】ニューモ 育毛剤 75ml 単品</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>ニューモ</t>
+        </is>
+      </c>
+      <c r="F658" t="n">
+        <v>7906</v>
+      </c>
+      <c r="G658" t="n">
+        <v>8</v>
+      </c>
+      <c r="H658" t="b">
+        <v>0</v>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139337511</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>1174798735</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>tamago-kichi</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>【公式】ヘアボーテ エクラ ボタニカルエアカラーフォームEX ライトブラウン 150g ヘアカラー 泡 白髪染め 毛染め</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>ヘアボーテエクラ</t>
+        </is>
+      </c>
+      <c r="F659" t="n">
+        <v>8120</v>
+      </c>
+      <c r="G659" t="n">
+        <v>6</v>
+      </c>
+      <c r="H659" t="b">
+        <v>0</v>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174798735</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J657"/>
+  <autoFilter ref="A1:J659"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 107, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$660</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$662</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J660"/>
+  <dimension ref="A1:J662"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27341,8 +27341,90 @@
         </is>
       </c>
     </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>1145945541</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>best-seller</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>エキスパート バリーダムローション MD 300g</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G661" t="n">
+        <v>0</v>
+      </c>
+      <c r="H661" t="b">
+        <v>0</v>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145945541</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>1145978793</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>best-seller</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>リジュビネックスクリーム10g PDRN 成分</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F662" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G662" t="n">
+        <v>3</v>
+      </c>
+      <c r="H662" t="b">
+        <v>0</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145978793</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J660"/>
+  <autoFilter ref="A1:J662"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 110, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$662</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$664</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J662"/>
+  <dimension ref="A1:J664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27423,8 +27423,90 @@
         </is>
       </c>
     </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>1194251862</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>lihaw</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>クリアピールケアマスク（7枚入り）5個セット シカパック シカマスク 日本製</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>LIHAW</t>
+        </is>
+      </c>
+      <c r="F663" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G663" t="n">
+        <v>0</v>
+      </c>
+      <c r="H663" t="b">
+        <v>0</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194251862</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>1213386491</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Liizofficial</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>リズ）イージー サン ライフ モイスチャー 365 水分密着UV（第3世代フィルター）</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>LIIZ</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>1960</v>
+      </c>
+      <c r="G664" t="n">
+        <v>7</v>
+      </c>
+      <c r="H664" t="b">
+        <v>0</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213386491</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J662"/>
+  <autoFilter ref="A1:J664"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 112, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$665</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$666</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J665"/>
+  <dimension ref="A1:J666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27546,8 +27546,49 @@
         </is>
       </c>
     </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>1196981396</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>tiam_official</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>【ビタミン爆誕セット】B3ソース＆ビタミンC24 美容液セット ナイアシンアミド・ビタミンC・美肌・透明肌・シミ・くすみ・そばかす</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>ティアム</t>
+        </is>
+      </c>
+      <c r="F666" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G666" t="n">
+        <v>1</v>
+      </c>
+      <c r="H666" t="b">
+        <v>0</v>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196981396</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J665"/>
+  <autoFilter ref="A1:J666"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 113, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$666</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$669</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J666"/>
+  <dimension ref="A1:J669"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27587,8 +27587,131 @@
         </is>
       </c>
     </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>1205740142</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>1586789523</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>フィキシングスプレー (100ml) だいようりょう 化粧崩れ防止 メイク長持ち 汗・皮脂に ナチュラル仕上げ高い保湿感</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>PRAMY</t>
+        </is>
+      </c>
+      <c r="F667" t="n">
+        <v>1789</v>
+      </c>
+      <c r="G667" t="n">
+        <v>1</v>
+      </c>
+      <c r="H667" t="b">
+        <v>0</v>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205740142</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>1205740119</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>1586789523</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>PRMAYフィキシングスプレー (100ml) だいようりょう 化粧崩れ防止 メイク長持ち 汗・皮脂に ナチュラル仕上げ高い保湿感</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>PRAMY</t>
+        </is>
+      </c>
+      <c r="F668" t="n">
+        <v>1689</v>
+      </c>
+      <c r="G668" t="n">
+        <v>1</v>
+      </c>
+      <c r="H668" t="b">
+        <v>0</v>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205740119</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>1210771351</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>beau-store</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>【使用期限：2027年3月】 ラロッシュポゼ ヒアルB5アイセラム 15ml 1本 La Roche-Posay Hyalu B5 Eye Serum 海外直送 日時指定不可 国際郵便発送</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>ラロッシュポゼ</t>
+        </is>
+      </c>
+      <c r="F669" t="n">
+        <v>7380</v>
+      </c>
+      <c r="G669" t="n">
+        <v>0</v>
+      </c>
+      <c r="H669" t="b">
+        <v>0</v>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210771351</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J666"/>
+  <autoFilter ref="A1:J669"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 115, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$673</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$674</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J673"/>
+  <dimension ref="A1:J674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27874,8 +27874,49 @@
         </is>
       </c>
     </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>1214443635</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>samuse</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>ドクターケイ (Dr.K) ABC-Gピールウォッシュ (200mL / 洗顔フォーム/泡洗顔) 角栓 角質ケア 毛穴 ピーリング 洗顔料 (レチノール/ナイアシンアミド/ビタミンC/グルタチオン</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>ドクターケイ</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>5380</v>
+      </c>
+      <c r="G674" t="n">
+        <v>0</v>
+      </c>
+      <c r="H674" t="b">
+        <v>0</v>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214443635</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J673"/>
+  <autoFilter ref="A1:J674"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 116, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$674</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$677</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J674"/>
+  <dimension ref="A1:J677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27915,8 +27915,131 @@
         </is>
       </c>
     </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>1125970375</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>better_future</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>BFマイルドミルク 150mL 乳液 敏感肌 顔用 全身用 ダチョウ抗体</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>better future</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>7920</v>
+      </c>
+      <c r="G675" t="n">
+        <v>0</v>
+      </c>
+      <c r="H675" t="b">
+        <v>0</v>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125970375</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>1125969599</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>better_future</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>BFオールインワンリッチセラム 50g 美容液 NMN配合 次世代エイジングケア 1つで7役 ダチョウ抗体</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>better future</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>5940</v>
+      </c>
+      <c r="G676" t="n">
+        <v>0</v>
+      </c>
+      <c r="H676" t="b">
+        <v>0</v>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125969599</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>1125968799</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>better_future</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>BFローション 150mL 化粧水 敏感肌 高保湿 ダチョウ抗体</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>better future</t>
+        </is>
+      </c>
+      <c r="F677" t="n">
+        <v>7920</v>
+      </c>
+      <c r="G677" t="n">
+        <v>1</v>
+      </c>
+      <c r="H677" t="b">
+        <v>0</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125968799</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J674"/>
+  <autoFilter ref="A1:J677"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 118, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$677</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$680</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J677"/>
+  <dimension ref="A1:J680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28038,8 +28038,131 @@
         </is>
       </c>
     </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>1207645599</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>whiteconc</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>【数量限定】薬用ホワイト ニングCC Cll 200ｇ シナモロール限定デザイン ／ CCクリーム 全身用 顔用 グレープフルーツの香り 保湿 トーンアップ 医薬部外品</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>ホワイトコンク</t>
+        </is>
+      </c>
+      <c r="F678" t="n">
+        <v>1210</v>
+      </c>
+      <c r="G678" t="n">
+        <v>9</v>
+      </c>
+      <c r="H678" t="b">
+        <v>0</v>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207645599</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>1102511351</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>whiteconc</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>薬用ホワイト ニングボディパックCll 70ｇ ／ インバス 全身用 グレープフルーツの香り くすみケア 保湿 医薬部外品</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>ホワイトコンク</t>
+        </is>
+      </c>
+      <c r="F679" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G679" t="n">
+        <v>3</v>
+      </c>
+      <c r="H679" t="b">
+        <v>0</v>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102511351</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>1102511107</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>whiteconc</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>薬用ホワイト ニングオイルCll 100mL ／ ボディオイル 全身用 グレープフルーツの香り 保湿 医薬部外品</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>ホワイトコンク</t>
+        </is>
+      </c>
+      <c r="F680" t="n">
+        <v>1485</v>
+      </c>
+      <c r="G680" t="n">
+        <v>6</v>
+      </c>
+      <c r="H680" t="b">
+        <v>0</v>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102511107</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J677"/>
+  <autoFilter ref="A1:J680"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 124, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$682</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$683</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J682"/>
+  <dimension ref="A1:J683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28243,8 +28243,49 @@
         </is>
       </c>
     </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>1178120837</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>forest_by_greenfinger_official</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>【１＋１】訳あり /フォレストピトン水分CICAクリーム 50ml /インナードライ/しっとり保湿</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>FoRest</t>
+        </is>
+      </c>
+      <c r="F683" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G683" t="n">
+        <v>8</v>
+      </c>
+      <c r="H683" t="b">
+        <v>0</v>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178120837</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J682"/>
+  <autoFilter ref="A1:J683"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 22, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$706</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$711</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J706"/>
+  <dimension ref="A1:J711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29227,8 +29227,213 @@
         </is>
       </c>
     </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>1143883992</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>AURORAPrincess</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>ミッドナイトファンタジーシャンプー 1L</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F707" t="n">
+        <v>1480</v>
+      </c>
+      <c r="G707" t="n">
+        <v>1</v>
+      </c>
+      <c r="H707" t="b">
+        <v>0</v>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J707" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143883992</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>1188140436</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>AURORAPrincess</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>サロン10 プロフェッショナル シカ プロテイン シャンプー 480ml</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F708" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G708" t="n">
+        <v>1</v>
+      </c>
+      <c r="H708" t="b">
+        <v>0</v>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J708" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188140436</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>1188143252</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>AURORAPrincess</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>サロン10プロフェッショナル シカ プロテイン トリートメント 215ml</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F709" t="n">
+        <v>1880</v>
+      </c>
+      <c r="G709" t="n">
+        <v>0</v>
+      </c>
+      <c r="H709" t="b">
+        <v>0</v>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J709" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188143252</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>1188136862</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>AURORAPrincess</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>サロン10プロテインノーウォッシュ アンプル トリートメント 200ml</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F710" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G710" t="n">
+        <v>0</v>
+      </c>
+      <c r="H710" t="b">
+        <v>0</v>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J710" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188136862</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>1142125065</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>AURORAPrincess</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>ラブリー アンド ロマンチック パフューム シャンプー 花の香り 980ml</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F711" t="n">
+        <v>1180</v>
+      </c>
+      <c r="G711" t="n">
+        <v>3</v>
+      </c>
+      <c r="H711" t="b">
+        <v>0</v>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J711" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142125065</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J706"/>
+  <autoFilter ref="A1:J711"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 25)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$711</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$713</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J711"/>
+  <dimension ref="A1:J713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29432,8 +29432,90 @@
         </is>
       </c>
     </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>1093944077</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>paimore</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>エコエイチビーエス　シャンプー　1700mL</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>パイモア</t>
+        </is>
+      </c>
+      <c r="F712" t="n">
+        <v>2344</v>
+      </c>
+      <c r="G712" t="n">
+        <v>1</v>
+      </c>
+      <c r="H712" t="b">
+        <v>0</v>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J712" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093944077</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>1093169243</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>paimore</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>エコエイチビーエス　シャンプー　500mL</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>パイモア</t>
+        </is>
+      </c>
+      <c r="F713" t="n">
+        <v>1528</v>
+      </c>
+      <c r="G713" t="n">
+        <v>0</v>
+      </c>
+      <c r="H713" t="b">
+        <v>0</v>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J713" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093169243</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J711"/>
+  <autoFilter ref="A1:J713"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 56, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$720</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$724</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J720"/>
+  <dimension ref="A1:J724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29801,8 +29801,172 @@
         </is>
       </c>
     </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>882304288</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>loveydovey</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>グーダル/GOODALビタcセラム/トナーパッド/アイパッチ/</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F721" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G721" t="n">
+        <v>0</v>
+      </c>
+      <c r="H721" t="b">
+        <v>0</v>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=882304288</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>1163519357</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>plats</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>【送料無料】ケラスターゼ CH マスク クロノロジスト R 75ml 6個セット　トリートメント マスク</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>ケラスターゼ</t>
+        </is>
+      </c>
+      <c r="F722" t="n">
+        <v>11500</v>
+      </c>
+      <c r="G722" t="n">
+        <v>0</v>
+      </c>
+      <c r="H722" t="b">
+        <v>0</v>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163519357</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>1161810704</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>plats</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>【送料無料】TAMBURINS タンバリンズ パフューム シェルエックス ハンドクリーム HOLY METAL ホーリーメタル 30ml 韓国コスメ ハンドケア 保湿 フレグランスハンドクリーム</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F723" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G723" t="n">
+        <v>3</v>
+      </c>
+      <c r="H723" t="b">
+        <v>0</v>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J723" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161810704</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>1163519340</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>plats</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>【送料無料】ケラスターゼ CH マスク クロノロジスト R 75ml 3個セット トリートメント マスク</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>ケラスターゼ</t>
+        </is>
+      </c>
+      <c r="F724" t="n">
+        <v>5980</v>
+      </c>
+      <c r="G724" t="n">
+        <v>2</v>
+      </c>
+      <c r="H724" t="b">
+        <v>0</v>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J724" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163519340</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J720"/>
+  <autoFilter ref="A1:J724"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 59, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$726</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$727</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J726"/>
+  <dimension ref="A1:J727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30047,8 +30047,49 @@
         </is>
       </c>
     </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>1114564602</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>areummall</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>【マスク1枚プレゼント】ピーチリップデュオデュオ 43g 　スクラブで角質除去　オリーブオイル配合で保湿バリア　しっとりなめらか　桃エキス　カモミール　シアバター　低刺激テスト　敏感肌</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>ココスター</t>
+        </is>
+      </c>
+      <c r="F727" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G727" t="n">
+        <v>0</v>
+      </c>
+      <c r="H727" t="b">
+        <v>0</v>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J727" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1114564602</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J726"/>
+  <autoFilter ref="A1:J727"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 67, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$728</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$730</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J728"/>
+  <dimension ref="A1:J730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30129,8 +30129,90 @@
         </is>
       </c>
     </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>1183278805</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>mizuhara</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>【公式店 / P10倍 / 国内発送】 「詰め替え用 450ml」 美BIO 集中補修 シルキーリペア パフューム トリートメント 450ml</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>エスプリーナ</t>
+        </is>
+      </c>
+      <c r="F729" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G729" t="n">
+        <v>1</v>
+      </c>
+      <c r="H729" t="b">
+        <v>0</v>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183278805</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>1183278433</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>mizuhara</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>【公式店 / P10倍 / 国内発送】 「詰め替え用 450ml」 美BIO 濃密炭酸 ミセラーヘッドスパ パフューム シャンプー 450ml</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>エスプリーナ</t>
+        </is>
+      </c>
+      <c r="F730" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G730" t="n">
+        <v>2</v>
+      </c>
+      <c r="H730" t="b">
+        <v>0</v>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183278433</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J728"/>
+  <autoFilter ref="A1:J730"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 68, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$730</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$731</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J730"/>
+  <dimension ref="A1:J731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30211,8 +30211,49 @@
         </is>
       </c>
     </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>1165218717</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>booh</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>ヒアルロン酸 EGF 夏 水分クリーム 100ML 2個（日光·熱気·乾燥までオールケア)</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>GONGSKIN</t>
+        </is>
+      </c>
+      <c r="F731" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G731" t="n">
+        <v>1</v>
+      </c>
+      <c r="H731" t="b">
+        <v>0</v>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165218717</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J730"/>
+  <autoFilter ref="A1:J731"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 31, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$770</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$771</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J770"/>
+  <dimension ref="A1:J771"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31851,8 +31851,49 @@
         </is>
       </c>
     </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>1177156734</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>cosmelulu</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>【正規販売店/選べる9種類】 ロアザバーム LOA バーム ブランシュ/シトラスベール/ジャスミンドレ/ラテローズ/ミスティックウッド/ネロリスモークティー 40g</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>ROAR</t>
+        </is>
+      </c>
+      <c r="F771" t="n">
+        <v>4950</v>
+      </c>
+      <c r="G771" t="n">
+        <v>8</v>
+      </c>
+      <c r="H771" t="b">
+        <v>0</v>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J771" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177156734</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J770"/>
+  <autoFilter ref="A1:J771"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 43)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$771</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$775</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J771"/>
+  <dimension ref="A1:J775"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31892,8 +31892,172 @@
         </is>
       </c>
     </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>1150194464</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>coreellejp</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>[公式] 肌のお悩みにあわせて選べる！THE POTIONS 美容液</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>ザ・ポーションズ</t>
+        </is>
+      </c>
+      <c r="F772" t="n">
+        <v>1330</v>
+      </c>
+      <c r="G772" t="n">
+        <v>1</v>
+      </c>
+      <c r="H772" t="b">
+        <v>0</v>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J772" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150194464</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>1120374130</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>coreellejp</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>[公式] ジェルクリームミキサー/10g/ミニサイズ/べたつかず軽い使い心地！さっぱり使える保湿クリームで脂性肌さんにおすすめ</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>ザ・ポーションズ</t>
+        </is>
+      </c>
+      <c r="F773" t="n">
+        <v>270</v>
+      </c>
+      <c r="G773" t="n">
+        <v>1</v>
+      </c>
+      <c r="H773" t="b">
+        <v>0</v>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J773" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120374130</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>949509489</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>coreellejp</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>[公式] ジェルクリームミキサー/50g/べたつかず軽い使い心地！さっぱり使える保湿クリームで脂性肌さんにおすすめ</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>ザ・ポーションズ</t>
+        </is>
+      </c>
+      <c r="F774" t="n">
+        <v>1680</v>
+      </c>
+      <c r="G774" t="n">
+        <v>5</v>
+      </c>
+      <c r="H774" t="b">
+        <v>0</v>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J774" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=949509489</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>702412027</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>coreellejp</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>[公式] ヒアルロン酸アンプル/20ml/水分爆発！乾燥肌にたっぷりのうるおいチャージ</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>ザ・ポーションズ</t>
+        </is>
+      </c>
+      <c r="F775" t="n">
+        <v>1330</v>
+      </c>
+      <c r="G775" t="n">
+        <v>3</v>
+      </c>
+      <c r="H775" t="b">
+        <v>0</v>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J775" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=702412027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J771"/>
+  <autoFilter ref="A1:J775"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 42)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$793</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$795</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J793"/>
+  <dimension ref="A1:J795"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32794,8 +32794,90 @@
         </is>
       </c>
     </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>1143447865</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>wone</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>薬用 汗拭き・スキンケアシート【30枚 × 4個入り】無香料 ノンアルコール やわらか あせも にきび 肌荒れ 予防 アラントイン ヒアルロン酸 乾燥肌 敏感肌 乾燥性敏感肌</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Dr.Heart</t>
+        </is>
+      </c>
+      <c r="F794" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G794" t="n">
+        <v>1</v>
+      </c>
+      <c r="H794" t="b">
+        <v>0</v>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143447865</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>1143447992</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>wone</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>薬用 汗拭き・スキンケアシート【30枚 × 10個入り】無香料 ノンアルコール やわらか あせも にきび 肌荒れ 予防 アラントイン ヒアルロン酸 乾燥肌 敏感肌 乾燥性敏感肌</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Dr.Heart</t>
+        </is>
+      </c>
+      <c r="F795" t="n">
+        <v>4600</v>
+      </c>
+      <c r="G795" t="n">
+        <v>0</v>
+      </c>
+      <c r="H795" t="b">
+        <v>0</v>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J795" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143447992</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J793"/>
+  <autoFilter ref="A1:J795"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 10)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$803</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$804</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J803"/>
+  <dimension ref="A1:J804"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33204,8 +33204,49 @@
         </is>
       </c>
     </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>1199396940</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>biooa</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>【公式】「サーモン由来高純度PDRN」T-PDRN ESSENCE TEEDLE 300 (50ml) 塗る針美容液・スピキュール・8種ヒアルロン酸・エイジングケア・韓国皮膚科監修</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>BIOOA</t>
+        </is>
+      </c>
+      <c r="F804" t="n">
+        <v>5900</v>
+      </c>
+      <c r="G804" t="n">
+        <v>0</v>
+      </c>
+      <c r="H804" t="b">
+        <v>0</v>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J804" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199396940</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J803"/>
+  <autoFilter ref="A1:J804"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 23, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$827</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$828</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J827"/>
+  <dimension ref="A1:J828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34188,8 +34188,49 @@
         </is>
       </c>
     </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>1215426365</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>noande</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>【詰め替えタイプ】デリケートゾーン ソープ VIO ニオイ 黒ずみ ムレ 保湿 フェムケア インティメイト ウォッシュ 弱酸性 135mL 日本製</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>NOANDE</t>
+        </is>
+      </c>
+      <c r="F828" t="n">
+        <v>1880</v>
+      </c>
+      <c r="G828" t="n">
+        <v>0</v>
+      </c>
+      <c r="H828" t="b">
+        <v>0</v>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J828" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215426365</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J827"/>
+  <autoFilter ref="A1:J828"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 4 own-file progress (반복 28, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_4.xlsx
+++ b/output/discovery_result_4.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$828</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$833</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J828"/>
+  <dimension ref="A1:J833"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34229,8 +34229,213 @@
         </is>
       </c>
     </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>1204359387</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>pouch24</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>POUCH 24 ハ・ジウォン スターターセット（クイーンズバーム 16g＋エッセンス 120mL）</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>POUCH24</t>
+        </is>
+      </c>
+      <c r="F829" t="n">
+        <v>10875</v>
+      </c>
+      <c r="G829" t="n">
+        <v>1</v>
+      </c>
+      <c r="H829" t="b">
+        <v>0</v>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J829" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204359387</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>1180304622</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>pouch24</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>POUCH 24 クイーンズバーム 16g</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>POUCH24</t>
+        </is>
+      </c>
+      <c r="F830" t="n">
+        <v>6560</v>
+      </c>
+      <c r="G830" t="n">
+        <v>2</v>
+      </c>
+      <c r="H830" t="b">
+        <v>0</v>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J830" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180304622</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>1208418385</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>pouch24</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>POUCH 24 CCC PINK</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>POUCH24</t>
+        </is>
+      </c>
+      <c r="F831" t="n">
+        <v>2880</v>
+      </c>
+      <c r="G831" t="n">
+        <v>0</v>
+      </c>
+      <c r="H831" t="b">
+        <v>0</v>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J831" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208418385</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>1204351865</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>pouch24</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>メルト＆シール セット</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>POUCH24</t>
+        </is>
+      </c>
+      <c r="F832" t="n">
+        <v>10125</v>
+      </c>
+      <c r="G832" t="n">
+        <v>2</v>
+      </c>
+      <c r="H832" t="b">
+        <v>0</v>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J832" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204351865</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>1204229455</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>pouch24</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>メルト＆モイスチャー セット</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>POUCH24</t>
+        </is>
+      </c>
+      <c r="F833" t="n">
+        <v>9375</v>
+      </c>
+      <c r="G833" t="n">
+        <v>0</v>
+      </c>
+      <c r="H833" t="b">
+        <v>0</v>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J833" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204229455</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J828"/>
+  <autoFilter ref="A1:J833"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>